<commit_message>
Add e prescription for doctor role
</commit_message>
<xml_diff>
--- a/CareOS-Hospital_ERP_System.xlsx
+++ b/CareOS-Hospital_ERP_System.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hetlimbani/Desktop/Self_Learning/CareOS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5186DCC-6AEB-344A-A03F-5E479526C7C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F4F4CE5-C3EF-5444-BF71-106CA3AE647A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19420" xr2:uid="{3BCF7A51-5C29-EE4C-8BC3-93CAF12DE1EA}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19420" activeTab="2" xr2:uid="{3BCF7A51-5C29-EE4C-8BC3-93CAF12DE1EA}"/>
   </bookViews>
   <sheets>
     <sheet name="ERP System" sheetId="1" r:id="rId1"/>
     <sheet name="Schema" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="Usefull" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="139">
   <si>
     <t>Total Roles</t>
   </si>
@@ -499,12 +499,24 @@
   <si>
     <t>insurance_policynumber</t>
   </si>
+  <si>
+    <t>Remaining work</t>
+  </si>
+  <si>
+    <t>FIX- OTP Bug during sent two otp at same time</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Add remember me functionality</t>
+  </si>
+  <si>
+    <t>patient cannot take twice appoinment in same time with different doctors</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -550,8 +562,29 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="9" tint="0.79998168889431442"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -570,6 +603,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -583,7 +622,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -607,9 +646,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -622,6 +658,11 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -971,36 +1012,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="B1" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="C1" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="16" t="s">
+      <c r="D1" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="16" t="s">
+      <c r="E1" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="16" t="s">
+      <c r="F1" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="16" t="s">
+      <c r="G1" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="16" t="s">
+      <c r="H1" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="16" t="s">
+      <c r="I1" s="15" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="I2" s="15"/>
+      <c r="I2" s="14"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
@@ -1032,7 +1073,7 @@
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B4" t="s">
+      <c r="B4" s="18" t="s">
         <v>9</v>
       </c>
       <c r="C4" t="s">
@@ -1061,7 +1102,7 @@
       <c r="B5" t="s">
         <v>16</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="18" t="s">
         <v>19</v>
       </c>
       <c r="D5" t="s">
@@ -1084,7 +1125,7 @@
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B6" t="s">
+      <c r="B6" s="18" t="s">
         <v>19</v>
       </c>
       <c r="C6" t="s">
@@ -1178,7 +1219,7 @@
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B11" t="s">
+      <c r="B11" s="18" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1218,6 +1259,21 @@
       <c r="D15" s="2" t="s">
         <v>33</v>
       </c>
+      <c r="E15" t="s">
+        <v>17</v>
+      </c>
+      <c r="F15" t="s">
+        <v>17</v>
+      </c>
+      <c r="G15" t="s">
+        <v>17</v>
+      </c>
+      <c r="H15" t="s">
+        <v>17</v>
+      </c>
+      <c r="I15" s="19" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B16" t="s">
@@ -1247,6 +1303,9 @@
       </c>
       <c r="C18" t="s">
         <v>25</v>
+      </c>
+      <c r="D18" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.2">
@@ -1272,12 +1331,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="13" t="s">
         <v>114</v>
       </c>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
       <c r="G1" s="10" t="s">
         <v>109</v>
       </c>
@@ -1472,12 +1531,12 @@
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B16" s="14" t="s">
+      <c r="B16" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="13"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
@@ -1701,12 +1760,12 @@
       <c r="C33" s="8"/>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B34" s="14" t="s">
+      <c r="B34" s="13" t="s">
         <v>116</v>
       </c>
-      <c r="C34" s="14"/>
-      <c r="D34" s="14"/>
-      <c r="E34" s="14"/>
+      <c r="C34" s="13"/>
+      <c r="D34" s="13"/>
+      <c r="E34" s="13"/>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
@@ -1821,12 +1880,12 @@
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B45" s="14" t="s">
+      <c r="B45" s="13" t="s">
         <v>118</v>
       </c>
-      <c r="C45" s="14"/>
-      <c r="D45" s="14"/>
-      <c r="E45" s="14"/>
+      <c r="C45" s="13"/>
+      <c r="D45" s="13"/>
+      <c r="E45" s="13"/>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46" s="4" t="s">
@@ -1914,38 +1973,38 @@
       <c r="A51">
         <v>5</v>
       </c>
-      <c r="B51" s="17" t="s">
+      <c r="B51" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="C51" s="17"/>
+      <c r="C51" s="16"/>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B52" s="17"/>
-      <c r="C52" s="17"/>
+      <c r="B52" s="16"/>
+      <c r="C52" s="16"/>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B53" s="17"/>
-      <c r="C53" s="17"/>
+      <c r="B53" s="16"/>
+      <c r="C53" s="16"/>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B54" s="17"/>
-      <c r="C54" s="17"/>
+      <c r="B54" s="16"/>
+      <c r="C54" s="16"/>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B55" s="17"/>
-      <c r="C55" s="17"/>
+      <c r="B55" s="16"/>
+      <c r="C55" s="16"/>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B56" s="17"/>
-      <c r="C56" s="17"/>
+      <c r="B56" s="16"/>
+      <c r="C56" s="16"/>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B57" s="17"/>
-      <c r="C57" s="17"/>
+      <c r="B57" s="16"/>
+      <c r="C57" s="16"/>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B58" s="17"/>
-      <c r="C58" s="17"/>
+      <c r="B58" s="16"/>
+      <c r="C58" s="16"/>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A60">
@@ -1998,12 +2057,12 @@
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B66" s="14" t="s">
+      <c r="B66" s="13" t="s">
         <v>119</v>
       </c>
-      <c r="C66" s="14"/>
-      <c r="D66" s="14"/>
-      <c r="E66" s="14"/>
+      <c r="C66" s="13"/>
+      <c r="D66" s="13"/>
+      <c r="E66" s="13"/>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A67" s="4" t="s">
@@ -2152,12 +2211,12 @@
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B79" s="14" t="s">
+      <c r="B79" s="13" t="s">
         <v>122</v>
       </c>
-      <c r="C79" s="14"/>
-      <c r="D79" s="14"/>
-      <c r="E79" s="14"/>
+      <c r="C79" s="13"/>
+      <c r="D79" s="13"/>
+      <c r="E79" s="13"/>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A80" s="4" t="s">
@@ -2231,26 +2290,26 @@
       <c r="A84">
         <v>4</v>
       </c>
-      <c r="B84" s="17" t="s">
+      <c r="B84" s="16" t="s">
         <v>105</v>
       </c>
-      <c r="C84" s="18"/>
+      <c r="C84" s="17"/>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B85" s="18"/>
-      <c r="C85" s="18"/>
+      <c r="B85" s="17"/>
+      <c r="C85" s="17"/>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B86" s="18"/>
-      <c r="C86" s="18"/>
+      <c r="B86" s="17"/>
+      <c r="C86" s="17"/>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B87" s="18"/>
-      <c r="C87" s="18"/>
+      <c r="B87" s="17"/>
+      <c r="C87" s="17"/>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B88" s="18"/>
-      <c r="C88" s="18"/>
+      <c r="B88" s="17"/>
+      <c r="C88" s="17"/>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A89">
@@ -2281,12 +2340,12 @@
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B93" s="14" t="s">
+      <c r="B93" s="13" t="s">
         <v>125</v>
       </c>
-      <c r="C93" s="14"/>
-      <c r="D93" s="14"/>
-      <c r="E93" s="14"/>
+      <c r="C93" s="13"/>
+      <c r="D93" s="13"/>
+      <c r="E93" s="13"/>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A94" s="4" t="s">
@@ -2382,26 +2441,26 @@
       <c r="A100">
         <v>6</v>
       </c>
-      <c r="B100" s="17" t="s">
+      <c r="B100" s="16" t="s">
         <v>111</v>
       </c>
-      <c r="C100" s="18"/>
+      <c r="C100" s="17"/>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B101" s="18"/>
-      <c r="C101" s="18"/>
+      <c r="B101" s="17"/>
+      <c r="C101" s="17"/>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B102" s="18"/>
-      <c r="C102" s="18"/>
+      <c r="B102" s="17"/>
+      <c r="C102" s="17"/>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B105" s="14" t="s">
+      <c r="B105" s="13" t="s">
         <v>126</v>
       </c>
-      <c r="C105" s="14"/>
-      <c r="D105" s="14"/>
-      <c r="E105" s="14"/>
+      <c r="C105" s="13"/>
+      <c r="D105" s="13"/>
+      <c r="E105" s="13"/>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A106" s="4" t="s">
@@ -2478,847 +2537,878 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD54E32F-1636-154F-88FF-57ECFAEA7F4B}">
   <dimension ref="A3:X41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="38.1640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:24" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="11" t="s">
         <v>112</v>
       </c>
-      <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12"/>
-      <c r="H3" s="12"/>
-      <c r="I3" s="12"/>
-      <c r="J3" s="12"/>
-      <c r="K3" s="12"/>
-      <c r="M3" s="13" t="s">
+      <c r="B3" s="11"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="11"/>
+      <c r="J3" s="11"/>
+      <c r="K3" s="11"/>
+      <c r="M3" s="12" t="s">
         <v>113</v>
       </c>
-      <c r="N3" s="13"/>
-      <c r="O3" s="13"/>
-      <c r="P3" s="13"/>
-      <c r="Q3" s="13"/>
-      <c r="R3" s="13"/>
-      <c r="S3" s="13"/>
-      <c r="T3" s="13"/>
-      <c r="U3" s="13"/>
-      <c r="V3" s="13"/>
-      <c r="W3" s="13"/>
-      <c r="X3" s="13"/>
+      <c r="N3" s="12"/>
+      <c r="O3" s="12"/>
+      <c r="P3" s="12"/>
+      <c r="Q3" s="12"/>
+      <c r="R3" s="12"/>
+      <c r="S3" s="12"/>
+      <c r="T3" s="12"/>
+      <c r="U3" s="12"/>
+      <c r="V3" s="12"/>
+      <c r="W3" s="12"/>
+      <c r="X3" s="12"/>
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A4" s="12"/>
-      <c r="B4" s="12"/>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="12"/>
-      <c r="G4" s="12"/>
-      <c r="H4" s="12"/>
-      <c r="I4" s="12"/>
-      <c r="J4" s="12"/>
-      <c r="K4" s="12"/>
-      <c r="M4" s="13"/>
-      <c r="N4" s="13"/>
-      <c r="O4" s="13"/>
-      <c r="P4" s="13"/>
-      <c r="Q4" s="13"/>
-      <c r="R4" s="13"/>
-      <c r="S4" s="13"/>
-      <c r="T4" s="13"/>
-      <c r="U4" s="13"/>
-      <c r="V4" s="13"/>
-      <c r="W4" s="13"/>
-      <c r="X4" s="13"/>
+      <c r="A4" s="11"/>
+      <c r="B4" s="11"/>
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="11"/>
+      <c r="F4" s="11"/>
+      <c r="G4" s="11"/>
+      <c r="H4" s="11"/>
+      <c r="I4" s="11"/>
+      <c r="J4" s="11"/>
+      <c r="K4" s="11"/>
+      <c r="M4" s="12"/>
+      <c r="N4" s="12"/>
+      <c r="O4" s="12"/>
+      <c r="P4" s="12"/>
+      <c r="Q4" s="12"/>
+      <c r="R4" s="12"/>
+      <c r="S4" s="12"/>
+      <c r="T4" s="12"/>
+      <c r="U4" s="12"/>
+      <c r="V4" s="12"/>
+      <c r="W4" s="12"/>
+      <c r="X4" s="12"/>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A5" s="12"/>
-      <c r="B5" s="12"/>
-      <c r="C5" s="12"/>
-      <c r="D5" s="12"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12"/>
-      <c r="H5" s="12"/>
-      <c r="I5" s="12"/>
-      <c r="J5" s="12"/>
-      <c r="K5" s="12"/>
-      <c r="M5" s="13"/>
-      <c r="N5" s="13"/>
-      <c r="O5" s="13"/>
-      <c r="P5" s="13"/>
-      <c r="Q5" s="13"/>
-      <c r="R5" s="13"/>
-      <c r="S5" s="13"/>
-      <c r="T5" s="13"/>
-      <c r="U5" s="13"/>
-      <c r="V5" s="13"/>
-      <c r="W5" s="13"/>
-      <c r="X5" s="13"/>
+      <c r="A5" s="11"/>
+      <c r="B5" s="11"/>
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="11"/>
+      <c r="J5" s="11"/>
+      <c r="K5" s="11"/>
+      <c r="M5" s="12"/>
+      <c r="N5" s="12"/>
+      <c r="O5" s="12"/>
+      <c r="P5" s="12"/>
+      <c r="Q5" s="12"/>
+      <c r="R5" s="12"/>
+      <c r="S5" s="12"/>
+      <c r="T5" s="12"/>
+      <c r="U5" s="12"/>
+      <c r="V5" s="12"/>
+      <c r="W5" s="12"/>
+      <c r="X5" s="12"/>
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A6" s="12"/>
-      <c r="B6" s="12"/>
-      <c r="C6" s="12"/>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="12"/>
-      <c r="G6" s="12"/>
-      <c r="H6" s="12"/>
-      <c r="I6" s="12"/>
-      <c r="J6" s="12"/>
-      <c r="K6" s="12"/>
-      <c r="M6" s="13"/>
-      <c r="N6" s="13"/>
-      <c r="O6" s="13"/>
-      <c r="P6" s="13"/>
-      <c r="Q6" s="13"/>
-      <c r="R6" s="13"/>
-      <c r="S6" s="13"/>
-      <c r="T6" s="13"/>
-      <c r="U6" s="13"/>
-      <c r="V6" s="13"/>
-      <c r="W6" s="13"/>
-      <c r="X6" s="13"/>
+      <c r="A6" s="11"/>
+      <c r="B6" s="11"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="11"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+      <c r="I6" s="11"/>
+      <c r="J6" s="11"/>
+      <c r="K6" s="11"/>
+      <c r="M6" s="12"/>
+      <c r="N6" s="12"/>
+      <c r="O6" s="12"/>
+      <c r="P6" s="12"/>
+      <c r="Q6" s="12"/>
+      <c r="R6" s="12"/>
+      <c r="S6" s="12"/>
+      <c r="T6" s="12"/>
+      <c r="U6" s="12"/>
+      <c r="V6" s="12"/>
+      <c r="W6" s="12"/>
+      <c r="X6" s="12"/>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A7" s="12"/>
-      <c r="B7" s="12"/>
-      <c r="C7" s="12"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
-      <c r="F7" s="12"/>
-      <c r="G7" s="12"/>
-      <c r="H7" s="12"/>
-      <c r="I7" s="12"/>
-      <c r="J7" s="12"/>
-      <c r="K7" s="12"/>
-      <c r="M7" s="13"/>
-      <c r="N7" s="13"/>
-      <c r="O7" s="13"/>
-      <c r="P7" s="13"/>
-      <c r="Q7" s="13"/>
-      <c r="R7" s="13"/>
-      <c r="S7" s="13"/>
-      <c r="T7" s="13"/>
-      <c r="U7" s="13"/>
-      <c r="V7" s="13"/>
-      <c r="W7" s="13"/>
-      <c r="X7" s="13"/>
+      <c r="A7" s="11"/>
+      <c r="B7" s="11"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="11"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="11"/>
+      <c r="I7" s="11"/>
+      <c r="J7" s="11"/>
+      <c r="K7" s="11"/>
+      <c r="M7" s="12"/>
+      <c r="N7" s="12"/>
+      <c r="O7" s="12"/>
+      <c r="P7" s="12"/>
+      <c r="Q7" s="12"/>
+      <c r="R7" s="12"/>
+      <c r="S7" s="12"/>
+      <c r="T7" s="12"/>
+      <c r="U7" s="12"/>
+      <c r="V7" s="12"/>
+      <c r="W7" s="12"/>
+      <c r="X7" s="12"/>
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A8" s="12"/>
-      <c r="B8" s="12"/>
-      <c r="C8" s="12"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
-      <c r="H8" s="12"/>
-      <c r="I8" s="12"/>
-      <c r="J8" s="12"/>
-      <c r="K8" s="12"/>
-      <c r="M8" s="13"/>
-      <c r="N8" s="13"/>
-      <c r="O8" s="13"/>
-      <c r="P8" s="13"/>
-      <c r="Q8" s="13"/>
-      <c r="R8" s="13"/>
-      <c r="S8" s="13"/>
-      <c r="T8" s="13"/>
-      <c r="U8" s="13"/>
-      <c r="V8" s="13"/>
-      <c r="W8" s="13"/>
-      <c r="X8" s="13"/>
+      <c r="A8" s="11"/>
+      <c r="B8" s="11"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="11"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="11"/>
+      <c r="G8" s="11"/>
+      <c r="H8" s="11"/>
+      <c r="I8" s="11"/>
+      <c r="J8" s="11"/>
+      <c r="K8" s="11"/>
+      <c r="M8" s="12"/>
+      <c r="N8" s="12"/>
+      <c r="O8" s="12"/>
+      <c r="P8" s="12"/>
+      <c r="Q8" s="12"/>
+      <c r="R8" s="12"/>
+      <c r="S8" s="12"/>
+      <c r="T8" s="12"/>
+      <c r="U8" s="12"/>
+      <c r="V8" s="12"/>
+      <c r="W8" s="12"/>
+      <c r="X8" s="12"/>
     </row>
     <row r="9" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A9" s="12"/>
-      <c r="B9" s="12"/>
-      <c r="C9" s="12"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="12"/>
-      <c r="G9" s="12"/>
-      <c r="H9" s="12"/>
-      <c r="I9" s="12"/>
-      <c r="J9" s="12"/>
-      <c r="K9" s="12"/>
-      <c r="M9" s="13"/>
-      <c r="N9" s="13"/>
-      <c r="O9" s="13"/>
-      <c r="P9" s="13"/>
-      <c r="Q9" s="13"/>
-      <c r="R9" s="13"/>
-      <c r="S9" s="13"/>
-      <c r="T9" s="13"/>
-      <c r="U9" s="13"/>
-      <c r="V9" s="13"/>
-      <c r="W9" s="13"/>
-      <c r="X9" s="13"/>
+      <c r="A9" s="11"/>
+      <c r="B9" s="11"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
+      <c r="I9" s="11"/>
+      <c r="J9" s="11"/>
+      <c r="K9" s="11"/>
+      <c r="M9" s="12"/>
+      <c r="N9" s="12"/>
+      <c r="O9" s="12"/>
+      <c r="P9" s="12"/>
+      <c r="Q9" s="12"/>
+      <c r="R9" s="12"/>
+      <c r="S9" s="12"/>
+      <c r="T9" s="12"/>
+      <c r="U9" s="12"/>
+      <c r="V9" s="12"/>
+      <c r="W9" s="12"/>
+      <c r="X9" s="12"/>
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A10" s="12"/>
-      <c r="B10" s="12"/>
-      <c r="C10" s="12"/>
-      <c r="D10" s="12"/>
-      <c r="E10" s="12"/>
-      <c r="F10" s="12"/>
-      <c r="G10" s="12"/>
-      <c r="H10" s="12"/>
-      <c r="I10" s="12"/>
-      <c r="J10" s="12"/>
-      <c r="K10" s="12"/>
-      <c r="M10" s="13"/>
-      <c r="N10" s="13"/>
-      <c r="O10" s="13"/>
-      <c r="P10" s="13"/>
-      <c r="Q10" s="13"/>
-      <c r="R10" s="13"/>
-      <c r="S10" s="13"/>
-      <c r="T10" s="13"/>
-      <c r="U10" s="13"/>
-      <c r="V10" s="13"/>
-      <c r="W10" s="13"/>
-      <c r="X10" s="13"/>
+      <c r="A10" s="11"/>
+      <c r="B10" s="11"/>
+      <c r="C10" s="11"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="11"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="11"/>
+      <c r="I10" s="11"/>
+      <c r="J10" s="11"/>
+      <c r="K10" s="11"/>
+      <c r="M10" s="12"/>
+      <c r="N10" s="12"/>
+      <c r="O10" s="12"/>
+      <c r="P10" s="12"/>
+      <c r="Q10" s="12"/>
+      <c r="R10" s="12"/>
+      <c r="S10" s="12"/>
+      <c r="T10" s="12"/>
+      <c r="U10" s="12"/>
+      <c r="V10" s="12"/>
+      <c r="W10" s="12"/>
+      <c r="X10" s="12"/>
     </row>
     <row r="11" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A11" s="12"/>
-      <c r="B11" s="12"/>
-      <c r="C11" s="12"/>
-      <c r="D11" s="12"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="12"/>
-      <c r="G11" s="12"/>
-      <c r="H11" s="12"/>
-      <c r="I11" s="12"/>
-      <c r="J11" s="12"/>
-      <c r="K11" s="12"/>
-      <c r="M11" s="13"/>
-      <c r="N11" s="13"/>
-      <c r="O11" s="13"/>
-      <c r="P11" s="13"/>
-      <c r="Q11" s="13"/>
-      <c r="R11" s="13"/>
-      <c r="S11" s="13"/>
-      <c r="T11" s="13"/>
-      <c r="U11" s="13"/>
-      <c r="V11" s="13"/>
-      <c r="W11" s="13"/>
-      <c r="X11" s="13"/>
+      <c r="A11" s="11"/>
+      <c r="B11" s="11"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="11"/>
+      <c r="H11" s="11"/>
+      <c r="I11" s="11"/>
+      <c r="J11" s="11"/>
+      <c r="K11" s="11"/>
+      <c r="M11" s="12"/>
+      <c r="N11" s="12"/>
+      <c r="O11" s="12"/>
+      <c r="P11" s="12"/>
+      <c r="Q11" s="12"/>
+      <c r="R11" s="12"/>
+      <c r="S11" s="12"/>
+      <c r="T11" s="12"/>
+      <c r="U11" s="12"/>
+      <c r="V11" s="12"/>
+      <c r="W11" s="12"/>
+      <c r="X11" s="12"/>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A12" s="12"/>
-      <c r="B12" s="12"/>
-      <c r="C12" s="12"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="12"/>
-      <c r="F12" s="12"/>
-      <c r="G12" s="12"/>
-      <c r="H12" s="12"/>
-      <c r="I12" s="12"/>
-      <c r="J12" s="12"/>
-      <c r="K12" s="12"/>
-      <c r="M12" s="13"/>
-      <c r="N12" s="13"/>
-      <c r="O12" s="13"/>
-      <c r="P12" s="13"/>
-      <c r="Q12" s="13"/>
-      <c r="R12" s="13"/>
-      <c r="S12" s="13"/>
-      <c r="T12" s="13"/>
-      <c r="U12" s="13"/>
-      <c r="V12" s="13"/>
-      <c r="W12" s="13"/>
-      <c r="X12" s="13"/>
+      <c r="A12" s="11"/>
+      <c r="B12" s="11"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="11"/>
+      <c r="I12" s="11"/>
+      <c r="J12" s="11"/>
+      <c r="K12" s="11"/>
+      <c r="M12" s="12"/>
+      <c r="N12" s="12"/>
+      <c r="O12" s="12"/>
+      <c r="P12" s="12"/>
+      <c r="Q12" s="12"/>
+      <c r="R12" s="12"/>
+      <c r="S12" s="12"/>
+      <c r="T12" s="12"/>
+      <c r="U12" s="12"/>
+      <c r="V12" s="12"/>
+      <c r="W12" s="12"/>
+      <c r="X12" s="12"/>
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A13" s="12"/>
-      <c r="B13" s="12"/>
-      <c r="C13" s="12"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="12"/>
-      <c r="H13" s="12"/>
-      <c r="I13" s="12"/>
-      <c r="J13" s="12"/>
-      <c r="K13" s="12"/>
-      <c r="M13" s="13"/>
-      <c r="N13" s="13"/>
-      <c r="O13" s="13"/>
-      <c r="P13" s="13"/>
-      <c r="Q13" s="13"/>
-      <c r="R13" s="13"/>
-      <c r="S13" s="13"/>
-      <c r="T13" s="13"/>
-      <c r="U13" s="13"/>
-      <c r="V13" s="13"/>
-      <c r="W13" s="13"/>
-      <c r="X13" s="13"/>
+      <c r="A13" s="11"/>
+      <c r="B13" s="11"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="11"/>
+      <c r="G13" s="11"/>
+      <c r="H13" s="11"/>
+      <c r="I13" s="11"/>
+      <c r="J13" s="11"/>
+      <c r="K13" s="11"/>
+      <c r="M13" s="12"/>
+      <c r="N13" s="12"/>
+      <c r="O13" s="12"/>
+      <c r="P13" s="12"/>
+      <c r="Q13" s="12"/>
+      <c r="R13" s="12"/>
+      <c r="S13" s="12"/>
+      <c r="T13" s="12"/>
+      <c r="U13" s="12"/>
+      <c r="V13" s="12"/>
+      <c r="W13" s="12"/>
+      <c r="X13" s="12"/>
     </row>
     <row r="14" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A14" s="12"/>
-      <c r="B14" s="12"/>
-      <c r="C14" s="12"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="12"/>
-      <c r="F14" s="12"/>
-      <c r="G14" s="12"/>
-      <c r="H14" s="12"/>
-      <c r="I14" s="12"/>
-      <c r="J14" s="12"/>
-      <c r="K14" s="12"/>
-      <c r="M14" s="13"/>
-      <c r="N14" s="13"/>
-      <c r="O14" s="13"/>
-      <c r="P14" s="13"/>
-      <c r="Q14" s="13"/>
-      <c r="R14" s="13"/>
-      <c r="S14" s="13"/>
-      <c r="T14" s="13"/>
-      <c r="U14" s="13"/>
-      <c r="V14" s="13"/>
-      <c r="W14" s="13"/>
-      <c r="X14" s="13"/>
+      <c r="A14" s="11"/>
+      <c r="B14" s="11"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="11"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="11"/>
+      <c r="I14" s="11"/>
+      <c r="J14" s="11"/>
+      <c r="K14" s="11"/>
+      <c r="M14" s="12"/>
+      <c r="N14" s="12"/>
+      <c r="O14" s="12"/>
+      <c r="P14" s="12"/>
+      <c r="Q14" s="12"/>
+      <c r="R14" s="12"/>
+      <c r="S14" s="12"/>
+      <c r="T14" s="12"/>
+      <c r="U14" s="12"/>
+      <c r="V14" s="12"/>
+      <c r="W14" s="12"/>
+      <c r="X14" s="12"/>
     </row>
     <row r="15" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A15" s="12"/>
-      <c r="B15" s="12"/>
-      <c r="C15" s="12"/>
-      <c r="D15" s="12"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="12"/>
-      <c r="H15" s="12"/>
-      <c r="I15" s="12"/>
-      <c r="J15" s="12"/>
-      <c r="K15" s="12"/>
-      <c r="M15" s="13"/>
-      <c r="N15" s="13"/>
-      <c r="O15" s="13"/>
-      <c r="P15" s="13"/>
-      <c r="Q15" s="13"/>
-      <c r="R15" s="13"/>
-      <c r="S15" s="13"/>
-      <c r="T15" s="13"/>
-      <c r="U15" s="13"/>
-      <c r="V15" s="13"/>
-      <c r="W15" s="13"/>
-      <c r="X15" s="13"/>
+      <c r="A15" s="11"/>
+      <c r="B15" s="11"/>
+      <c r="C15" s="11"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="11"/>
+      <c r="G15" s="11"/>
+      <c r="H15" s="11"/>
+      <c r="I15" s="11"/>
+      <c r="J15" s="11"/>
+      <c r="K15" s="11"/>
+      <c r="M15" s="12"/>
+      <c r="N15" s="12"/>
+      <c r="O15" s="12"/>
+      <c r="P15" s="12"/>
+      <c r="Q15" s="12"/>
+      <c r="R15" s="12"/>
+      <c r="S15" s="12"/>
+      <c r="T15" s="12"/>
+      <c r="U15" s="12"/>
+      <c r="V15" s="12"/>
+      <c r="W15" s="12"/>
+      <c r="X15" s="12"/>
     </row>
     <row r="16" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A16" s="12"/>
-      <c r="B16" s="12"/>
-      <c r="C16" s="12"/>
-      <c r="D16" s="12"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="12"/>
-      <c r="G16" s="12"/>
-      <c r="H16" s="12"/>
-      <c r="I16" s="12"/>
-      <c r="J16" s="12"/>
-      <c r="K16" s="12"/>
-      <c r="M16" s="13"/>
-      <c r="N16" s="13"/>
-      <c r="O16" s="13"/>
-      <c r="P16" s="13"/>
-      <c r="Q16" s="13"/>
-      <c r="R16" s="13"/>
-      <c r="S16" s="13"/>
-      <c r="T16" s="13"/>
-      <c r="U16" s="13"/>
-      <c r="V16" s="13"/>
-      <c r="W16" s="13"/>
-      <c r="X16" s="13"/>
+      <c r="A16" s="11"/>
+      <c r="B16" s="11"/>
+      <c r="C16" s="11"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="11"/>
+      <c r="G16" s="11"/>
+      <c r="H16" s="11"/>
+      <c r="I16" s="11"/>
+      <c r="J16" s="11"/>
+      <c r="K16" s="11"/>
+      <c r="M16" s="12"/>
+      <c r="N16" s="12"/>
+      <c r="O16" s="12"/>
+      <c r="P16" s="12"/>
+      <c r="Q16" s="12"/>
+      <c r="R16" s="12"/>
+      <c r="S16" s="12"/>
+      <c r="T16" s="12"/>
+      <c r="U16" s="12"/>
+      <c r="V16" s="12"/>
+      <c r="W16" s="12"/>
+      <c r="X16" s="12"/>
     </row>
     <row r="17" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A17" s="12"/>
-      <c r="B17" s="12"/>
-      <c r="C17" s="12"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="12"/>
-      <c r="F17" s="12"/>
-      <c r="G17" s="12"/>
-      <c r="H17" s="12"/>
-      <c r="I17" s="12"/>
-      <c r="J17" s="12"/>
-      <c r="K17" s="12"/>
-      <c r="M17" s="13"/>
-      <c r="N17" s="13"/>
-      <c r="O17" s="13"/>
-      <c r="P17" s="13"/>
-      <c r="Q17" s="13"/>
-      <c r="R17" s="13"/>
-      <c r="S17" s="13"/>
-      <c r="T17" s="13"/>
-      <c r="U17" s="13"/>
-      <c r="V17" s="13"/>
-      <c r="W17" s="13"/>
-      <c r="X17" s="13"/>
+      <c r="A17" s="11"/>
+      <c r="B17" s="11"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="11"/>
+      <c r="H17" s="11"/>
+      <c r="I17" s="11"/>
+      <c r="J17" s="11"/>
+      <c r="K17" s="11"/>
+      <c r="M17" s="12"/>
+      <c r="N17" s="12"/>
+      <c r="O17" s="12"/>
+      <c r="P17" s="12"/>
+      <c r="Q17" s="12"/>
+      <c r="R17" s="12"/>
+      <c r="S17" s="12"/>
+      <c r="T17" s="12"/>
+      <c r="U17" s="12"/>
+      <c r="V17" s="12"/>
+      <c r="W17" s="12"/>
+      <c r="X17" s="12"/>
     </row>
     <row r="18" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A18" s="12"/>
-      <c r="B18" s="12"/>
-      <c r="C18" s="12"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="12"/>
-      <c r="G18" s="12"/>
-      <c r="H18" s="12"/>
-      <c r="I18" s="12"/>
-      <c r="J18" s="12"/>
-      <c r="K18" s="12"/>
-      <c r="M18" s="13"/>
-      <c r="N18" s="13"/>
-      <c r="O18" s="13"/>
-      <c r="P18" s="13"/>
-      <c r="Q18" s="13"/>
-      <c r="R18" s="13"/>
-      <c r="S18" s="13"/>
-      <c r="T18" s="13"/>
-      <c r="U18" s="13"/>
-      <c r="V18" s="13"/>
-      <c r="W18" s="13"/>
-      <c r="X18" s="13"/>
+      <c r="A18" s="11"/>
+      <c r="B18" s="11"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="11"/>
+      <c r="I18" s="11"/>
+      <c r="J18" s="11"/>
+      <c r="K18" s="11"/>
+      <c r="M18" s="12"/>
+      <c r="N18" s="12"/>
+      <c r="O18" s="12"/>
+      <c r="P18" s="12"/>
+      <c r="Q18" s="12"/>
+      <c r="R18" s="12"/>
+      <c r="S18" s="12"/>
+      <c r="T18" s="12"/>
+      <c r="U18" s="12"/>
+      <c r="V18" s="12"/>
+      <c r="W18" s="12"/>
+      <c r="X18" s="12"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A19" s="12"/>
-      <c r="B19" s="12"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="12"/>
-      <c r="I19" s="12"/>
-      <c r="J19" s="12"/>
-      <c r="K19" s="12"/>
-      <c r="M19" s="13"/>
-      <c r="N19" s="13"/>
-      <c r="O19" s="13"/>
-      <c r="P19" s="13"/>
-      <c r="Q19" s="13"/>
-      <c r="R19" s="13"/>
-      <c r="S19" s="13"/>
-      <c r="T19" s="13"/>
-      <c r="U19" s="13"/>
-      <c r="V19" s="13"/>
-      <c r="W19" s="13"/>
-      <c r="X19" s="13"/>
+      <c r="A19" s="11"/>
+      <c r="B19" s="11"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="11"/>
+      <c r="H19" s="11"/>
+      <c r="I19" s="11"/>
+      <c r="J19" s="11"/>
+      <c r="K19" s="11"/>
+      <c r="M19" s="12"/>
+      <c r="N19" s="12"/>
+      <c r="O19" s="12"/>
+      <c r="P19" s="12"/>
+      <c r="Q19" s="12"/>
+      <c r="R19" s="12"/>
+      <c r="S19" s="12"/>
+      <c r="T19" s="12"/>
+      <c r="U19" s="12"/>
+      <c r="V19" s="12"/>
+      <c r="W19" s="12"/>
+      <c r="X19" s="12"/>
     </row>
     <row r="20" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A20" s="12"/>
-      <c r="B20" s="12"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="12"/>
-      <c r="E20" s="12"/>
-      <c r="F20" s="12"/>
-      <c r="G20" s="12"/>
-      <c r="H20" s="12"/>
-      <c r="I20" s="12"/>
-      <c r="J20" s="12"/>
-      <c r="K20" s="12"/>
-      <c r="M20" s="13"/>
-      <c r="N20" s="13"/>
-      <c r="O20" s="13"/>
-      <c r="P20" s="13"/>
-      <c r="Q20" s="13"/>
-      <c r="R20" s="13"/>
-      <c r="S20" s="13"/>
-      <c r="T20" s="13"/>
-      <c r="U20" s="13"/>
-      <c r="V20" s="13"/>
-      <c r="W20" s="13"/>
-      <c r="X20" s="13"/>
+      <c r="A20" s="11"/>
+      <c r="B20" s="11"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="11"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="11"/>
+      <c r="H20" s="11"/>
+      <c r="I20" s="11"/>
+      <c r="J20" s="11"/>
+      <c r="K20" s="11"/>
+      <c r="M20" s="12"/>
+      <c r="N20" s="12"/>
+      <c r="O20" s="12"/>
+      <c r="P20" s="12"/>
+      <c r="Q20" s="12"/>
+      <c r="R20" s="12"/>
+      <c r="S20" s="12"/>
+      <c r="T20" s="12"/>
+      <c r="U20" s="12"/>
+      <c r="V20" s="12"/>
+      <c r="W20" s="12"/>
+      <c r="X20" s="12"/>
     </row>
     <row r="21" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A21" s="12"/>
-      <c r="B21" s="12"/>
-      <c r="C21" s="12"/>
-      <c r="D21" s="12"/>
-      <c r="E21" s="12"/>
-      <c r="F21" s="12"/>
-      <c r="G21" s="12"/>
-      <c r="H21" s="12"/>
-      <c r="I21" s="12"/>
-      <c r="J21" s="12"/>
-      <c r="K21" s="12"/>
-      <c r="M21" s="13"/>
-      <c r="N21" s="13"/>
-      <c r="O21" s="13"/>
-      <c r="P21" s="13"/>
-      <c r="Q21" s="13"/>
-      <c r="R21" s="13"/>
-      <c r="S21" s="13"/>
-      <c r="T21" s="13"/>
-      <c r="U21" s="13"/>
-      <c r="V21" s="13"/>
-      <c r="W21" s="13"/>
-      <c r="X21" s="13"/>
+      <c r="A21" s="11"/>
+      <c r="B21" s="11"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="11"/>
+      <c r="G21" s="11"/>
+      <c r="H21" s="11"/>
+      <c r="I21" s="11"/>
+      <c r="J21" s="11"/>
+      <c r="K21" s="11"/>
+      <c r="M21" s="12"/>
+      <c r="N21" s="12"/>
+      <c r="O21" s="12"/>
+      <c r="P21" s="12"/>
+      <c r="Q21" s="12"/>
+      <c r="R21" s="12"/>
+      <c r="S21" s="12"/>
+      <c r="T21" s="12"/>
+      <c r="U21" s="12"/>
+      <c r="V21" s="12"/>
+      <c r="W21" s="12"/>
+      <c r="X21" s="12"/>
     </row>
     <row r="22" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A22" s="12"/>
-      <c r="B22" s="12"/>
-      <c r="C22" s="12"/>
-      <c r="D22" s="12"/>
-      <c r="E22" s="12"/>
-      <c r="F22" s="12"/>
-      <c r="G22" s="12"/>
-      <c r="H22" s="12"/>
-      <c r="I22" s="12"/>
-      <c r="J22" s="12"/>
-      <c r="K22" s="12"/>
-      <c r="M22" s="13"/>
-      <c r="N22" s="13"/>
-      <c r="O22" s="13"/>
-      <c r="P22" s="13"/>
-      <c r="Q22" s="13"/>
-      <c r="R22" s="13"/>
-      <c r="S22" s="13"/>
-      <c r="T22" s="13"/>
-      <c r="U22" s="13"/>
-      <c r="V22" s="13"/>
-      <c r="W22" s="13"/>
-      <c r="X22" s="13"/>
+      <c r="A22" s="11"/>
+      <c r="B22" s="11"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="11"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="11"/>
+      <c r="G22" s="11"/>
+      <c r="H22" s="11"/>
+      <c r="I22" s="11"/>
+      <c r="J22" s="11"/>
+      <c r="K22" s="11"/>
+      <c r="M22" s="12"/>
+      <c r="N22" s="12"/>
+      <c r="O22" s="12"/>
+      <c r="P22" s="12"/>
+      <c r="Q22" s="12"/>
+      <c r="R22" s="12"/>
+      <c r="S22" s="12"/>
+      <c r="T22" s="12"/>
+      <c r="U22" s="12"/>
+      <c r="V22" s="12"/>
+      <c r="W22" s="12"/>
+      <c r="X22" s="12"/>
     </row>
     <row r="23" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A23" s="12"/>
-      <c r="B23" s="12"/>
-      <c r="C23" s="12"/>
-      <c r="D23" s="12"/>
-      <c r="E23" s="12"/>
-      <c r="F23" s="12"/>
-      <c r="G23" s="12"/>
-      <c r="H23" s="12"/>
-      <c r="I23" s="12"/>
-      <c r="J23" s="12"/>
-      <c r="K23" s="12"/>
-      <c r="M23" s="13"/>
-      <c r="N23" s="13"/>
-      <c r="O23" s="13"/>
-      <c r="P23" s="13"/>
-      <c r="Q23" s="13"/>
-      <c r="R23" s="13"/>
-      <c r="S23" s="13"/>
-      <c r="T23" s="13"/>
-      <c r="U23" s="13"/>
-      <c r="V23" s="13"/>
-      <c r="W23" s="13"/>
-      <c r="X23" s="13"/>
+      <c r="A23" s="11"/>
+      <c r="B23" s="11"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="11"/>
+      <c r="F23" s="11"/>
+      <c r="G23" s="11"/>
+      <c r="H23" s="11"/>
+      <c r="I23" s="11"/>
+      <c r="J23" s="11"/>
+      <c r="K23" s="11"/>
+      <c r="M23" s="12"/>
+      <c r="N23" s="12"/>
+      <c r="O23" s="12"/>
+      <c r="P23" s="12"/>
+      <c r="Q23" s="12"/>
+      <c r="R23" s="12"/>
+      <c r="S23" s="12"/>
+      <c r="T23" s="12"/>
+      <c r="U23" s="12"/>
+      <c r="V23" s="12"/>
+      <c r="W23" s="12"/>
+      <c r="X23" s="12"/>
     </row>
     <row r="24" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A24" s="12"/>
-      <c r="B24" s="12"/>
-      <c r="C24" s="12"/>
-      <c r="D24" s="12"/>
-      <c r="E24" s="12"/>
-      <c r="F24" s="12"/>
-      <c r="G24" s="12"/>
-      <c r="H24" s="12"/>
-      <c r="I24" s="12"/>
-      <c r="J24" s="12"/>
-      <c r="K24" s="12"/>
-      <c r="M24" s="13"/>
-      <c r="N24" s="13"/>
-      <c r="O24" s="13"/>
-      <c r="P24" s="13"/>
-      <c r="Q24" s="13"/>
-      <c r="R24" s="13"/>
-      <c r="S24" s="13"/>
-      <c r="T24" s="13"/>
-      <c r="U24" s="13"/>
-      <c r="V24" s="13"/>
-      <c r="W24" s="13"/>
-      <c r="X24" s="13"/>
+      <c r="A24" s="11"/>
+      <c r="B24" s="11"/>
+      <c r="C24" s="11"/>
+      <c r="D24" s="11"/>
+      <c r="E24" s="11"/>
+      <c r="F24" s="11"/>
+      <c r="G24" s="11"/>
+      <c r="H24" s="11"/>
+      <c r="I24" s="11"/>
+      <c r="J24" s="11"/>
+      <c r="K24" s="11"/>
+      <c r="M24" s="12"/>
+      <c r="N24" s="12"/>
+      <c r="O24" s="12"/>
+      <c r="P24" s="12"/>
+      <c r="Q24" s="12"/>
+      <c r="R24" s="12"/>
+      <c r="S24" s="12"/>
+      <c r="T24" s="12"/>
+      <c r="U24" s="12"/>
+      <c r="V24" s="12"/>
+      <c r="W24" s="12"/>
+      <c r="X24" s="12"/>
     </row>
     <row r="25" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A25" s="12"/>
-      <c r="B25" s="12"/>
-      <c r="C25" s="12"/>
-      <c r="D25" s="12"/>
-      <c r="E25" s="12"/>
-      <c r="F25" s="12"/>
-      <c r="G25" s="12"/>
-      <c r="H25" s="12"/>
-      <c r="I25" s="12"/>
-      <c r="J25" s="12"/>
-      <c r="K25" s="12"/>
-      <c r="M25" s="13"/>
-      <c r="N25" s="13"/>
-      <c r="O25" s="13"/>
-      <c r="P25" s="13"/>
-      <c r="Q25" s="13"/>
-      <c r="R25" s="13"/>
-      <c r="S25" s="13"/>
-      <c r="T25" s="13"/>
-      <c r="U25" s="13"/>
-      <c r="V25" s="13"/>
-      <c r="W25" s="13"/>
-      <c r="X25" s="13"/>
+      <c r="A25" s="11"/>
+      <c r="B25" s="11"/>
+      <c r="C25" s="11"/>
+      <c r="D25" s="11"/>
+      <c r="E25" s="11"/>
+      <c r="F25" s="11"/>
+      <c r="G25" s="11"/>
+      <c r="H25" s="11"/>
+      <c r="I25" s="11"/>
+      <c r="J25" s="11"/>
+      <c r="K25" s="11"/>
+      <c r="M25" s="12"/>
+      <c r="N25" s="12"/>
+      <c r="O25" s="12"/>
+      <c r="P25" s="12"/>
+      <c r="Q25" s="12"/>
+      <c r="R25" s="12"/>
+      <c r="S25" s="12"/>
+      <c r="T25" s="12"/>
+      <c r="U25" s="12"/>
+      <c r="V25" s="12"/>
+      <c r="W25" s="12"/>
+      <c r="X25" s="12"/>
     </row>
     <row r="26" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A26" s="12"/>
-      <c r="B26" s="12"/>
-      <c r="C26" s="12"/>
-      <c r="D26" s="12"/>
-      <c r="E26" s="12"/>
-      <c r="F26" s="12"/>
-      <c r="G26" s="12"/>
-      <c r="H26" s="12"/>
-      <c r="I26" s="12"/>
-      <c r="J26" s="12"/>
-      <c r="K26" s="12"/>
-      <c r="M26" s="13"/>
-      <c r="N26" s="13"/>
-      <c r="O26" s="13"/>
-      <c r="P26" s="13"/>
-      <c r="Q26" s="13"/>
-      <c r="R26" s="13"/>
-      <c r="S26" s="13"/>
-      <c r="T26" s="13"/>
-      <c r="U26" s="13"/>
-      <c r="V26" s="13"/>
-      <c r="W26" s="13"/>
-      <c r="X26" s="13"/>
+      <c r="A26" s="11"/>
+      <c r="B26" s="11"/>
+      <c r="C26" s="11"/>
+      <c r="D26" s="11"/>
+      <c r="E26" s="11"/>
+      <c r="F26" s="11"/>
+      <c r="G26" s="11"/>
+      <c r="H26" s="11"/>
+      <c r="I26" s="11"/>
+      <c r="J26" s="11"/>
+      <c r="K26" s="11"/>
+      <c r="M26" s="12"/>
+      <c r="N26" s="12"/>
+      <c r="O26" s="12"/>
+      <c r="P26" s="12"/>
+      <c r="Q26" s="12"/>
+      <c r="R26" s="12"/>
+      <c r="S26" s="12"/>
+      <c r="T26" s="12"/>
+      <c r="U26" s="12"/>
+      <c r="V26" s="12"/>
+      <c r="W26" s="12"/>
+      <c r="X26" s="12"/>
     </row>
     <row r="27" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A27" s="12"/>
-      <c r="B27" s="12"/>
-      <c r="C27" s="12"/>
-      <c r="D27" s="12"/>
-      <c r="E27" s="12"/>
-      <c r="F27" s="12"/>
-      <c r="G27" s="12"/>
-      <c r="H27" s="12"/>
-      <c r="I27" s="12"/>
-      <c r="J27" s="12"/>
-      <c r="K27" s="12"/>
-      <c r="M27" s="13"/>
-      <c r="N27" s="13"/>
-      <c r="O27" s="13"/>
-      <c r="P27" s="13"/>
-      <c r="Q27" s="13"/>
-      <c r="R27" s="13"/>
-      <c r="S27" s="13"/>
-      <c r="T27" s="13"/>
-      <c r="U27" s="13"/>
-      <c r="V27" s="13"/>
-      <c r="W27" s="13"/>
-      <c r="X27" s="13"/>
+      <c r="A27" s="11"/>
+      <c r="B27" s="11"/>
+      <c r="C27" s="11"/>
+      <c r="D27" s="11"/>
+      <c r="E27" s="11"/>
+      <c r="F27" s="11"/>
+      <c r="G27" s="11"/>
+      <c r="H27" s="11"/>
+      <c r="I27" s="11"/>
+      <c r="J27" s="11"/>
+      <c r="K27" s="11"/>
+      <c r="M27" s="12"/>
+      <c r="N27" s="12"/>
+      <c r="O27" s="12"/>
+      <c r="P27" s="12"/>
+      <c r="Q27" s="12"/>
+      <c r="R27" s="12"/>
+      <c r="S27" s="12"/>
+      <c r="T27" s="12"/>
+      <c r="U27" s="12"/>
+      <c r="V27" s="12"/>
+      <c r="W27" s="12"/>
+      <c r="X27" s="12"/>
     </row>
     <row r="28" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A28" s="12"/>
-      <c r="B28" s="12"/>
-      <c r="C28" s="12"/>
-      <c r="D28" s="12"/>
-      <c r="E28" s="12"/>
-      <c r="F28" s="12"/>
-      <c r="G28" s="12"/>
-      <c r="H28" s="12"/>
-      <c r="I28" s="12"/>
-      <c r="J28" s="12"/>
-      <c r="K28" s="12"/>
-      <c r="M28" s="13"/>
-      <c r="N28" s="13"/>
-      <c r="O28" s="13"/>
-      <c r="P28" s="13"/>
-      <c r="Q28" s="13"/>
-      <c r="R28" s="13"/>
-      <c r="S28" s="13"/>
-      <c r="T28" s="13"/>
-      <c r="U28" s="13"/>
-      <c r="V28" s="13"/>
-      <c r="W28" s="13"/>
-      <c r="X28" s="13"/>
+      <c r="A28" s="11"/>
+      <c r="B28" s="11"/>
+      <c r="C28" s="11"/>
+      <c r="D28" s="11"/>
+      <c r="E28" s="11"/>
+      <c r="F28" s="11"/>
+      <c r="G28" s="11"/>
+      <c r="H28" s="11"/>
+      <c r="I28" s="11"/>
+      <c r="J28" s="11"/>
+      <c r="K28" s="11"/>
+      <c r="M28" s="12"/>
+      <c r="N28" s="12"/>
+      <c r="O28" s="12"/>
+      <c r="P28" s="12"/>
+      <c r="Q28" s="12"/>
+      <c r="R28" s="12"/>
+      <c r="S28" s="12"/>
+      <c r="T28" s="12"/>
+      <c r="U28" s="12"/>
+      <c r="V28" s="12"/>
+      <c r="W28" s="12"/>
+      <c r="X28" s="12"/>
     </row>
     <row r="29" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="M29" s="13"/>
-      <c r="N29" s="13"/>
-      <c r="O29" s="13"/>
-      <c r="P29" s="13"/>
-      <c r="Q29" s="13"/>
-      <c r="R29" s="13"/>
-      <c r="S29" s="13"/>
-      <c r="T29" s="13"/>
-      <c r="U29" s="13"/>
-      <c r="V29" s="13"/>
-      <c r="W29" s="13"/>
-      <c r="X29" s="13"/>
+      <c r="M29" s="12"/>
+      <c r="N29" s="12"/>
+      <c r="O29" s="12"/>
+      <c r="P29" s="12"/>
+      <c r="Q29" s="12"/>
+      <c r="R29" s="12"/>
+      <c r="S29" s="12"/>
+      <c r="T29" s="12"/>
+      <c r="U29" s="12"/>
+      <c r="V29" s="12"/>
+      <c r="W29" s="12"/>
+      <c r="X29" s="12"/>
     </row>
     <row r="30" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="M30" s="13"/>
-      <c r="N30" s="13"/>
-      <c r="O30" s="13"/>
-      <c r="P30" s="13"/>
-      <c r="Q30" s="13"/>
-      <c r="R30" s="13"/>
-      <c r="S30" s="13"/>
-      <c r="T30" s="13"/>
-      <c r="U30" s="13"/>
-      <c r="V30" s="13"/>
-      <c r="W30" s="13"/>
-      <c r="X30" s="13"/>
+      <c r="M30" s="12"/>
+      <c r="N30" s="12"/>
+      <c r="O30" s="12"/>
+      <c r="P30" s="12"/>
+      <c r="Q30" s="12"/>
+      <c r="R30" s="12"/>
+      <c r="S30" s="12"/>
+      <c r="T30" s="12"/>
+      <c r="U30" s="12"/>
+      <c r="V30" s="12"/>
+      <c r="W30" s="12"/>
+      <c r="X30" s="12"/>
     </row>
     <row r="31" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="M31" s="13"/>
-      <c r="N31" s="13"/>
-      <c r="O31" s="13"/>
-      <c r="P31" s="13"/>
-      <c r="Q31" s="13"/>
-      <c r="R31" s="13"/>
-      <c r="S31" s="13"/>
-      <c r="T31" s="13"/>
-      <c r="U31" s="13"/>
-      <c r="V31" s="13"/>
-      <c r="W31" s="13"/>
-      <c r="X31" s="13"/>
+      <c r="M31" s="12"/>
+      <c r="N31" s="12"/>
+      <c r="O31" s="12"/>
+      <c r="P31" s="12"/>
+      <c r="Q31" s="12"/>
+      <c r="R31" s="12"/>
+      <c r="S31" s="12"/>
+      <c r="T31" s="12"/>
+      <c r="U31" s="12"/>
+      <c r="V31" s="12"/>
+      <c r="W31" s="12"/>
+      <c r="X31" s="12"/>
     </row>
     <row r="32" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="M32" s="13"/>
-      <c r="N32" s="13"/>
-      <c r="O32" s="13"/>
-      <c r="P32" s="13"/>
-      <c r="Q32" s="13"/>
-      <c r="R32" s="13"/>
-      <c r="S32" s="13"/>
-      <c r="T32" s="13"/>
-      <c r="U32" s="13"/>
-      <c r="V32" s="13"/>
-      <c r="W32" s="13"/>
-      <c r="X32" s="13"/>
-    </row>
-    <row r="33" spans="13:24" x14ac:dyDescent="0.2">
-      <c r="M33" s="13"/>
-      <c r="N33" s="13"/>
-      <c r="O33" s="13"/>
-      <c r="P33" s="13"/>
-      <c r="Q33" s="13"/>
-      <c r="R33" s="13"/>
-      <c r="S33" s="13"/>
-      <c r="T33" s="13"/>
-      <c r="U33" s="13"/>
-      <c r="V33" s="13"/>
-      <c r="W33" s="13"/>
-      <c r="X33" s="13"/>
-    </row>
-    <row r="34" spans="13:24" x14ac:dyDescent="0.2">
-      <c r="M34" s="13"/>
-      <c r="N34" s="13"/>
-      <c r="O34" s="13"/>
-      <c r="P34" s="13"/>
-      <c r="Q34" s="13"/>
-      <c r="R34" s="13"/>
-      <c r="S34" s="13"/>
-      <c r="T34" s="13"/>
-      <c r="U34" s="13"/>
-      <c r="V34" s="13"/>
-      <c r="W34" s="13"/>
-      <c r="X34" s="13"/>
-    </row>
-    <row r="35" spans="13:24" x14ac:dyDescent="0.2">
-      <c r="M35" s="13"/>
-      <c r="N35" s="13"/>
-      <c r="O35" s="13"/>
-      <c r="P35" s="13"/>
-      <c r="Q35" s="13"/>
-      <c r="R35" s="13"/>
-      <c r="S35" s="13"/>
-      <c r="T35" s="13"/>
-      <c r="U35" s="13"/>
-      <c r="V35" s="13"/>
-      <c r="W35" s="13"/>
-      <c r="X35" s="13"/>
-    </row>
-    <row r="36" spans="13:24" x14ac:dyDescent="0.2">
-      <c r="M36" s="13"/>
-      <c r="N36" s="13"/>
-      <c r="O36" s="13"/>
-      <c r="P36" s="13"/>
-      <c r="Q36" s="13"/>
-      <c r="R36" s="13"/>
-      <c r="S36" s="13"/>
-      <c r="T36" s="13"/>
-      <c r="U36" s="13"/>
-      <c r="V36" s="13"/>
-      <c r="W36" s="13"/>
-      <c r="X36" s="13"/>
-    </row>
-    <row r="37" spans="13:24" x14ac:dyDescent="0.2">
-      <c r="M37" s="13"/>
-      <c r="N37" s="13"/>
-      <c r="O37" s="13"/>
-      <c r="P37" s="13"/>
-      <c r="Q37" s="13"/>
-      <c r="R37" s="13"/>
-      <c r="S37" s="13"/>
-      <c r="T37" s="13"/>
-      <c r="U37" s="13"/>
-      <c r="V37" s="13"/>
-      <c r="W37" s="13"/>
-      <c r="X37" s="13"/>
-    </row>
-    <row r="38" spans="13:24" x14ac:dyDescent="0.2">
-      <c r="M38" s="13"/>
-      <c r="N38" s="13"/>
-      <c r="O38" s="13"/>
-      <c r="P38" s="13"/>
-      <c r="Q38" s="13"/>
-      <c r="R38" s="13"/>
-      <c r="S38" s="13"/>
-      <c r="T38" s="13"/>
-      <c r="U38" s="13"/>
-      <c r="V38" s="13"/>
-      <c r="W38" s="13"/>
-      <c r="X38" s="13"/>
-    </row>
-    <row r="39" spans="13:24" x14ac:dyDescent="0.2">
-      <c r="M39" s="13"/>
-      <c r="N39" s="13"/>
-      <c r="O39" s="13"/>
-      <c r="P39" s="13"/>
-      <c r="Q39" s="13"/>
-      <c r="R39" s="13"/>
-      <c r="S39" s="13"/>
-      <c r="T39" s="13"/>
-      <c r="U39" s="13"/>
-      <c r="V39" s="13"/>
-      <c r="W39" s="13"/>
-      <c r="X39" s="13"/>
-    </row>
-    <row r="40" spans="13:24" x14ac:dyDescent="0.2">
-      <c r="M40" s="13"/>
-      <c r="N40" s="13"/>
-      <c r="O40" s="13"/>
-      <c r="P40" s="13"/>
-      <c r="Q40" s="13"/>
-      <c r="R40" s="13"/>
-      <c r="S40" s="13"/>
-      <c r="T40" s="13"/>
-      <c r="U40" s="13"/>
-      <c r="V40" s="13"/>
-      <c r="W40" s="13"/>
-      <c r="X40" s="13"/>
-    </row>
-    <row r="41" spans="13:24" x14ac:dyDescent="0.2">
-      <c r="M41" s="13"/>
-      <c r="N41" s="13"/>
-      <c r="O41" s="13"/>
-      <c r="P41" s="13"/>
-      <c r="Q41" s="13"/>
-      <c r="R41" s="13"/>
-      <c r="S41" s="13"/>
-      <c r="T41" s="13"/>
-      <c r="U41" s="13"/>
-      <c r="V41" s="13"/>
-      <c r="W41" s="13"/>
-      <c r="X41" s="13"/>
+      <c r="M32" s="12"/>
+      <c r="N32" s="12"/>
+      <c r="O32" s="12"/>
+      <c r="P32" s="12"/>
+      <c r="Q32" s="12"/>
+      <c r="R32" s="12"/>
+      <c r="S32" s="12"/>
+      <c r="T32" s="12"/>
+      <c r="U32" s="12"/>
+      <c r="V32" s="12"/>
+      <c r="W32" s="12"/>
+      <c r="X32" s="12"/>
+    </row>
+    <row r="33" spans="1:24" ht="24" x14ac:dyDescent="0.3">
+      <c r="A33" s="20" t="s">
+        <v>135</v>
+      </c>
+      <c r="B33" s="20"/>
+      <c r="C33" s="20"/>
+      <c r="D33" s="20"/>
+      <c r="E33" s="20"/>
+      <c r="F33" s="20"/>
+      <c r="G33" s="20"/>
+      <c r="M33" s="12"/>
+      <c r="N33" s="12"/>
+      <c r="O33" s="12"/>
+      <c r="P33" s="12"/>
+      <c r="Q33" s="12"/>
+      <c r="R33" s="12"/>
+      <c r="S33" s="12"/>
+      <c r="T33" s="12"/>
+      <c r="U33" s="12"/>
+      <c r="V33" s="12"/>
+      <c r="W33" s="12"/>
+      <c r="X33" s="12"/>
+    </row>
+    <row r="34" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A34">
+        <v>1</v>
+      </c>
+      <c r="B34" t="s">
+        <v>136</v>
+      </c>
+      <c r="M34" s="12"/>
+      <c r="N34" s="12"/>
+      <c r="O34" s="12"/>
+      <c r="P34" s="12"/>
+      <c r="Q34" s="12"/>
+      <c r="R34" s="12"/>
+      <c r="S34" s="12"/>
+      <c r="T34" s="12"/>
+      <c r="U34" s="12"/>
+      <c r="V34" s="12"/>
+      <c r="W34" s="12"/>
+      <c r="X34" s="12"/>
+    </row>
+    <row r="35" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A35">
+        <v>2</v>
+      </c>
+      <c r="B35" t="s">
+        <v>137</v>
+      </c>
+      <c r="M35" s="12"/>
+      <c r="N35" s="12"/>
+      <c r="O35" s="12"/>
+      <c r="P35" s="12"/>
+      <c r="Q35" s="12"/>
+      <c r="R35" s="12"/>
+      <c r="S35" s="12"/>
+      <c r="T35" s="12"/>
+      <c r="U35" s="12"/>
+      <c r="V35" s="12"/>
+      <c r="W35" s="12"/>
+      <c r="X35" s="12"/>
+    </row>
+    <row r="36" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A36">
+        <v>3</v>
+      </c>
+      <c r="B36" t="s">
+        <v>138</v>
+      </c>
+      <c r="M36" s="12"/>
+      <c r="N36" s="12"/>
+      <c r="O36" s="12"/>
+      <c r="P36" s="12"/>
+      <c r="Q36" s="12"/>
+      <c r="R36" s="12"/>
+      <c r="S36" s="12"/>
+      <c r="T36" s="12"/>
+      <c r="U36" s="12"/>
+      <c r="V36" s="12"/>
+      <c r="W36" s="12"/>
+      <c r="X36" s="12"/>
+    </row>
+    <row r="37" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="M37" s="12"/>
+      <c r="N37" s="12"/>
+      <c r="O37" s="12"/>
+      <c r="P37" s="12"/>
+      <c r="Q37" s="12"/>
+      <c r="R37" s="12"/>
+      <c r="S37" s="12"/>
+      <c r="T37" s="12"/>
+      <c r="U37" s="12"/>
+      <c r="V37" s="12"/>
+      <c r="W37" s="12"/>
+      <c r="X37" s="12"/>
+    </row>
+    <row r="38" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="M38" s="12"/>
+      <c r="N38" s="12"/>
+      <c r="O38" s="12"/>
+      <c r="P38" s="12"/>
+      <c r="Q38" s="12"/>
+      <c r="R38" s="12"/>
+      <c r="S38" s="12"/>
+      <c r="T38" s="12"/>
+      <c r="U38" s="12"/>
+      <c r="V38" s="12"/>
+      <c r="W38" s="12"/>
+      <c r="X38" s="12"/>
+    </row>
+    <row r="39" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="M39" s="12"/>
+      <c r="N39" s="12"/>
+      <c r="O39" s="12"/>
+      <c r="P39" s="12"/>
+      <c r="Q39" s="12"/>
+      <c r="R39" s="12"/>
+      <c r="S39" s="12"/>
+      <c r="T39" s="12"/>
+      <c r="U39" s="12"/>
+      <c r="V39" s="12"/>
+      <c r="W39" s="12"/>
+      <c r="X39" s="12"/>
+    </row>
+    <row r="40" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="M40" s="12"/>
+      <c r="N40" s="12"/>
+      <c r="O40" s="12"/>
+      <c r="P40" s="12"/>
+      <c r="Q40" s="12"/>
+      <c r="R40" s="12"/>
+      <c r="S40" s="12"/>
+      <c r="T40" s="12"/>
+      <c r="U40" s="12"/>
+      <c r="V40" s="12"/>
+      <c r="W40" s="12"/>
+      <c r="X40" s="12"/>
+    </row>
+    <row r="41" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="M41" s="12"/>
+      <c r="N41" s="12"/>
+      <c r="O41" s="12"/>
+      <c r="P41" s="12"/>
+      <c r="Q41" s="12"/>
+      <c r="R41" s="12"/>
+      <c r="S41" s="12"/>
+      <c r="T41" s="12"/>
+      <c r="U41" s="12"/>
+      <c r="V41" s="12"/>
+      <c r="W41" s="12"/>
+      <c r="X41" s="12"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A3:K28"/>
     <mergeCell ref="M3:X41"/>
+    <mergeCell ref="A33:G33"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add lab report in patient role
</commit_message>
<xml_diff>
--- a/CareOS-Hospital_ERP_System.xlsx
+++ b/CareOS-Hospital_ERP_System.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hetlimbani/Desktop/Self_Learning/CareOS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69EDB50F-ECE7-8A4E-B9F3-81A03757C6E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24CD4F9D-04BB-284E-A6FC-9F536F93CD86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="680" windowWidth="34200" windowHeight="19420" xr2:uid="{3BCF7A51-5C29-EE4C-8BC3-93CAF12DE1EA}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19420" xr2:uid="{3BCF7A51-5C29-EE4C-8BC3-93CAF12DE1EA}"/>
   </bookViews>
   <sheets>
     <sheet name="ERP System" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="135">
   <si>
     <t>Total Roles</t>
   </si>
@@ -136,9 +136,6 @@
     <t>Admission Processing</t>
   </si>
   <si>
-    <t xml:space="preserve"> Billing</t>
-  </si>
-  <si>
     <t>Test Requests</t>
   </si>
   <si>
@@ -152,9 +149,6 @@
   </si>
   <si>
     <t>Report Verification</t>
-  </si>
-  <si>
-    <t>Equipment Status</t>
   </si>
   <si>
     <t>Medicine Inventory</t>
@@ -617,7 +611,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -661,6 +655,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1000,13 +995,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08157DB4-050D-DB49-BEDF-9CEE3097D5D6}">
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.5" customWidth="1"/>
     <col min="2" max="3" width="22.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="32.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="27.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="18.5" customWidth="1"/>
     <col min="7" max="7" width="24" customWidth="1"/>
     <col min="8" max="8" width="22.1640625" bestFit="1" customWidth="1"/>
@@ -1018,7 +1013,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C1" s="14" t="s">
         <v>1</v>
@@ -1050,28 +1045,28 @@
         <v>8</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
@@ -1087,17 +1082,17 @@
       <c r="E4" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="F4" t="s">
-        <v>32</v>
+      <c r="F4" s="17" t="s">
+        <v>31</v>
       </c>
       <c r="G4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="H4" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="I4" s="20" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
@@ -1113,17 +1108,17 @@
       <c r="E5" t="s">
         <v>30</v>
       </c>
-      <c r="F5" t="s">
-        <v>33</v>
+      <c r="F5" s="17" t="s">
+        <v>32</v>
       </c>
       <c r="G5" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="H5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I5" s="20" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
@@ -1139,22 +1134,22 @@
       <c r="E6" t="s">
         <v>29</v>
       </c>
-      <c r="F6" t="s">
-        <v>34</v>
+      <c r="F6" s="17" t="s">
+        <v>33</v>
       </c>
       <c r="G6" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="H6" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="I6" s="20" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B7" s="17" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C7" s="17" t="s">
         <v>18</v>
@@ -1163,53 +1158,53 @@
         <v>26</v>
       </c>
       <c r="E7" t="s">
-        <v>31</v>
-      </c>
-      <c r="F7" t="s">
-        <v>35</v>
+        <v>55</v>
+      </c>
+      <c r="F7" s="17" t="s">
+        <v>34</v>
       </c>
       <c r="G7" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="H7" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="I7" s="20" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B8" t="s">
-        <v>56</v>
+      <c r="B8" s="17" t="s">
+        <v>54</v>
       </c>
       <c r="C8" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="F8" t="s">
-        <v>36</v>
+      <c r="F8" s="17" t="s">
+        <v>35</v>
       </c>
       <c r="G8" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="H8" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C9" t="s">
         <v>17</v>
       </c>
       <c r="F9" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="G9" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="H9" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
@@ -1220,85 +1215,93 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B13" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="H13" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="I13" s="3" t="s">
-        <v>55</v>
-      </c>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="C11" s="17" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="C12" s="23"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B14" t="s">
+      <c r="B14" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B15" t="s">
         <v>11</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C15" t="s">
         <v>14</v>
       </c>
-      <c r="D14" s="21" t="s">
+      <c r="D15" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E15" t="s">
         <v>14</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F15" t="s">
         <v>14</v>
       </c>
-      <c r="G14" t="s">
+      <c r="G15" t="s">
         <v>14</v>
       </c>
-      <c r="H14" t="s">
+      <c r="H15" t="s">
         <v>14</v>
       </c>
-      <c r="I14" s="18" t="s">
+      <c r="I15" s="18" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B15" s="1" t="s">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B16" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C16" t="s">
         <v>20</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D16" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B16" t="s">
+    <row r="17" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B17" t="s">
         <v>14</v>
       </c>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4" t="s">
+      <c r="C17" s="4"/>
+      <c r="D17" s="4" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="D17" t="s">
+    <row r="18" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="D18" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B18" s="1"/>
+    <row r="19" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B19" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1319,13 +1322,13 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B1" s="11" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C1" s="11"/>
       <c r="D1" s="11"/>
       <c r="E1" s="11"/>
       <c r="G1" s="8" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="H1" s="8"/>
       <c r="I1" s="8"/>
@@ -1337,23 +1340,23 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="C2" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="D2" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="E2" s="2" t="s">
         <v>68</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>70</v>
       </c>
       <c r="F2" s="5"/>
       <c r="G2" s="8" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="H2" s="8"/>
       <c r="I2" s="8"/>
@@ -1368,16 +1371,16 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D3">
         <v>20</v>
       </c>
       <c r="E3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.2">
@@ -1385,10 +1388,10 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D4">
         <v>50</v>
@@ -1399,10 +1402,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D5">
         <v>50</v>
@@ -1413,16 +1416,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C6" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D6">
         <v>100</v>
       </c>
       <c r="E6" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
@@ -1430,10 +1433,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C7" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D7">
         <v>100</v>
@@ -1444,10 +1447,10 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C8" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D8">
         <v>15</v>
@@ -1458,10 +1461,10 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C9" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D9">
         <v>15</v>
@@ -1472,10 +1475,10 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C10" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D10">
         <v>100</v>
@@ -1486,10 +1489,10 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C11" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D11">
         <v>1</v>
@@ -1500,10 +1503,10 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C12" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.2">
@@ -1511,15 +1514,15 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C13" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B16" s="11" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C16" s="11"/>
       <c r="D16" s="11"/>
@@ -1527,19 +1530,19 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="C17" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="D17" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="E17" s="2" t="s">
         <v>68</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
@@ -1547,16 +1550,16 @@
         <v>1</v>
       </c>
       <c r="B18" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C18" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D18">
         <v>20</v>
       </c>
       <c r="E18" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
@@ -1564,16 +1567,16 @@
         <v>2</v>
       </c>
       <c r="B19" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C19" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D19">
         <v>20</v>
       </c>
       <c r="E19" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
@@ -1581,10 +1584,10 @@
         <v>3</v>
       </c>
       <c r="B20" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C20" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
@@ -1592,10 +1595,10 @@
         <v>4</v>
       </c>
       <c r="B21" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C21" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D21">
         <v>10</v>
@@ -1606,10 +1609,10 @@
         <v>5</v>
       </c>
       <c r="B22" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C22" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D22">
         <v>5</v>
@@ -1620,10 +1623,10 @@
         <v>6</v>
       </c>
       <c r="B23" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C23" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D23">
         <v>200</v>
@@ -1634,10 +1637,10 @@
         <v>7</v>
       </c>
       <c r="B24" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C24" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D24">
         <v>50</v>
@@ -1648,10 +1651,10 @@
         <v>8</v>
       </c>
       <c r="B25" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C25" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D25">
         <v>15</v>
@@ -1662,10 +1665,10 @@
         <v>9</v>
       </c>
       <c r="B26" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C26" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D26">
         <v>15</v>
@@ -1676,10 +1679,10 @@
         <v>10</v>
       </c>
       <c r="B27" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C27" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D27">
         <v>50</v>
@@ -1690,10 +1693,10 @@
         <v>11</v>
       </c>
       <c r="B28" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C28" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D28">
         <v>15</v>
@@ -1704,10 +1707,10 @@
         <v>12</v>
       </c>
       <c r="B29" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C29" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D29">
         <v>15</v>
@@ -1718,10 +1721,10 @@
         <v>13</v>
       </c>
       <c r="B30" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C30" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D30">
         <v>50</v>
@@ -1732,10 +1735,10 @@
         <v>14</v>
       </c>
       <c r="B31" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C31" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D31">
         <v>20</v>
@@ -1748,7 +1751,7 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B34" s="11" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C34" s="11"/>
       <c r="D34" s="11"/>
@@ -1756,19 +1759,19 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B35" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="C35" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="B35" s="7" t="s">
+      <c r="D35" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C35" s="7" t="s">
+      <c r="E35" s="2" t="s">
         <v>68</v>
-      </c>
-      <c r="D35" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="E35" s="2" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
@@ -1776,16 +1779,16 @@
         <v>1</v>
       </c>
       <c r="B36" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C36" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D36">
         <v>20</v>
       </c>
       <c r="E36" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
@@ -1793,16 +1796,16 @@
         <v>2</v>
       </c>
       <c r="B37" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C37" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D37">
         <v>20</v>
       </c>
       <c r="E37" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
@@ -1810,10 +1813,10 @@
         <v>3</v>
       </c>
       <c r="B38" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C38" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D38">
         <v>50</v>
@@ -1824,10 +1827,10 @@
         <v>4</v>
       </c>
       <c r="B39" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C39" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D39">
         <v>50</v>
@@ -1838,10 +1841,10 @@
         <v>5</v>
       </c>
       <c r="B40" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C40" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
@@ -1849,10 +1852,10 @@
         <v>6</v>
       </c>
       <c r="B41" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C41" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D41">
         <v>15</v>
@@ -1863,12 +1866,12 @@
         <v>7</v>
       </c>
       <c r="B42" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B45" s="11" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C45" s="11"/>
       <c r="D45" s="11"/>
@@ -1876,19 +1879,19 @@
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B46" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="C46" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="B46" s="7" t="s">
+      <c r="D46" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C46" s="7" t="s">
+      <c r="E46" s="2" t="s">
         <v>68</v>
-      </c>
-      <c r="D46" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="E46" s="2" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.2">
@@ -1896,16 +1899,16 @@
         <v>1</v>
       </c>
       <c r="B47" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C47" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D47">
         <v>20</v>
       </c>
       <c r="E47" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.2">
@@ -1913,16 +1916,16 @@
         <v>2</v>
       </c>
       <c r="B48" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C48" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D48">
         <v>20</v>
       </c>
       <c r="E48" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.2">
@@ -1930,16 +1933,16 @@
         <v>3</v>
       </c>
       <c r="B49" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C49" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D49">
         <v>20</v>
       </c>
       <c r="E49" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.2">
@@ -1947,10 +1950,10 @@
         <v>4</v>
       </c>
       <c r="B50" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C50" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D50">
         <v>15</v>
@@ -1961,7 +1964,7 @@
         <v>5</v>
       </c>
       <c r="B51" s="15" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C51" s="15"/>
     </row>
@@ -1998,10 +2001,10 @@
         <v>6</v>
       </c>
       <c r="B60" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C60" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D60">
         <v>200</v>
@@ -2012,10 +2015,10 @@
         <v>7</v>
       </c>
       <c r="B61" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C61" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D61">
         <v>1000</v>
@@ -2026,10 +2029,10 @@
         <v>8</v>
       </c>
       <c r="B62" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C62" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.2">
@@ -2037,15 +2040,15 @@
         <v>9</v>
       </c>
       <c r="B63" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C63" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B66" s="11" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C66" s="11"/>
       <c r="D66" s="11"/>
@@ -2053,19 +2056,19 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A67" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B67" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="C67" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="B67" s="7" t="s">
+      <c r="D67" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C67" s="7" t="s">
+      <c r="E67" s="2" t="s">
         <v>68</v>
-      </c>
-      <c r="D67" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="E67" s="2" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.2">
@@ -2073,16 +2076,16 @@
         <v>1</v>
       </c>
       <c r="B68" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C68" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D68">
         <v>20</v>
       </c>
       <c r="E68" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.2">
@@ -2090,16 +2093,16 @@
         <v>2</v>
       </c>
       <c r="B69" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C69" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D69">
         <v>20</v>
       </c>
       <c r="E69" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.2">
@@ -2107,16 +2110,16 @@
         <v>3</v>
       </c>
       <c r="B70" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C70" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D70">
         <v>20</v>
       </c>
       <c r="E70" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.2">
@@ -2124,10 +2127,10 @@
         <v>4</v>
       </c>
       <c r="B71" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C71" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D71">
         <v>100</v>
@@ -2138,10 +2141,10 @@
         <v>5</v>
       </c>
       <c r="B72" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C72" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D72">
         <v>500</v>
@@ -2152,10 +2155,10 @@
         <v>6</v>
       </c>
       <c r="B73" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C73" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D73">
         <v>1000</v>
@@ -2166,10 +2169,10 @@
         <v>7</v>
       </c>
       <c r="B74" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C74" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D74">
         <v>1000</v>
@@ -2180,10 +2183,10 @@
         <v>8</v>
       </c>
       <c r="B75" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C75" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.2">
@@ -2191,15 +2194,15 @@
         <v>9</v>
       </c>
       <c r="B76" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C76" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B79" s="11" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C79" s="11"/>
       <c r="D79" s="11"/>
@@ -2207,19 +2210,19 @@
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A80" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B80" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="C80" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="B80" s="7" t="s">
+      <c r="D80" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C80" s="7" t="s">
+      <c r="E80" s="2" t="s">
         <v>68</v>
-      </c>
-      <c r="D80" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="E80" s="2" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.2">
@@ -2227,16 +2230,16 @@
         <v>1</v>
       </c>
       <c r="B81" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C81" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D81">
         <v>20</v>
       </c>
       <c r="E81" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.2">
@@ -2244,16 +2247,16 @@
         <v>2</v>
       </c>
       <c r="B82" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C82" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D82">
         <v>20</v>
       </c>
       <c r="E82" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.2">
@@ -2261,16 +2264,16 @@
         <v>3</v>
       </c>
       <c r="B83" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C83" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D83">
         <v>20</v>
       </c>
       <c r="E83" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.2">
@@ -2278,7 +2281,7 @@
         <v>4</v>
       </c>
       <c r="B84" s="15" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C84" s="16"/>
     </row>
@@ -2303,10 +2306,10 @@
         <v>5</v>
       </c>
       <c r="B89" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C89" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D89">
         <v>500</v>
@@ -2317,10 +2320,10 @@
         <v>6</v>
       </c>
       <c r="B90" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C90" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D90">
         <v>1000</v>
@@ -2328,7 +2331,7 @@
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B93" s="11" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C93" s="11"/>
       <c r="D93" s="11"/>
@@ -2336,19 +2339,19 @@
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A94" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B94" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="C94" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="B94" s="7" t="s">
+      <c r="D94" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C94" s="7" t="s">
+      <c r="E94" s="2" t="s">
         <v>68</v>
-      </c>
-      <c r="D94" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="E94" s="2" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.2">
@@ -2356,16 +2359,16 @@
         <v>1</v>
       </c>
       <c r="B95" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C95" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D95">
         <v>20</v>
       </c>
       <c r="E95" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.2">
@@ -2373,16 +2376,16 @@
         <v>2</v>
       </c>
       <c r="B96" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C96" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D96">
         <v>20</v>
       </c>
       <c r="E96" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.2">
@@ -2390,10 +2393,10 @@
         <v>3</v>
       </c>
       <c r="B97" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C97" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D97">
         <v>50</v>
@@ -2404,10 +2407,10 @@
         <v>4</v>
       </c>
       <c r="B98" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C98" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D98">
         <v>3</v>
@@ -2418,10 +2421,10 @@
         <v>5</v>
       </c>
       <c r="B99" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C99" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.2">
@@ -2429,7 +2432,7 @@
         <v>6</v>
       </c>
       <c r="B100" s="15" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C100" s="16"/>
     </row>
@@ -2443,7 +2446,7 @@
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B105" s="11" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C105" s="11"/>
       <c r="D105" s="11"/>
@@ -2451,19 +2454,19 @@
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A106" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B106" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="C106" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="B106" s="7" t="s">
+      <c r="D106" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C106" s="7" t="s">
+      <c r="E106" s="2" t="s">
         <v>68</v>
-      </c>
-      <c r="D106" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="E106" s="2" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.2">
@@ -2471,16 +2474,16 @@
         <v>1</v>
       </c>
       <c r="B107" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C107" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D107">
         <v>20</v>
       </c>
       <c r="E107" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.2">
@@ -2488,16 +2491,16 @@
         <v>2</v>
       </c>
       <c r="B108" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C108" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D108">
         <v>20</v>
       </c>
       <c r="E108" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>
@@ -2530,7 +2533,7 @@
   <sheetData>
     <row r="3" spans="1:24" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="9" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B3" s="9"/>
       <c r="C3" s="9"/>
@@ -2543,7 +2546,7 @@
       <c r="J3" s="9"/>
       <c r="K3" s="9"/>
       <c r="M3" s="10" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="N3" s="10"/>
       <c r="O3" s="10"/>
@@ -3240,7 +3243,7 @@
     </row>
     <row r="33" spans="1:24" ht="24" x14ac:dyDescent="0.3">
       <c r="A33" s="19" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B33" s="19"/>
       <c r="C33" s="19"/>
@@ -3266,7 +3269,7 @@
         <v>1</v>
       </c>
       <c r="B34" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="M34" s="10"/>
       <c r="N34" s="10"/>
@@ -3286,7 +3289,7 @@
         <v>2</v>
       </c>
       <c r="B35" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="M35" s="10"/>
       <c r="N35" s="10"/>
@@ -3306,7 +3309,7 @@
         <v>3</v>
       </c>
       <c r="B36" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="M36" s="10"/>
       <c r="N36" s="10"/>
@@ -3326,7 +3329,7 @@
         <v>4</v>
       </c>
       <c r="B37" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="M37" s="10"/>
       <c r="N37" s="10"/>
@@ -3346,7 +3349,7 @@
         <v>5</v>
       </c>
       <c r="B38" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="M38" s="10"/>
       <c r="N38" s="10"/>

</xml_diff>

<commit_message>
Add prescription processing and billing funcionality in pharmacist role
</commit_message>
<xml_diff>
--- a/CareOS-Hospital_ERP_System.xlsx
+++ b/CareOS-Hospital_ERP_System.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hetlimbani/Desktop/Self_Learning/CareOS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C820117-36D2-DF41-B918-616F31779918}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB9A2D45-5403-0740-93A9-62BA2816802E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19420" xr2:uid="{3BCF7A51-5C29-EE4C-8BC3-93CAF12DE1EA}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="134">
   <si>
     <t>Total Roles</t>
   </si>
@@ -160,13 +160,7 @@
     <t>Billing</t>
   </si>
   <si>
-    <t>Stock Alerts</t>
-  </si>
-  <si>
     <t>Supplier Management</t>
-  </si>
-  <si>
-    <t>Medicine Expiry Tracking</t>
   </si>
   <si>
     <t>Staff Management</t>
@@ -498,6 +492,9 @@
   </si>
   <si>
     <t>receptionist add patient then patient signup so that's time resolve otp issue</t>
+  </si>
+  <si>
+    <t>In E-prescription add not required field in medicine and lab report at doctor role</t>
   </si>
 </sst>
 </file>
@@ -611,7 +608,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -647,6 +644,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1012,7 +1010,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C1" s="13" t="s">
         <v>1</v>
@@ -1044,28 +1042,28 @@
         <v>8</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
@@ -1078,7 +1076,7 @@
       <c r="D4" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="21" t="s">
+      <c r="E4" s="22" t="s">
         <v>15</v>
       </c>
       <c r="F4" s="16" t="s">
@@ -1088,10 +1086,10 @@
         <v>36</v>
       </c>
       <c r="H4" t="s">
-        <v>42</v>
-      </c>
-      <c r="I4" s="19" t="s">
-        <v>48</v>
+        <v>40</v>
+      </c>
+      <c r="I4" s="20" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
@@ -1110,14 +1108,14 @@
       <c r="F5" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" s="16" t="s">
         <v>37</v>
       </c>
       <c r="H5" t="s">
-        <v>43</v>
-      </c>
-      <c r="I5" s="19" t="s">
-        <v>49</v>
+        <v>41</v>
+      </c>
+      <c r="I5" s="20" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
@@ -1136,19 +1134,19 @@
       <c r="F6" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" s="16" t="s">
         <v>38</v>
       </c>
       <c r="H6" t="s">
-        <v>44</v>
-      </c>
-      <c r="I6" s="19" t="s">
-        <v>50</v>
+        <v>42</v>
+      </c>
+      <c r="I6" s="20" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B7" s="16" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C7" s="16" t="s">
         <v>18</v>
@@ -1157,24 +1155,21 @@
         <v>26</v>
       </c>
       <c r="E7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F7" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="G7" t="s">
-        <v>39</v>
-      </c>
       <c r="H7" t="s">
-        <v>45</v>
-      </c>
-      <c r="I7" s="19" t="s">
-        <v>51</v>
+        <v>43</v>
+      </c>
+      <c r="I7" s="20" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B8" s="16" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C8" s="16" t="s">
         <v>19</v>
@@ -1183,27 +1178,24 @@
         <v>35</v>
       </c>
       <c r="G8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H8" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C9" t="s">
         <v>17</v>
       </c>
       <c r="F9" t="s">
-        <v>55</v>
-      </c>
-      <c r="G9" t="s">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="H9" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
@@ -1220,32 +1212,32 @@
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C12" s="22"/>
+      <c r="C12" s="23"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B14" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
@@ -1255,7 +1247,7 @@
       <c r="C15" t="s">
         <v>14</v>
       </c>
-      <c r="D15" s="20" t="s">
+      <c r="D15" s="21" t="s">
         <v>28</v>
       </c>
       <c r="E15" t="s">
@@ -1270,7 +1262,7 @@
       <c r="H15" t="s">
         <v>14</v>
       </c>
-      <c r="I15" s="17" t="s">
+      <c r="I15" s="18" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1321,13 +1313,13 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B1" s="11" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C1" s="11"/>
       <c r="D1" s="11"/>
       <c r="E1" s="11"/>
       <c r="G1" s="8" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="H1" s="8"/>
       <c r="I1" s="8"/>
@@ -1339,23 +1331,23 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="C2" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="D2" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="E2" s="2" t="s">
         <v>66</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>68</v>
       </c>
       <c r="F2" s="5"/>
       <c r="G2" s="8" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="H2" s="8"/>
       <c r="I2" s="8"/>
@@ -1370,16 +1362,16 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D3">
         <v>20</v>
       </c>
       <c r="E3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.2">
@@ -1387,10 +1379,10 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D4">
         <v>50</v>
@@ -1401,10 +1393,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D5">
         <v>50</v>
@@ -1415,16 +1407,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C6" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D6">
         <v>100</v>
       </c>
       <c r="E6" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
@@ -1432,10 +1424,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C7" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D7">
         <v>100</v>
@@ -1446,10 +1438,10 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C8" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D8">
         <v>15</v>
@@ -1460,10 +1452,10 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C9" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D9">
         <v>15</v>
@@ -1474,10 +1466,10 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C10" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D10">
         <v>100</v>
@@ -1488,10 +1480,10 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C11" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D11">
         <v>1</v>
@@ -1502,10 +1494,10 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C12" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.2">
@@ -1513,15 +1505,15 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C13" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B16" s="11" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C16" s="11"/>
       <c r="D16" s="11"/>
@@ -1529,19 +1521,19 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="C17" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="D17" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="E17" s="2" t="s">
         <v>66</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
@@ -1549,16 +1541,16 @@
         <v>1</v>
       </c>
       <c r="B18" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C18" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D18">
         <v>20</v>
       </c>
       <c r="E18" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
@@ -1566,16 +1558,16 @@
         <v>2</v>
       </c>
       <c r="B19" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C19" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D19">
         <v>20</v>
       </c>
       <c r="E19" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
@@ -1583,10 +1575,10 @@
         <v>3</v>
       </c>
       <c r="B20" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C20" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
@@ -1594,10 +1586,10 @@
         <v>4</v>
       </c>
       <c r="B21" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C21" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D21">
         <v>10</v>
@@ -1608,10 +1600,10 @@
         <v>5</v>
       </c>
       <c r="B22" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C22" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D22">
         <v>5</v>
@@ -1622,10 +1614,10 @@
         <v>6</v>
       </c>
       <c r="B23" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C23" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D23">
         <v>200</v>
@@ -1636,10 +1628,10 @@
         <v>7</v>
       </c>
       <c r="B24" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C24" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D24">
         <v>50</v>
@@ -1650,10 +1642,10 @@
         <v>8</v>
       </c>
       <c r="B25" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C25" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D25">
         <v>15</v>
@@ -1664,10 +1656,10 @@
         <v>9</v>
       </c>
       <c r="B26" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C26" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D26">
         <v>15</v>
@@ -1678,10 +1670,10 @@
         <v>10</v>
       </c>
       <c r="B27" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C27" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D27">
         <v>50</v>
@@ -1692,10 +1684,10 @@
         <v>11</v>
       </c>
       <c r="B28" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C28" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D28">
         <v>15</v>
@@ -1706,10 +1698,10 @@
         <v>12</v>
       </c>
       <c r="B29" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C29" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D29">
         <v>15</v>
@@ -1720,10 +1712,10 @@
         <v>13</v>
       </c>
       <c r="B30" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C30" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D30">
         <v>50</v>
@@ -1734,10 +1726,10 @@
         <v>14</v>
       </c>
       <c r="B31" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C31" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D31">
         <v>20</v>
@@ -1750,7 +1742,7 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B34" s="11" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C34" s="11"/>
       <c r="D34" s="11"/>
@@ -1758,19 +1750,19 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B35" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="C35" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="B35" s="7" t="s">
+      <c r="D35" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C35" s="7" t="s">
+      <c r="E35" s="2" t="s">
         <v>66</v>
-      </c>
-      <c r="D35" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="E35" s="2" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
@@ -1778,16 +1770,16 @@
         <v>1</v>
       </c>
       <c r="B36" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C36" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D36">
         <v>20</v>
       </c>
       <c r="E36" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
@@ -1795,16 +1787,16 @@
         <v>2</v>
       </c>
       <c r="B37" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C37" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D37">
         <v>20</v>
       </c>
       <c r="E37" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
@@ -1812,10 +1804,10 @@
         <v>3</v>
       </c>
       <c r="B38" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C38" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D38">
         <v>50</v>
@@ -1826,10 +1818,10 @@
         <v>4</v>
       </c>
       <c r="B39" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C39" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D39">
         <v>50</v>
@@ -1840,10 +1832,10 @@
         <v>5</v>
       </c>
       <c r="B40" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C40" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
@@ -1851,10 +1843,10 @@
         <v>6</v>
       </c>
       <c r="B41" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C41" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D41">
         <v>15</v>
@@ -1865,12 +1857,12 @@
         <v>7</v>
       </c>
       <c r="B42" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B45" s="11" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C45" s="11"/>
       <c r="D45" s="11"/>
@@ -1878,19 +1870,19 @@
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B46" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="C46" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="B46" s="7" t="s">
+      <c r="D46" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C46" s="7" t="s">
+      <c r="E46" s="2" t="s">
         <v>66</v>
-      </c>
-      <c r="D46" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="E46" s="2" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.2">
@@ -1898,16 +1890,16 @@
         <v>1</v>
       </c>
       <c r="B47" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C47" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D47">
         <v>20</v>
       </c>
       <c r="E47" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.2">
@@ -1915,16 +1907,16 @@
         <v>2</v>
       </c>
       <c r="B48" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C48" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D48">
         <v>20</v>
       </c>
       <c r="E48" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.2">
@@ -1932,16 +1924,16 @@
         <v>3</v>
       </c>
       <c r="B49" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C49" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D49">
         <v>20</v>
       </c>
       <c r="E49" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.2">
@@ -1949,10 +1941,10 @@
         <v>4</v>
       </c>
       <c r="B50" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C50" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D50">
         <v>15</v>
@@ -1963,7 +1955,7 @@
         <v>5</v>
       </c>
       <c r="B51" s="14" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C51" s="14"/>
     </row>
@@ -2000,10 +1992,10 @@
         <v>6</v>
       </c>
       <c r="B60" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C60" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D60">
         <v>200</v>
@@ -2014,10 +2006,10 @@
         <v>7</v>
       </c>
       <c r="B61" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C61" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D61">
         <v>1000</v>
@@ -2028,10 +2020,10 @@
         <v>8</v>
       </c>
       <c r="B62" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C62" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.2">
@@ -2039,15 +2031,15 @@
         <v>9</v>
       </c>
       <c r="B63" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C63" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B66" s="11" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C66" s="11"/>
       <c r="D66" s="11"/>
@@ -2055,19 +2047,19 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A67" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B67" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="C67" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="B67" s="7" t="s">
+      <c r="D67" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C67" s="7" t="s">
+      <c r="E67" s="2" t="s">
         <v>66</v>
-      </c>
-      <c r="D67" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="E67" s="2" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.2">
@@ -2075,16 +2067,16 @@
         <v>1</v>
       </c>
       <c r="B68" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C68" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D68">
         <v>20</v>
       </c>
       <c r="E68" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.2">
@@ -2092,16 +2084,16 @@
         <v>2</v>
       </c>
       <c r="B69" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C69" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D69">
         <v>20</v>
       </c>
       <c r="E69" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.2">
@@ -2109,16 +2101,16 @@
         <v>3</v>
       </c>
       <c r="B70" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C70" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D70">
         <v>20</v>
       </c>
       <c r="E70" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.2">
@@ -2126,10 +2118,10 @@
         <v>4</v>
       </c>
       <c r="B71" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C71" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D71">
         <v>100</v>
@@ -2140,10 +2132,10 @@
         <v>5</v>
       </c>
       <c r="B72" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C72" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D72">
         <v>500</v>
@@ -2154,10 +2146,10 @@
         <v>6</v>
       </c>
       <c r="B73" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C73" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D73">
         <v>1000</v>
@@ -2168,10 +2160,10 @@
         <v>7</v>
       </c>
       <c r="B74" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C74" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D74">
         <v>1000</v>
@@ -2182,10 +2174,10 @@
         <v>8</v>
       </c>
       <c r="B75" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C75" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.2">
@@ -2193,15 +2185,15 @@
         <v>9</v>
       </c>
       <c r="B76" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C76" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B79" s="11" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C79" s="11"/>
       <c r="D79" s="11"/>
@@ -2209,19 +2201,19 @@
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A80" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B80" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="C80" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="B80" s="7" t="s">
+      <c r="D80" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C80" s="7" t="s">
+      <c r="E80" s="2" t="s">
         <v>66</v>
-      </c>
-      <c r="D80" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="E80" s="2" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.2">
@@ -2229,16 +2221,16 @@
         <v>1</v>
       </c>
       <c r="B81" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C81" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D81">
         <v>20</v>
       </c>
       <c r="E81" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.2">
@@ -2246,16 +2238,16 @@
         <v>2</v>
       </c>
       <c r="B82" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C82" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D82">
         <v>20</v>
       </c>
       <c r="E82" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.2">
@@ -2263,16 +2255,16 @@
         <v>3</v>
       </c>
       <c r="B83" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C83" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D83">
         <v>20</v>
       </c>
       <c r="E83" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.2">
@@ -2280,7 +2272,7 @@
         <v>4</v>
       </c>
       <c r="B84" s="14" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C84" s="15"/>
     </row>
@@ -2305,10 +2297,10 @@
         <v>5</v>
       </c>
       <c r="B89" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C89" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D89">
         <v>500</v>
@@ -2319,10 +2311,10 @@
         <v>6</v>
       </c>
       <c r="B90" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C90" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D90">
         <v>1000</v>
@@ -2330,7 +2322,7 @@
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B93" s="11" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C93" s="11"/>
       <c r="D93" s="11"/>
@@ -2338,19 +2330,19 @@
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A94" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B94" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="C94" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="B94" s="7" t="s">
+      <c r="D94" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C94" s="7" t="s">
+      <c r="E94" s="2" t="s">
         <v>66</v>
-      </c>
-      <c r="D94" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="E94" s="2" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.2">
@@ -2358,16 +2350,16 @@
         <v>1</v>
       </c>
       <c r="B95" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C95" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D95">
         <v>20</v>
       </c>
       <c r="E95" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.2">
@@ -2375,16 +2367,16 @@
         <v>2</v>
       </c>
       <c r="B96" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C96" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D96">
         <v>20</v>
       </c>
       <c r="E96" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.2">
@@ -2392,10 +2384,10 @@
         <v>3</v>
       </c>
       <c r="B97" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C97" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D97">
         <v>50</v>
@@ -2406,10 +2398,10 @@
         <v>4</v>
       </c>
       <c r="B98" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C98" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D98">
         <v>3</v>
@@ -2420,10 +2412,10 @@
         <v>5</v>
       </c>
       <c r="B99" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C99" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.2">
@@ -2431,7 +2423,7 @@
         <v>6</v>
       </c>
       <c r="B100" s="14" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C100" s="15"/>
     </row>
@@ -2445,7 +2437,7 @@
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B105" s="11" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C105" s="11"/>
       <c r="D105" s="11"/>
@@ -2453,19 +2445,19 @@
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A106" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B106" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="C106" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="B106" s="7" t="s">
+      <c r="D106" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C106" s="7" t="s">
+      <c r="E106" s="2" t="s">
         <v>66</v>
-      </c>
-      <c r="D106" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="E106" s="2" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.2">
@@ -2473,16 +2465,16 @@
         <v>1</v>
       </c>
       <c r="B107" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C107" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D107">
         <v>20</v>
       </c>
       <c r="E107" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.2">
@@ -2490,16 +2482,16 @@
         <v>2</v>
       </c>
       <c r="B108" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C108" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D108">
         <v>20</v>
       </c>
       <c r="E108" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -2532,7 +2524,7 @@
   <sheetData>
     <row r="3" spans="1:24" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="9" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B3" s="9"/>
       <c r="C3" s="9"/>
@@ -2545,7 +2537,7 @@
       <c r="J3" s="9"/>
       <c r="K3" s="9"/>
       <c r="M3" s="10" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="N3" s="10"/>
       <c r="O3" s="10"/>
@@ -3241,15 +3233,15 @@
       <c r="X32" s="10"/>
     </row>
     <row r="33" spans="1:24" ht="24" x14ac:dyDescent="0.3">
-      <c r="A33" s="18" t="s">
-        <v>128</v>
-      </c>
-      <c r="B33" s="18"/>
-      <c r="C33" s="18"/>
-      <c r="D33" s="18"/>
-      <c r="E33" s="18"/>
-      <c r="F33" s="18"/>
-      <c r="G33" s="18"/>
+      <c r="A33" s="19" t="s">
+        <v>126</v>
+      </c>
+      <c r="B33" s="19"/>
+      <c r="C33" s="19"/>
+      <c r="D33" s="19"/>
+      <c r="E33" s="19"/>
+      <c r="F33" s="19"/>
+      <c r="G33" s="19"/>
       <c r="M33" s="10"/>
       <c r="N33" s="10"/>
       <c r="O33" s="10"/>
@@ -3268,7 +3260,7 @@
         <v>1</v>
       </c>
       <c r="B34" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="M34" s="10"/>
       <c r="N34" s="10"/>
@@ -3288,7 +3280,7 @@
         <v>2</v>
       </c>
       <c r="B35" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="M35" s="10"/>
       <c r="N35" s="10"/>
@@ -3308,7 +3300,7 @@
         <v>3</v>
       </c>
       <c r="B36" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="M36" s="10"/>
       <c r="N36" s="10"/>
@@ -3328,7 +3320,7 @@
         <v>4</v>
       </c>
       <c r="B37" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="M37" s="10"/>
       <c r="N37" s="10"/>
@@ -3348,7 +3340,7 @@
         <v>5</v>
       </c>
       <c r="B38" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="M38" s="10"/>
       <c r="N38" s="10"/>
@@ -3364,6 +3356,15 @@
       <c r="X38" s="10"/>
     </row>
     <row r="39" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A39">
+        <v>6</v>
+      </c>
+      <c r="B39" s="16" t="s">
+        <v>133</v>
+      </c>
+      <c r="C39" s="17"/>
+      <c r="D39" s="17"/>
+      <c r="E39" s="17"/>
       <c r="M39" s="10"/>
       <c r="N39" s="10"/>
       <c r="O39" s="10"/>

</xml_diff>

<commit_message>
Add medicine inventory in pharmacist role
</commit_message>
<xml_diff>
--- a/CareOS-Hospital_ERP_System.xlsx
+++ b/CareOS-Hospital_ERP_System.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hetlimbani/Desktop/Self_Learning/CareOS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB9A2D45-5403-0740-93A9-62BA2816802E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDA38D97-1783-794E-88D9-D3C8BC848EAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19420" xr2:uid="{3BCF7A51-5C29-EE4C-8BC3-93CAF12DE1EA}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="133">
   <si>
     <t>Total Roles</t>
   </si>
@@ -158,9 +158,6 @@
   </si>
   <si>
     <t>Billing</t>
-  </si>
-  <si>
-    <t>Supplier Management</t>
   </si>
   <si>
     <t>Staff Management</t>
@@ -1010,7 +1007,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C1" s="13" t="s">
         <v>1</v>
@@ -1042,28 +1039,28 @@
         <v>8</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
@@ -1086,10 +1083,10 @@
         <v>36</v>
       </c>
       <c r="H4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I4" s="20" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
@@ -1112,10 +1109,10 @@
         <v>37</v>
       </c>
       <c r="H5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I5" s="20" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
@@ -1138,15 +1135,15 @@
         <v>38</v>
       </c>
       <c r="H6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I6" s="20" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B7" s="16" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C7" s="16" t="s">
         <v>18</v>
@@ -1155,21 +1152,21 @@
         <v>26</v>
       </c>
       <c r="E7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F7" s="16" t="s">
         <v>34</v>
       </c>
       <c r="H7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I7" s="20" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B8" s="16" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C8" s="16" t="s">
         <v>19</v>
@@ -1177,25 +1174,22 @@
       <c r="F8" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="G8" t="s">
-        <v>39</v>
-      </c>
       <c r="H8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C9" t="s">
         <v>17</v>
       </c>
       <c r="F9" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
@@ -1216,28 +1210,28 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B14" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
@@ -1313,13 +1307,13 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B1" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C1" s="11"/>
       <c r="D1" s="11"/>
       <c r="E1" s="11"/>
       <c r="G1" s="8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H1" s="8"/>
       <c r="I1" s="8"/>
@@ -1331,23 +1325,23 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B2" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="C2" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="D2" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>65</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>66</v>
       </c>
       <c r="F2" s="5"/>
       <c r="G2" s="8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H2" s="8"/>
       <c r="I2" s="8"/>
@@ -1362,16 +1356,16 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D3">
         <v>20</v>
       </c>
       <c r="E3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.2">
@@ -1379,10 +1373,10 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D4">
         <v>50</v>
@@ -1393,10 +1387,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D5">
         <v>50</v>
@@ -1407,16 +1401,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D6">
         <v>100</v>
       </c>
       <c r="E6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
@@ -1424,10 +1418,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D7">
         <v>100</v>
@@ -1438,10 +1432,10 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D8">
         <v>15</v>
@@ -1452,10 +1446,10 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D9">
         <v>15</v>
@@ -1466,10 +1460,10 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C10" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D10">
         <v>100</v>
@@ -1480,10 +1474,10 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D11">
         <v>1</v>
@@ -1494,10 +1488,10 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.2">
@@ -1505,15 +1499,15 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C13" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B16" s="11" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C16" s="11"/>
       <c r="D16" s="11"/>
@@ -1521,19 +1515,19 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B17" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="C17" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="D17" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="E17" s="2" t="s">
         <v>65</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
@@ -1541,16 +1535,16 @@
         <v>1</v>
       </c>
       <c r="B18" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C18" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D18">
         <v>20</v>
       </c>
       <c r="E18" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
@@ -1558,16 +1552,16 @@
         <v>2</v>
       </c>
       <c r="B19" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C19" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D19">
         <v>20</v>
       </c>
       <c r="E19" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
@@ -1575,10 +1569,10 @@
         <v>3</v>
       </c>
       <c r="B20" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C20" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
@@ -1586,10 +1580,10 @@
         <v>4</v>
       </c>
       <c r="B21" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C21" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D21">
         <v>10</v>
@@ -1600,10 +1594,10 @@
         <v>5</v>
       </c>
       <c r="B22" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C22" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D22">
         <v>5</v>
@@ -1614,10 +1608,10 @@
         <v>6</v>
       </c>
       <c r="B23" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C23" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D23">
         <v>200</v>
@@ -1628,10 +1622,10 @@
         <v>7</v>
       </c>
       <c r="B24" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C24" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D24">
         <v>50</v>
@@ -1642,10 +1636,10 @@
         <v>8</v>
       </c>
       <c r="B25" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C25" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D25">
         <v>15</v>
@@ -1656,10 +1650,10 @@
         <v>9</v>
       </c>
       <c r="B26" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C26" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D26">
         <v>15</v>
@@ -1670,10 +1664,10 @@
         <v>10</v>
       </c>
       <c r="B27" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C27" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D27">
         <v>50</v>
@@ -1684,10 +1678,10 @@
         <v>11</v>
       </c>
       <c r="B28" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C28" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D28">
         <v>15</v>
@@ -1698,10 +1692,10 @@
         <v>12</v>
       </c>
       <c r="B29" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C29" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D29">
         <v>15</v>
@@ -1712,10 +1706,10 @@
         <v>13</v>
       </c>
       <c r="B30" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C30" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D30">
         <v>50</v>
@@ -1726,10 +1720,10 @@
         <v>14</v>
       </c>
       <c r="B31" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C31" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D31">
         <v>20</v>
@@ -1742,7 +1736,7 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B34" s="11" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C34" s="11"/>
       <c r="D34" s="11"/>
@@ -1750,19 +1744,19 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B35" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="B35" s="7" t="s">
+      <c r="C35" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="C35" s="7" t="s">
+      <c r="D35" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="D35" s="2" t="s">
+      <c r="E35" s="2" t="s">
         <v>65</v>
-      </c>
-      <c r="E35" s="2" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
@@ -1770,16 +1764,16 @@
         <v>1</v>
       </c>
       <c r="B36" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C36" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D36">
         <v>20</v>
       </c>
       <c r="E36" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
@@ -1787,16 +1781,16 @@
         <v>2</v>
       </c>
       <c r="B37" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C37" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D37">
         <v>20</v>
       </c>
       <c r="E37" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
@@ -1804,10 +1798,10 @@
         <v>3</v>
       </c>
       <c r="B38" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C38" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D38">
         <v>50</v>
@@ -1818,10 +1812,10 @@
         <v>4</v>
       </c>
       <c r="B39" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C39" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D39">
         <v>50</v>
@@ -1832,10 +1826,10 @@
         <v>5</v>
       </c>
       <c r="B40" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C40" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
@@ -1843,10 +1837,10 @@
         <v>6</v>
       </c>
       <c r="B41" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C41" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D41">
         <v>15</v>
@@ -1857,12 +1851,12 @@
         <v>7</v>
       </c>
       <c r="B42" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B45" s="11" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C45" s="11"/>
       <c r="D45" s="11"/>
@@ -1870,19 +1864,19 @@
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B46" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="B46" s="7" t="s">
+      <c r="C46" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="C46" s="7" t="s">
+      <c r="D46" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="D46" s="2" t="s">
+      <c r="E46" s="2" t="s">
         <v>65</v>
-      </c>
-      <c r="E46" s="2" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.2">
@@ -1890,16 +1884,16 @@
         <v>1</v>
       </c>
       <c r="B47" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C47" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D47">
         <v>20</v>
       </c>
       <c r="E47" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.2">
@@ -1907,16 +1901,16 @@
         <v>2</v>
       </c>
       <c r="B48" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C48" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D48">
         <v>20</v>
       </c>
       <c r="E48" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.2">
@@ -1924,16 +1918,16 @@
         <v>3</v>
       </c>
       <c r="B49" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C49" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D49">
         <v>20</v>
       </c>
       <c r="E49" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.2">
@@ -1941,10 +1935,10 @@
         <v>4</v>
       </c>
       <c r="B50" t="s">
+        <v>86</v>
+      </c>
+      <c r="C50" t="s">
         <v>87</v>
-      </c>
-      <c r="C50" t="s">
-        <v>88</v>
       </c>
       <c r="D50">
         <v>15</v>
@@ -1955,7 +1949,7 @@
         <v>5</v>
       </c>
       <c r="B51" s="14" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C51" s="14"/>
     </row>
@@ -1992,10 +1986,10 @@
         <v>6</v>
       </c>
       <c r="B60" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C60" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D60">
         <v>200</v>
@@ -2006,10 +2000,10 @@
         <v>7</v>
       </c>
       <c r="B61" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C61" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D61">
         <v>1000</v>
@@ -2020,10 +2014,10 @@
         <v>8</v>
       </c>
       <c r="B62" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C62" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.2">
@@ -2031,15 +2025,15 @@
         <v>9</v>
       </c>
       <c r="B63" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C63" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B66" s="11" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C66" s="11"/>
       <c r="D66" s="11"/>
@@ -2047,19 +2041,19 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A67" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B67" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="B67" s="7" t="s">
+      <c r="C67" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="C67" s="7" t="s">
+      <c r="D67" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="D67" s="2" t="s">
+      <c r="E67" s="2" t="s">
         <v>65</v>
-      </c>
-      <c r="E67" s="2" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.2">
@@ -2067,16 +2061,16 @@
         <v>1</v>
       </c>
       <c r="B68" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C68" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D68">
         <v>20</v>
       </c>
       <c r="E68" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.2">
@@ -2084,16 +2078,16 @@
         <v>2</v>
       </c>
       <c r="B69" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C69" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D69">
         <v>20</v>
       </c>
       <c r="E69" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.2">
@@ -2101,16 +2095,16 @@
         <v>3</v>
       </c>
       <c r="B70" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C70" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D70">
         <v>20</v>
       </c>
       <c r="E70" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.2">
@@ -2118,10 +2112,10 @@
         <v>4</v>
       </c>
       <c r="B71" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C71" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D71">
         <v>100</v>
@@ -2132,10 +2126,10 @@
         <v>5</v>
       </c>
       <c r="B72" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C72" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D72">
         <v>500</v>
@@ -2146,10 +2140,10 @@
         <v>6</v>
       </c>
       <c r="B73" t="s">
+        <v>110</v>
+      </c>
+      <c r="C73" t="s">
         <v>111</v>
-      </c>
-      <c r="C73" t="s">
-        <v>112</v>
       </c>
       <c r="D73">
         <v>1000</v>
@@ -2160,10 +2154,10 @@
         <v>7</v>
       </c>
       <c r="B74" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C74" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D74">
         <v>1000</v>
@@ -2174,10 +2168,10 @@
         <v>8</v>
       </c>
       <c r="B75" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C75" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.2">
@@ -2185,15 +2179,15 @@
         <v>9</v>
       </c>
       <c r="B76" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C76" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B79" s="11" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C79" s="11"/>
       <c r="D79" s="11"/>
@@ -2201,19 +2195,19 @@
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A80" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B80" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="B80" s="7" t="s">
+      <c r="C80" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="C80" s="7" t="s">
+      <c r="D80" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="D80" s="2" t="s">
+      <c r="E80" s="2" t="s">
         <v>65</v>
-      </c>
-      <c r="E80" s="2" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.2">
@@ -2221,16 +2215,16 @@
         <v>1</v>
       </c>
       <c r="B81" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C81" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D81">
         <v>20</v>
       </c>
       <c r="E81" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.2">
@@ -2238,16 +2232,16 @@
         <v>2</v>
       </c>
       <c r="B82" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C82" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D82">
         <v>20</v>
       </c>
       <c r="E82" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.2">
@@ -2255,16 +2249,16 @@
         <v>3</v>
       </c>
       <c r="B83" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C83" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D83">
         <v>20</v>
       </c>
       <c r="E83" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.2">
@@ -2272,7 +2266,7 @@
         <v>4</v>
       </c>
       <c r="B84" s="14" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C84" s="15"/>
     </row>
@@ -2297,10 +2291,10 @@
         <v>5</v>
       </c>
       <c r="B89" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C89" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D89">
         <v>500</v>
@@ -2311,10 +2305,10 @@
         <v>6</v>
       </c>
       <c r="B90" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C90" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D90">
         <v>1000</v>
@@ -2322,7 +2316,7 @@
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B93" s="11" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C93" s="11"/>
       <c r="D93" s="11"/>
@@ -2330,19 +2324,19 @@
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A94" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B94" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="B94" s="7" t="s">
+      <c r="C94" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="C94" s="7" t="s">
+      <c r="D94" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="D94" s="2" t="s">
+      <c r="E94" s="2" t="s">
         <v>65</v>
-      </c>
-      <c r="E94" s="2" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.2">
@@ -2350,16 +2344,16 @@
         <v>1</v>
       </c>
       <c r="B95" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C95" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D95">
         <v>20</v>
       </c>
       <c r="E95" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.2">
@@ -2367,16 +2361,16 @@
         <v>2</v>
       </c>
       <c r="B96" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C96" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D96">
         <v>20</v>
       </c>
       <c r="E96" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.2">
@@ -2384,10 +2378,10 @@
         <v>3</v>
       </c>
       <c r="B97" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C97" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D97">
         <v>50</v>
@@ -2398,10 +2392,10 @@
         <v>4</v>
       </c>
       <c r="B98" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C98" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D98">
         <v>3</v>
@@ -2412,10 +2406,10 @@
         <v>5</v>
       </c>
       <c r="B99" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C99" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.2">
@@ -2423,7 +2417,7 @@
         <v>6</v>
       </c>
       <c r="B100" s="14" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C100" s="15"/>
     </row>
@@ -2437,7 +2431,7 @@
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B105" s="11" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C105" s="11"/>
       <c r="D105" s="11"/>
@@ -2445,19 +2439,19 @@
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A106" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B106" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="B106" s="7" t="s">
+      <c r="C106" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="C106" s="7" t="s">
+      <c r="D106" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="D106" s="2" t="s">
+      <c r="E106" s="2" t="s">
         <v>65</v>
-      </c>
-      <c r="E106" s="2" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.2">
@@ -2465,16 +2459,16 @@
         <v>1</v>
       </c>
       <c r="B107" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C107" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D107">
         <v>20</v>
       </c>
       <c r="E107" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.2">
@@ -2482,16 +2476,16 @@
         <v>2</v>
       </c>
       <c r="B108" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C108" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D108">
         <v>20</v>
       </c>
       <c r="E108" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -2524,7 +2518,7 @@
   <sheetData>
     <row r="3" spans="1:24" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B3" s="9"/>
       <c r="C3" s="9"/>
@@ -2537,7 +2531,7 @@
       <c r="J3" s="9"/>
       <c r="K3" s="9"/>
       <c r="M3" s="10" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="N3" s="10"/>
       <c r="O3" s="10"/>
@@ -3234,7 +3228,7 @@
     </row>
     <row r="33" spans="1:24" ht="24" x14ac:dyDescent="0.3">
       <c r="A33" s="19" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B33" s="19"/>
       <c r="C33" s="19"/>
@@ -3260,7 +3254,7 @@
         <v>1</v>
       </c>
       <c r="B34" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="M34" s="10"/>
       <c r="N34" s="10"/>
@@ -3280,7 +3274,7 @@
         <v>2</v>
       </c>
       <c r="B35" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="M35" s="10"/>
       <c r="N35" s="10"/>
@@ -3300,7 +3294,7 @@
         <v>3</v>
       </c>
       <c r="B36" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="M36" s="10"/>
       <c r="N36" s="10"/>
@@ -3320,7 +3314,7 @@
         <v>4</v>
       </c>
       <c r="B37" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="M37" s="10"/>
       <c r="N37" s="10"/>
@@ -3340,7 +3334,7 @@
         <v>5</v>
       </c>
       <c r="B38" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="M38" s="10"/>
       <c r="N38" s="10"/>
@@ -3360,7 +3354,7 @@
         <v>6</v>
       </c>
       <c r="B39" s="16" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C39" s="17"/>
       <c r="D39" s="17"/>

</xml_diff>

<commit_message>
admission process work intialize for receptionist role
</commit_message>
<xml_diff>
--- a/CareOS-Hospital_ERP_System.xlsx
+++ b/CareOS-Hospital_ERP_System.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hetlimbani/Desktop/Self_Learning/CareOS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDA38D97-1783-794E-88D9-D3C8BC848EAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F6CB6AC-05FF-0147-8AD5-B97C90CC276F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19420" xr2:uid="{3BCF7A51-5C29-EE4C-8BC3-93CAF12DE1EA}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="132">
   <si>
     <t>Total Roles</t>
   </si>
@@ -116,9 +116,6 @@
   </si>
   <si>
     <t>Shift Management</t>
-  </si>
-  <si>
-    <t>Emergency Alerts</t>
   </si>
   <si>
     <t>Assigned Tasks</t>
@@ -1007,7 +1004,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C1" s="13" t="s">
         <v>1</v>
@@ -1039,28 +1036,28 @@
         <v>8</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
@@ -1076,17 +1073,17 @@
       <c r="E4" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="F4" s="16" t="s">
-        <v>31</v>
+      <c r="F4" t="s">
+        <v>13</v>
       </c>
       <c r="G4" t="s">
-        <v>36</v>
+        <v>13</v>
       </c>
       <c r="H4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I4" s="20" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
@@ -1100,19 +1097,19 @@
         <v>23</v>
       </c>
       <c r="E5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F5" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="F5" s="16" t="s">
-        <v>32</v>
-      </c>
       <c r="G5" s="16" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I5" s="20" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
@@ -1123,73 +1120,76 @@
         <v>16</v>
       </c>
       <c r="D6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F6" s="16" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="H6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I6" s="20" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B7" s="16" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C7" s="16" t="s">
         <v>18</v>
       </c>
       <c r="D7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>34</v>
+        <v>32</v>
+      </c>
+      <c r="G7" s="16" t="s">
+        <v>37</v>
       </c>
       <c r="H7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I7" s="20" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B8" s="16" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C8" s="16" t="s">
         <v>19</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="H8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C9" t="s">
         <v>17</v>
       </c>
-      <c r="F9" t="s">
-        <v>52</v>
+      <c r="F9" s="16" t="s">
+        <v>34</v>
       </c>
       <c r="H9" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
@@ -1199,6 +1199,9 @@
       <c r="C10" t="s">
         <v>21</v>
       </c>
+      <c r="F10" s="16" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="C11" s="16" t="s">
@@ -1210,28 +1213,28 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B14" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
@@ -1242,7 +1245,7 @@
         <v>14</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E15" t="s">
         <v>14</v>
@@ -1276,12 +1279,7 @@
         <v>14</v>
       </c>
       <c r="C17" s="4"/>
-      <c r="D17" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="D18" t="s">
+      <c r="D17" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1307,13 +1305,13 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B1" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C1" s="11"/>
       <c r="D1" s="11"/>
       <c r="E1" s="11"/>
       <c r="G1" s="8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="H1" s="8"/>
       <c r="I1" s="8"/>
@@ -1325,23 +1323,23 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B2" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="C2" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="D2" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>64</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>65</v>
       </c>
       <c r="F2" s="5"/>
       <c r="G2" s="8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H2" s="8"/>
       <c r="I2" s="8"/>
@@ -1356,16 +1354,16 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D3">
         <v>20</v>
       </c>
       <c r="E3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.2">
@@ -1373,10 +1371,10 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D4">
         <v>50</v>
@@ -1387,10 +1385,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D5">
         <v>50</v>
@@ -1401,16 +1399,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D6">
         <v>100</v>
       </c>
       <c r="E6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
@@ -1418,10 +1416,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D7">
         <v>100</v>
@@ -1432,10 +1430,10 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D8">
         <v>15</v>
@@ -1446,10 +1444,10 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D9">
         <v>15</v>
@@ -1460,10 +1458,10 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D10">
         <v>100</v>
@@ -1474,10 +1472,10 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C11" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D11">
         <v>1</v>
@@ -1488,10 +1486,10 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.2">
@@ -1499,15 +1497,15 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C13" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B16" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C16" s="11"/>
       <c r="D16" s="11"/>
@@ -1515,19 +1513,19 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B17" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="C17" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="D17" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="E17" s="2" t="s">
         <v>64</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
@@ -1535,16 +1533,16 @@
         <v>1</v>
       </c>
       <c r="B18" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C18" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D18">
         <v>20</v>
       </c>
       <c r="E18" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
@@ -1552,16 +1550,16 @@
         <v>2</v>
       </c>
       <c r="B19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C19" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D19">
         <v>20</v>
       </c>
       <c r="E19" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
@@ -1569,10 +1567,10 @@
         <v>3</v>
       </c>
       <c r="B20" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C20" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
@@ -1580,10 +1578,10 @@
         <v>4</v>
       </c>
       <c r="B21" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C21" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D21">
         <v>10</v>
@@ -1594,10 +1592,10 @@
         <v>5</v>
       </c>
       <c r="B22" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C22" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D22">
         <v>5</v>
@@ -1608,10 +1606,10 @@
         <v>6</v>
       </c>
       <c r="B23" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C23" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D23">
         <v>200</v>
@@ -1622,10 +1620,10 @@
         <v>7</v>
       </c>
       <c r="B24" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C24" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D24">
         <v>50</v>
@@ -1636,10 +1634,10 @@
         <v>8</v>
       </c>
       <c r="B25" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C25" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D25">
         <v>15</v>
@@ -1650,10 +1648,10 @@
         <v>9</v>
       </c>
       <c r="B26" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C26" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D26">
         <v>15</v>
@@ -1664,10 +1662,10 @@
         <v>10</v>
       </c>
       <c r="B27" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C27" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D27">
         <v>50</v>
@@ -1678,10 +1676,10 @@
         <v>11</v>
       </c>
       <c r="B28" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C28" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D28">
         <v>15</v>
@@ -1692,10 +1690,10 @@
         <v>12</v>
       </c>
       <c r="B29" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C29" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D29">
         <v>15</v>
@@ -1706,10 +1704,10 @@
         <v>13</v>
       </c>
       <c r="B30" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C30" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D30">
         <v>50</v>
@@ -1720,10 +1718,10 @@
         <v>14</v>
       </c>
       <c r="B31" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C31" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D31">
         <v>20</v>
@@ -1736,7 +1734,7 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B34" s="11" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C34" s="11"/>
       <c r="D34" s="11"/>
@@ -1744,19 +1742,19 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B35" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="B35" s="7" t="s">
+      <c r="C35" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="C35" s="7" t="s">
+      <c r="D35" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D35" s="2" t="s">
+      <c r="E35" s="2" t="s">
         <v>64</v>
-      </c>
-      <c r="E35" s="2" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
@@ -1764,16 +1762,16 @@
         <v>1</v>
       </c>
       <c r="B36" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C36" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D36">
         <v>20</v>
       </c>
       <c r="E36" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
@@ -1781,16 +1779,16 @@
         <v>2</v>
       </c>
       <c r="B37" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C37" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D37">
         <v>20</v>
       </c>
       <c r="E37" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
@@ -1798,10 +1796,10 @@
         <v>3</v>
       </c>
       <c r="B38" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C38" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D38">
         <v>50</v>
@@ -1812,10 +1810,10 @@
         <v>4</v>
       </c>
       <c r="B39" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C39" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D39">
         <v>50</v>
@@ -1826,10 +1824,10 @@
         <v>5</v>
       </c>
       <c r="B40" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C40" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
@@ -1837,10 +1835,10 @@
         <v>6</v>
       </c>
       <c r="B41" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C41" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D41">
         <v>15</v>
@@ -1851,12 +1849,12 @@
         <v>7</v>
       </c>
       <c r="B42" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B45" s="11" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C45" s="11"/>
       <c r="D45" s="11"/>
@@ -1864,19 +1862,19 @@
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B46" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="B46" s="7" t="s">
+      <c r="C46" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="C46" s="7" t="s">
+      <c r="D46" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D46" s="2" t="s">
+      <c r="E46" s="2" t="s">
         <v>64</v>
-      </c>
-      <c r="E46" s="2" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.2">
@@ -1884,16 +1882,16 @@
         <v>1</v>
       </c>
       <c r="B47" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C47" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D47">
         <v>20</v>
       </c>
       <c r="E47" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.2">
@@ -1901,16 +1899,16 @@
         <v>2</v>
       </c>
       <c r="B48" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C48" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D48">
         <v>20</v>
       </c>
       <c r="E48" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.2">
@@ -1918,16 +1916,16 @@
         <v>3</v>
       </c>
       <c r="B49" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C49" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D49">
         <v>20</v>
       </c>
       <c r="E49" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.2">
@@ -1935,10 +1933,10 @@
         <v>4</v>
       </c>
       <c r="B50" t="s">
+        <v>85</v>
+      </c>
+      <c r="C50" t="s">
         <v>86</v>
-      </c>
-      <c r="C50" t="s">
-        <v>87</v>
       </c>
       <c r="D50">
         <v>15</v>
@@ -1949,7 +1947,7 @@
         <v>5</v>
       </c>
       <c r="B51" s="14" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C51" s="14"/>
     </row>
@@ -1986,10 +1984,10 @@
         <v>6</v>
       </c>
       <c r="B60" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C60" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D60">
         <v>200</v>
@@ -2000,10 +1998,10 @@
         <v>7</v>
       </c>
       <c r="B61" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C61" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D61">
         <v>1000</v>
@@ -2014,10 +2012,10 @@
         <v>8</v>
       </c>
       <c r="B62" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C62" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.2">
@@ -2025,15 +2023,15 @@
         <v>9</v>
       </c>
       <c r="B63" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C63" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B66" s="11" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C66" s="11"/>
       <c r="D66" s="11"/>
@@ -2041,19 +2039,19 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A67" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B67" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="B67" s="7" t="s">
+      <c r="C67" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="C67" s="7" t="s">
+      <c r="D67" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D67" s="2" t="s">
+      <c r="E67" s="2" t="s">
         <v>64</v>
-      </c>
-      <c r="E67" s="2" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.2">
@@ -2061,16 +2059,16 @@
         <v>1</v>
       </c>
       <c r="B68" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C68" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D68">
         <v>20</v>
       </c>
       <c r="E68" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.2">
@@ -2078,16 +2076,16 @@
         <v>2</v>
       </c>
       <c r="B69" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C69" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D69">
         <v>20</v>
       </c>
       <c r="E69" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.2">
@@ -2095,16 +2093,16 @@
         <v>3</v>
       </c>
       <c r="B70" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C70" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D70">
         <v>20</v>
       </c>
       <c r="E70" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.2">
@@ -2112,10 +2110,10 @@
         <v>4</v>
       </c>
       <c r="B71" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C71" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D71">
         <v>100</v>
@@ -2126,10 +2124,10 @@
         <v>5</v>
       </c>
       <c r="B72" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C72" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D72">
         <v>500</v>
@@ -2140,10 +2138,10 @@
         <v>6</v>
       </c>
       <c r="B73" t="s">
+        <v>109</v>
+      </c>
+      <c r="C73" t="s">
         <v>110</v>
-      </c>
-      <c r="C73" t="s">
-        <v>111</v>
       </c>
       <c r="D73">
         <v>1000</v>
@@ -2154,10 +2152,10 @@
         <v>7</v>
       </c>
       <c r="B74" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C74" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D74">
         <v>1000</v>
@@ -2168,10 +2166,10 @@
         <v>8</v>
       </c>
       <c r="B75" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C75" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.2">
@@ -2179,15 +2177,15 @@
         <v>9</v>
       </c>
       <c r="B76" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C76" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B79" s="11" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C79" s="11"/>
       <c r="D79" s="11"/>
@@ -2195,19 +2193,19 @@
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A80" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B80" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="B80" s="7" t="s">
+      <c r="C80" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="C80" s="7" t="s">
+      <c r="D80" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D80" s="2" t="s">
+      <c r="E80" s="2" t="s">
         <v>64</v>
-      </c>
-      <c r="E80" s="2" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.2">
@@ -2215,16 +2213,16 @@
         <v>1</v>
       </c>
       <c r="B81" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C81" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D81">
         <v>20</v>
       </c>
       <c r="E81" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.2">
@@ -2232,16 +2230,16 @@
         <v>2</v>
       </c>
       <c r="B82" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C82" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D82">
         <v>20</v>
       </c>
       <c r="E82" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.2">
@@ -2249,16 +2247,16 @@
         <v>3</v>
       </c>
       <c r="B83" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C83" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D83">
         <v>20</v>
       </c>
       <c r="E83" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.2">
@@ -2266,7 +2264,7 @@
         <v>4</v>
       </c>
       <c r="B84" s="14" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C84" s="15"/>
     </row>
@@ -2291,10 +2289,10 @@
         <v>5</v>
       </c>
       <c r="B89" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C89" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D89">
         <v>500</v>
@@ -2305,10 +2303,10 @@
         <v>6</v>
       </c>
       <c r="B90" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C90" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D90">
         <v>1000</v>
@@ -2316,7 +2314,7 @@
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B93" s="11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C93" s="11"/>
       <c r="D93" s="11"/>
@@ -2324,19 +2322,19 @@
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A94" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B94" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="B94" s="7" t="s">
+      <c r="C94" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="C94" s="7" t="s">
+      <c r="D94" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D94" s="2" t="s">
+      <c r="E94" s="2" t="s">
         <v>64</v>
-      </c>
-      <c r="E94" s="2" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.2">
@@ -2344,16 +2342,16 @@
         <v>1</v>
       </c>
       <c r="B95" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C95" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D95">
         <v>20</v>
       </c>
       <c r="E95" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.2">
@@ -2361,16 +2359,16 @@
         <v>2</v>
       </c>
       <c r="B96" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C96" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D96">
         <v>20</v>
       </c>
       <c r="E96" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.2">
@@ -2378,10 +2376,10 @@
         <v>3</v>
       </c>
       <c r="B97" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C97" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D97">
         <v>50</v>
@@ -2392,10 +2390,10 @@
         <v>4</v>
       </c>
       <c r="B98" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C98" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D98">
         <v>3</v>
@@ -2406,10 +2404,10 @@
         <v>5</v>
       </c>
       <c r="B99" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C99" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.2">
@@ -2417,7 +2415,7 @@
         <v>6</v>
       </c>
       <c r="B100" s="14" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C100" s="15"/>
     </row>
@@ -2431,7 +2429,7 @@
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B105" s="11" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C105" s="11"/>
       <c r="D105" s="11"/>
@@ -2439,19 +2437,19 @@
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A106" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B106" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="B106" s="7" t="s">
+      <c r="C106" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="C106" s="7" t="s">
+      <c r="D106" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D106" s="2" t="s">
+      <c r="E106" s="2" t="s">
         <v>64</v>
-      </c>
-      <c r="E106" s="2" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.2">
@@ -2459,16 +2457,16 @@
         <v>1</v>
       </c>
       <c r="B107" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C107" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D107">
         <v>20</v>
       </c>
       <c r="E107" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.2">
@@ -2476,16 +2474,16 @@
         <v>2</v>
       </c>
       <c r="B108" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C108" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D108">
         <v>20</v>
       </c>
       <c r="E108" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -2518,7 +2516,7 @@
   <sheetData>
     <row r="3" spans="1:24" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B3" s="9"/>
       <c r="C3" s="9"/>
@@ -2531,7 +2529,7 @@
       <c r="J3" s="9"/>
       <c r="K3" s="9"/>
       <c r="M3" s="10" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="N3" s="10"/>
       <c r="O3" s="10"/>
@@ -3228,7 +3226,7 @@
     </row>
     <row r="33" spans="1:24" ht="24" x14ac:dyDescent="0.3">
       <c r="A33" s="19" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B33" s="19"/>
       <c r="C33" s="19"/>
@@ -3254,7 +3252,7 @@
         <v>1</v>
       </c>
       <c r="B34" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="M34" s="10"/>
       <c r="N34" s="10"/>
@@ -3274,7 +3272,7 @@
         <v>2</v>
       </c>
       <c r="B35" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="M35" s="10"/>
       <c r="N35" s="10"/>
@@ -3294,7 +3292,7 @@
         <v>3</v>
       </c>
       <c r="B36" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="M36" s="10"/>
       <c r="N36" s="10"/>
@@ -3314,7 +3312,7 @@
         <v>4</v>
       </c>
       <c r="B37" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="M37" s="10"/>
       <c r="N37" s="10"/>
@@ -3334,7 +3332,7 @@
         <v>5</v>
       </c>
       <c r="B38" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="M38" s="10"/>
       <c r="N38" s="10"/>
@@ -3354,7 +3352,7 @@
         <v>6</v>
       </c>
       <c r="B39" s="16" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C39" s="17"/>
       <c r="D39" s="17"/>

</xml_diff>

<commit_message>
Added request consultancy backend and frontend for receptionist role
</commit_message>
<xml_diff>
--- a/CareOS-Hospital_ERP_System.xlsx
+++ b/CareOS-Hospital_ERP_System.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hetlimbani/Desktop/Self_Learning/CareOS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F6CB6AC-05FF-0147-8AD5-B97C90CC276F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1947C72-1928-A743-B258-7B6CC3320418}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19420" xr2:uid="{3BCF7A51-5C29-EE4C-8BC3-93CAF12DE1EA}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="135">
   <si>
     <t>Total Roles</t>
   </si>
@@ -489,6 +489,15 @@
   </si>
   <si>
     <t>In E-prescription add not required field in medicine and lab report at doctor role</t>
+  </si>
+  <si>
+    <t>Add request consultancy by patient store in receptionsit role</t>
+  </si>
+  <si>
+    <t>update data in landing page</t>
+  </si>
+  <si>
+    <t>Consultation request</t>
   </si>
 </sst>
 </file>
@@ -1122,8 +1131,8 @@
       <c r="D6" t="s">
         <v>26</v>
       </c>
-      <c r="E6" t="s">
-        <v>28</v>
+      <c r="E6" s="16" t="s">
+        <v>134</v>
       </c>
       <c r="F6" s="16" t="s">
         <v>31</v>
@@ -1149,7 +1158,7 @@
         <v>25</v>
       </c>
       <c r="E7" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="F7" s="16" t="s">
         <v>32</v>
@@ -1170,6 +1179,9 @@
       </c>
       <c r="C8" s="16" t="s">
         <v>19</v>
+      </c>
+      <c r="E8" t="s">
+        <v>51</v>
       </c>
       <c r="F8" s="16" t="s">
         <v>33</v>
@@ -3371,6 +3383,12 @@
       <c r="X39" s="10"/>
     </row>
     <row r="40" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A40">
+        <v>7</v>
+      </c>
+      <c r="B40" t="s">
+        <v>132</v>
+      </c>
       <c r="M40" s="10"/>
       <c r="N40" s="10"/>
       <c r="O40" s="10"/>
@@ -3385,6 +3403,12 @@
       <c r="X40" s="10"/>
     </row>
     <row r="41" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A41">
+        <v>8</v>
+      </c>
+      <c r="B41" t="s">
+        <v>133</v>
+      </c>
       <c r="M41" s="10"/>
       <c r="N41" s="10"/>
       <c r="O41" s="10"/>

</xml_diff>

<commit_message>
Add patent record file in nurse role
</commit_message>
<xml_diff>
--- a/CareOS-Hospital_ERP_System.xlsx
+++ b/CareOS-Hospital_ERP_System.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hetlimbani/Desktop/Self_Learning/CareOS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BA9B325-4980-1A40-853B-28E6E9AB851E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1D95565-9B04-734E-9F32-8CC1CE99E3DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19420" xr2:uid="{3BCF7A51-5C29-EE4C-8BC3-93CAF12DE1EA}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="147">
   <si>
     <t>Total Roles</t>
   </si>
@@ -527,6 +527,9 @@
   </si>
   <si>
     <t>message</t>
+  </si>
+  <si>
+    <t>patient lab record</t>
   </si>
 </sst>
 </file>
@@ -1102,7 +1105,7 @@
       <c r="C4" t="s">
         <v>13</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="15" t="s">
         <v>22</v>
       </c>
       <c r="E4" s="21" t="s">
@@ -1205,6 +1208,9 @@
       </c>
       <c r="C8" s="15" t="s">
         <v>19</v>
+      </c>
+      <c r="D8" s="15" t="s">
+        <v>146</v>
       </c>
       <c r="E8" t="s">
         <v>51</v>

</xml_diff>

<commit_message>
Add ward review in doctor role
</commit_message>
<xml_diff>
--- a/CareOS-Hospital_ERP_System.xlsx
+++ b/CareOS-Hospital_ERP_System.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hetlimbani/Desktop/Self_Learning/CareOS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1D95565-9B04-734E-9F32-8CC1CE99E3DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{833C039B-B0B0-EF40-93A0-D24CA074E828}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19420" xr2:uid="{3BCF7A51-5C29-EE4C-8BC3-93CAF12DE1EA}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19420" activeTab="2" xr2:uid="{3BCF7A51-5C29-EE4C-8BC3-93CAF12DE1EA}"/>
   </bookViews>
   <sheets>
     <sheet name="ERP System" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="148">
   <si>
     <t>Total Roles</t>
   </si>
@@ -119,9 +119,6 @@
   </si>
   <si>
     <t>Assigned Tasks</t>
-  </si>
-  <si>
-    <t>Medicine Administration (Description)</t>
   </si>
   <si>
     <t>Reminder</t>
@@ -530,6 +527,12 @@
   </si>
   <si>
     <t>patient lab record</t>
+  </si>
+  <si>
+    <t>E-Prescription record file</t>
+  </si>
+  <si>
+    <t>Edit lab report functionality after adding new  lab report by nurse or doctor in lab technician role</t>
   </si>
 </sst>
 </file>
@@ -1042,7 +1045,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C1" s="12" t="s">
         <v>1</v>
@@ -1074,28 +1077,28 @@
         <v>8</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
@@ -1118,10 +1121,10 @@
         <v>13</v>
       </c>
       <c r="H4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I4" s="19" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
@@ -1135,19 +1138,19 @@
         <v>23</v>
       </c>
       <c r="E5" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="F5" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="F5" s="15" t="s">
-        <v>30</v>
-      </c>
       <c r="G5" s="15" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I5" s="19" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
@@ -1157,28 +1160,28 @@
       <c r="C6" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="D6" t="s">
-        <v>26</v>
+      <c r="D6" s="15" t="s">
+        <v>146</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F6" s="15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G6" s="15" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I6" s="19" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B7" s="15" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C7" s="15" t="s">
         <v>18</v>
@@ -1187,53 +1190,53 @@
         <v>25</v>
       </c>
       <c r="E7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G7" s="15" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I7" s="19" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B8" s="15" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C8" s="15" t="s">
         <v>19</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F8" s="15" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C9" t="s">
         <v>17</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
@@ -1244,7 +1247,7 @@
         <v>21</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
@@ -1257,28 +1260,28 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B14" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
@@ -1289,7 +1292,7 @@
         <v>14</v>
       </c>
       <c r="D15" s="20" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E15" t="s">
         <v>14</v>
@@ -1349,7 +1352,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B1" s="10" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C1" s="10"/>
       <c r="D1" s="10"/>
@@ -1357,19 +1360,19 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B2" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="C2" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="D2" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>61</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>62</v>
       </c>
       <c r="F2" s="5"/>
     </row>
@@ -1378,16 +1381,16 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D3">
         <v>20</v>
       </c>
       <c r="E3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -1395,10 +1398,10 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D4">
         <v>50</v>
@@ -1409,10 +1412,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D5">
         <v>50</v>
@@ -1423,16 +1426,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D6">
         <v>100</v>
       </c>
       <c r="E6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -1440,10 +1443,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D7">
         <v>100</v>
@@ -1454,10 +1457,10 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C8" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D8">
         <v>15</v>
@@ -1468,10 +1471,10 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D9">
         <v>5</v>
@@ -1482,10 +1485,10 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D10">
         <v>15</v>
@@ -1496,10 +1499,10 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C11" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D11">
         <v>100</v>
@@ -1510,10 +1513,10 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C12" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D12">
         <v>1</v>
@@ -1524,10 +1527,10 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C13" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -1535,15 +1538,15 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C14" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B17" s="10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C17" s="10"/>
       <c r="D17" s="10"/>
@@ -1551,19 +1554,19 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B18" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="C18" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="D18" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="E18" s="2" t="s">
         <v>61</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
@@ -1571,16 +1574,16 @@
         <v>1</v>
       </c>
       <c r="B19" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C19" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D19">
         <v>20</v>
       </c>
       <c r="E19" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
@@ -1588,16 +1591,16 @@
         <v>2</v>
       </c>
       <c r="B20" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C20" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D20">
         <v>20</v>
       </c>
       <c r="E20" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
@@ -1605,10 +1608,10 @@
         <v>3</v>
       </c>
       <c r="B21" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C21" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
@@ -1616,10 +1619,10 @@
         <v>4</v>
       </c>
       <c r="B22" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C22" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D22">
         <v>10</v>
@@ -1630,10 +1633,10 @@
         <v>5</v>
       </c>
       <c r="B23" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C23" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D23">
         <v>5</v>
@@ -1644,10 +1647,10 @@
         <v>6</v>
       </c>
       <c r="B24" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D24">
         <v>200</v>
@@ -1658,10 +1661,10 @@
         <v>7</v>
       </c>
       <c r="B25" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C25" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D25">
         <v>50</v>
@@ -1672,10 +1675,10 @@
         <v>8</v>
       </c>
       <c r="B26" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C26" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D26">
         <v>15</v>
@@ -1686,10 +1689,10 @@
         <v>9</v>
       </c>
       <c r="B27" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C27" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D27">
         <v>15</v>
@@ -1700,10 +1703,10 @@
         <v>10</v>
       </c>
       <c r="B28" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C28" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D28">
         <v>50</v>
@@ -1714,10 +1717,10 @@
         <v>11</v>
       </c>
       <c r="B29" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C29" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D29">
         <v>15</v>
@@ -1728,10 +1731,10 @@
         <v>12</v>
       </c>
       <c r="B30" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C30" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D30">
         <v>15</v>
@@ -1742,10 +1745,10 @@
         <v>13</v>
       </c>
       <c r="B31" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C31" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D31">
         <v>50</v>
@@ -1756,10 +1759,10 @@
         <v>14</v>
       </c>
       <c r="B32" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C32" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D32">
         <v>20</v>
@@ -1772,7 +1775,7 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B35" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C35" s="10"/>
       <c r="D35" s="10"/>
@@ -1780,19 +1783,19 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B36" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B36" s="7" t="s">
+      <c r="C36" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="C36" s="7" t="s">
+      <c r="D36" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D36" s="2" t="s">
+      <c r="E36" s="2" t="s">
         <v>61</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
@@ -1800,16 +1803,16 @@
         <v>1</v>
       </c>
       <c r="B37" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C37" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D37">
         <v>20</v>
       </c>
       <c r="E37" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
@@ -1817,16 +1820,16 @@
         <v>2</v>
       </c>
       <c r="B38" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C38" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D38">
         <v>20</v>
       </c>
       <c r="E38" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
@@ -1834,10 +1837,10 @@
         <v>3</v>
       </c>
       <c r="B39" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C39" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D39">
         <v>50</v>
@@ -1848,10 +1851,10 @@
         <v>4</v>
       </c>
       <c r="B40" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C40" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D40">
         <v>50</v>
@@ -1862,10 +1865,10 @@
         <v>5</v>
       </c>
       <c r="B41" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C41" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
@@ -1873,10 +1876,10 @@
         <v>6</v>
       </c>
       <c r="B42" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C42" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D42">
         <v>5</v>
@@ -1887,10 +1890,10 @@
         <v>7</v>
       </c>
       <c r="B43" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C43" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D43">
         <v>200</v>
@@ -1901,10 +1904,10 @@
         <v>8</v>
       </c>
       <c r="B44" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C44" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D44">
         <v>100</v>
@@ -1912,7 +1915,7 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B47" s="10" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C47" s="10"/>
       <c r="D47" s="10"/>
@@ -1920,19 +1923,19 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B48" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B48" s="7" t="s">
+      <c r="C48" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="C48" s="7" t="s">
+      <c r="D48" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D48" s="2" t="s">
+      <c r="E48" s="2" t="s">
         <v>61</v>
-      </c>
-      <c r="E48" s="2" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.2">
@@ -1940,16 +1943,16 @@
         <v>1</v>
       </c>
       <c r="B49" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C49" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D49">
         <v>20</v>
       </c>
       <c r="E49" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.2">
@@ -1957,16 +1960,16 @@
         <v>2</v>
       </c>
       <c r="B50" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C50" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D50">
         <v>20</v>
       </c>
       <c r="E50" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.2">
@@ -1974,10 +1977,10 @@
         <v>3</v>
       </c>
       <c r="B51" t="s">
+        <v>128</v>
+      </c>
+      <c r="C51" t="s">
         <v>129</v>
-      </c>
-      <c r="C51" t="s">
-        <v>130</v>
       </c>
       <c r="D51">
         <v>50</v>
@@ -1988,10 +1991,10 @@
         <v>4</v>
       </c>
       <c r="B52" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C52" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.2">
@@ -1999,15 +2002,15 @@
         <v>5</v>
       </c>
       <c r="B53" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C53" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B56" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C56" s="10"/>
       <c r="D56" s="10"/>
@@ -2015,19 +2018,19 @@
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A57" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B57" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B57" s="7" t="s">
+      <c r="C57" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="C57" s="7" t="s">
+      <c r="D57" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D57" s="2" t="s">
+      <c r="E57" s="2" t="s">
         <v>61</v>
-      </c>
-      <c r="E57" s="2" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.2">
@@ -2035,16 +2038,16 @@
         <v>1</v>
       </c>
       <c r="B58" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C58" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D58">
         <v>20</v>
       </c>
       <c r="E58" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.2">
@@ -2052,16 +2055,16 @@
         <v>2</v>
       </c>
       <c r="B59" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C59" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D59">
         <v>20</v>
       </c>
       <c r="E59" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.2">
@@ -2069,10 +2072,10 @@
         <v>3</v>
       </c>
       <c r="B60" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C60" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D60">
         <v>50</v>
@@ -2083,10 +2086,10 @@
         <v>4</v>
       </c>
       <c r="B61" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C61" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D61">
         <v>50</v>
@@ -2097,10 +2100,10 @@
         <v>5</v>
       </c>
       <c r="B62" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C62" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D62">
         <v>200</v>
@@ -2111,10 +2114,10 @@
         <v>6</v>
       </c>
       <c r="B63" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C63" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D63">
         <v>100</v>
@@ -2122,7 +2125,7 @@
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B65" s="10" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C65" s="10"/>
       <c r="D65" s="10"/>
@@ -2130,19 +2133,19 @@
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B66" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B66" s="7" t="s">
+      <c r="C66" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="C66" s="7" t="s">
+      <c r="D66" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D66" s="2" t="s">
+      <c r="E66" s="2" t="s">
         <v>61</v>
-      </c>
-      <c r="E66" s="2" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.2">
@@ -2150,16 +2153,16 @@
         <v>1</v>
       </c>
       <c r="B67" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C67" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D67">
         <v>20</v>
       </c>
       <c r="E67" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.2">
@@ -2167,16 +2170,16 @@
         <v>2</v>
       </c>
       <c r="B68" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C68" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D68">
         <v>50</v>
       </c>
       <c r="E68" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.2">
@@ -2184,10 +2187,10 @@
         <v>3</v>
       </c>
       <c r="B69" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C69" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D69">
         <v>50</v>
@@ -2198,10 +2201,10 @@
         <v>4</v>
       </c>
       <c r="B70" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C70" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D70">
         <v>50</v>
@@ -2212,10 +2215,10 @@
         <v>5</v>
       </c>
       <c r="B71" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C71" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D71">
         <v>200</v>
@@ -2226,10 +2229,10 @@
         <v>6</v>
       </c>
       <c r="B72" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C72" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D72">
         <v>20</v>
@@ -2240,10 +2243,10 @@
         <v>7</v>
       </c>
       <c r="B73" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C73" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.2">
@@ -2251,15 +2254,15 @@
         <v>8</v>
       </c>
       <c r="B74" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C74" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B77" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C77" s="10"/>
       <c r="D77" s="10"/>
@@ -2267,19 +2270,19 @@
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A78" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B78" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B78" s="7" t="s">
+      <c r="C78" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="C78" s="7" t="s">
+      <c r="D78" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D78" s="2" t="s">
+      <c r="E78" s="2" t="s">
         <v>61</v>
-      </c>
-      <c r="E78" s="2" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.2">
@@ -2287,16 +2290,16 @@
         <v>1</v>
       </c>
       <c r="B79" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C79" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D79">
         <v>20</v>
       </c>
       <c r="E79" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.2">
@@ -2304,16 +2307,16 @@
         <v>2</v>
       </c>
       <c r="B80" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C80" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D80">
         <v>20</v>
       </c>
       <c r="E80" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.2">
@@ -2321,16 +2324,16 @@
         <v>3</v>
       </c>
       <c r="B81" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C81" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D81">
         <v>20</v>
       </c>
       <c r="E81" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.2">
@@ -2338,10 +2341,10 @@
         <v>4</v>
       </c>
       <c r="B82" t="s">
+        <v>82</v>
+      </c>
+      <c r="C82" t="s">
         <v>83</v>
-      </c>
-      <c r="C82" t="s">
-        <v>84</v>
       </c>
       <c r="D82">
         <v>15</v>
@@ -2352,10 +2355,10 @@
         <v>5</v>
       </c>
       <c r="B83" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C83" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D83">
         <v>20</v>
@@ -2366,10 +2369,10 @@
         <v>6</v>
       </c>
       <c r="B84" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C84" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D84">
         <v>200</v>
@@ -2380,10 +2383,10 @@
         <v>7</v>
       </c>
       <c r="B85" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C85" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D85">
         <v>20</v>
@@ -2394,10 +2397,10 @@
         <v>8</v>
       </c>
       <c r="B86" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C86" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.2">
@@ -2405,15 +2408,15 @@
         <v>9</v>
       </c>
       <c r="B87" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C87" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B90" s="10" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C90" s="10"/>
       <c r="D90" s="10"/>
@@ -2421,19 +2424,19 @@
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A91" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B91" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B91" s="7" t="s">
+      <c r="C91" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="C91" s="7" t="s">
+      <c r="D91" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D91" s="2" t="s">
+      <c r="E91" s="2" t="s">
         <v>61</v>
-      </c>
-      <c r="E91" s="2" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.2">
@@ -2441,16 +2444,16 @@
         <v>1</v>
       </c>
       <c r="B92" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C92" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D92">
         <v>20</v>
       </c>
       <c r="E92" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.2">
@@ -2458,16 +2461,16 @@
         <v>2</v>
       </c>
       <c r="B93" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C93" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D93">
         <v>20</v>
       </c>
       <c r="E93" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.2">
@@ -2475,16 +2478,16 @@
         <v>3</v>
       </c>
       <c r="B94" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C94" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D94">
         <v>20</v>
       </c>
       <c r="E94" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.2">
@@ -2492,10 +2495,10 @@
         <v>4</v>
       </c>
       <c r="B95" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C95" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D95">
         <v>100</v>
@@ -2506,10 +2509,10 @@
         <v>5</v>
       </c>
       <c r="B96" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C96" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D96">
         <v>500</v>
@@ -2520,10 +2523,10 @@
         <v>6</v>
       </c>
       <c r="B97" t="s">
+        <v>96</v>
+      </c>
+      <c r="C97" t="s">
         <v>97</v>
-      </c>
-      <c r="C97" t="s">
-        <v>98</v>
       </c>
       <c r="D97">
         <v>1000</v>
@@ -2534,10 +2537,10 @@
         <v>7</v>
       </c>
       <c r="B98" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C98" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D98">
         <v>1000</v>
@@ -2548,10 +2551,10 @@
         <v>8</v>
       </c>
       <c r="B99" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C99" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.2">
@@ -2559,15 +2562,15 @@
         <v>9</v>
       </c>
       <c r="B100" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C100" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B103" s="10" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C103" s="10"/>
       <c r="D103" s="10"/>
@@ -2575,19 +2578,19 @@
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A104" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B104" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B104" s="7" t="s">
+      <c r="C104" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="C104" s="7" t="s">
+      <c r="D104" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D104" s="2" t="s">
+      <c r="E104" s="2" t="s">
         <v>61</v>
-      </c>
-      <c r="E104" s="2" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.2">
@@ -2595,16 +2598,16 @@
         <v>1</v>
       </c>
       <c r="B105" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C105" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D105">
         <v>20</v>
       </c>
       <c r="E105" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.2">
@@ -2612,16 +2615,16 @@
         <v>2</v>
       </c>
       <c r="B106" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C106" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D106">
         <v>20</v>
       </c>
       <c r="E106" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.2">
@@ -2629,16 +2632,16 @@
         <v>3</v>
       </c>
       <c r="B107" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C107" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D107">
         <v>20</v>
       </c>
       <c r="E107" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.2">
@@ -2646,7 +2649,7 @@
         <v>4</v>
       </c>
       <c r="B108" s="13" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C108" s="14"/>
     </row>
@@ -2671,10 +2674,10 @@
         <v>5</v>
       </c>
       <c r="B113" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C113" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D113">
         <v>500</v>
@@ -2685,10 +2688,10 @@
         <v>6</v>
       </c>
       <c r="B114" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C114" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D114">
         <v>1000</v>
@@ -2696,7 +2699,7 @@
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B117" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C117" s="10"/>
       <c r="D117" s="10"/>
@@ -2704,19 +2707,19 @@
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A118" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B118" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B118" s="7" t="s">
+      <c r="C118" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="C118" s="7" t="s">
+      <c r="D118" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D118" s="2" t="s">
+      <c r="E118" s="2" t="s">
         <v>61</v>
-      </c>
-      <c r="E118" s="2" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.2">
@@ -2724,16 +2727,16 @@
         <v>1</v>
       </c>
       <c r="B119" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C119" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D119">
         <v>20</v>
       </c>
       <c r="E119" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.2">
@@ -2741,16 +2744,16 @@
         <v>2</v>
       </c>
       <c r="B120" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C120" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D120">
         <v>20</v>
       </c>
       <c r="E120" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.2">
@@ -2758,10 +2761,10 @@
         <v>3</v>
       </c>
       <c r="B121" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C121" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D121">
         <v>50</v>
@@ -2772,10 +2775,10 @@
         <v>4</v>
       </c>
       <c r="B122" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C122" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D122">
         <v>3</v>
@@ -2786,10 +2789,10 @@
         <v>5</v>
       </c>
       <c r="B123" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C123" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.2">
@@ -2797,7 +2800,7 @@
         <v>6</v>
       </c>
       <c r="B124" s="13" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C124" s="14"/>
     </row>
@@ -2811,7 +2814,7 @@
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B129" s="10" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C129" s="10"/>
       <c r="D129" s="10"/>
@@ -2819,19 +2822,19 @@
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A130" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B130" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B130" s="7" t="s">
+      <c r="C130" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="C130" s="7" t="s">
+      <c r="D130" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D130" s="2" t="s">
+      <c r="E130" s="2" t="s">
         <v>61</v>
-      </c>
-      <c r="E130" s="2" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.2">
@@ -2839,16 +2842,16 @@
         <v>1</v>
       </c>
       <c r="B131" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C131" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D131">
         <v>20</v>
       </c>
       <c r="E131" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.2">
@@ -2856,16 +2859,16 @@
         <v>2</v>
       </c>
       <c r="B132" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C132" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D132">
         <v>20</v>
       </c>
       <c r="E132" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>
@@ -2890,7 +2893,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD54E32F-1636-154F-88FF-57ECFAEA7F4B}">
-  <dimension ref="A3:X42"/>
+  <dimension ref="A3:X43"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="38.1640625" bestFit="1" customWidth="1"/>
@@ -2898,7 +2901,7 @@
   <sheetData>
     <row r="3" spans="1:24" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B3" s="8"/>
       <c r="C3" s="8"/>
@@ -2911,7 +2914,7 @@
       <c r="J3" s="8"/>
       <c r="K3" s="8"/>
       <c r="M3" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="N3" s="9"/>
       <c r="O3" s="9"/>
@@ -3608,7 +3611,7 @@
     </row>
     <row r="33" spans="1:24" ht="24" x14ac:dyDescent="0.3">
       <c r="A33" s="18" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B33" s="18"/>
       <c r="C33" s="18"/>
@@ -3634,7 +3637,7 @@
         <v>1</v>
       </c>
       <c r="B34" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="M34" s="9"/>
       <c r="N34" s="9"/>
@@ -3654,7 +3657,7 @@
         <v>2</v>
       </c>
       <c r="B35" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="M35" s="9"/>
       <c r="N35" s="9"/>
@@ -3674,7 +3677,7 @@
         <v>3</v>
       </c>
       <c r="B36" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="M36" s="9"/>
       <c r="N36" s="9"/>
@@ -3694,7 +3697,7 @@
         <v>4</v>
       </c>
       <c r="B37" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="M37" s="9"/>
       <c r="N37" s="9"/>
@@ -3714,7 +3717,7 @@
         <v>5</v>
       </c>
       <c r="B38" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="M38" s="9"/>
       <c r="N38" s="9"/>
@@ -3734,7 +3737,7 @@
         <v>6</v>
       </c>
       <c r="B39" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C39" s="16"/>
       <c r="D39" s="16"/>
@@ -3757,7 +3760,7 @@
         <v>7</v>
       </c>
       <c r="B40" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="M40" s="9"/>
       <c r="N40" s="9"/>
@@ -3777,7 +3780,7 @@
         <v>8</v>
       </c>
       <c r="B41" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="M41" s="9"/>
       <c r="N41" s="9"/>
@@ -3797,7 +3800,15 @@
         <v>9</v>
       </c>
       <c r="B42" t="s">
-        <v>123</v>
+        <v>122</v>
+      </c>
+    </row>
+    <row r="43" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A43">
+        <v>10</v>
+      </c>
+      <c r="B43" t="s">
+        <v>147</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add treatment plan page functionality for doctor role
</commit_message>
<xml_diff>
--- a/CareOS-Hospital_ERP_System.xlsx
+++ b/CareOS-Hospital_ERP_System.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hetlimbani/Desktop/Self_Learning/CareOS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{833C039B-B0B0-EF40-93A0-D24CA074E828}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE8FD07A-0966-B649-93B4-486B25F446A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19420" activeTab="2" xr2:uid="{3BCF7A51-5C29-EE4C-8BC3-93CAF12DE1EA}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19420" xr2:uid="{3BCF7A51-5C29-EE4C-8BC3-93CAF12DE1EA}"/>
   </bookViews>
   <sheets>
     <sheet name="ERP System" sheetId="1" r:id="rId1"/>
@@ -1117,7 +1117,7 @@
       <c r="F4" t="s">
         <v>13</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" s="15" t="s">
         <v>13</v>
       </c>
       <c r="H4" t="s">
@@ -1229,7 +1229,7 @@
       <c r="B9" t="s">
         <v>50</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="15" t="s">
         <v>17</v>
       </c>
       <c r="F9" s="15" t="s">
@@ -1243,7 +1243,7 @@
       <c r="B10" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="15" t="s">
         <v>21</v>
       </c>
       <c r="F10" s="15" t="s">
@@ -3759,9 +3759,10 @@
       <c r="A40">
         <v>7</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B40" s="15" t="s">
         <v>119</v>
       </c>
+      <c r="C40" s="16"/>
       <c r="M40" s="9"/>
       <c r="N40" s="9"/>
       <c r="O40" s="9"/>

</xml_diff>

<commit_message>
Add treatment plans code in doctor and nurse role
</commit_message>
<xml_diff>
--- a/CareOS-Hospital_ERP_System.xlsx
+++ b/CareOS-Hospital_ERP_System.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hetlimbani/Desktop/Self_Learning/CareOS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE8FD07A-0966-B649-93B4-486B25F446A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D11A3F93-F5F8-BF44-8E0F-F59B412B0A37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19420" xr2:uid="{3BCF7A51-5C29-EE4C-8BC3-93CAF12DE1EA}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="147">
   <si>
     <t>Total Roles</t>
   </si>
@@ -116,9 +116,6 @@
   </si>
   <si>
     <t>Shift Management</t>
-  </si>
-  <si>
-    <t>Assigned Tasks</t>
   </si>
   <si>
     <t>Reminder</t>
@@ -1045,7 +1042,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C1" s="12" t="s">
         <v>1</v>
@@ -1077,28 +1074,28 @@
         <v>8</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
@@ -1121,10 +1118,10 @@
         <v>13</v>
       </c>
       <c r="H4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="I4" s="19" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
@@ -1134,23 +1131,23 @@
       <c r="C5" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="15" t="s">
         <v>23</v>
       </c>
       <c r="E5" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="F5" s="15" t="s">
-        <v>29</v>
-      </c>
       <c r="G5" s="15" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I5" s="19" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
@@ -1161,82 +1158,79 @@
         <v>16</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F6" s="15" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G6" s="15" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I6" s="19" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B7" s="15" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C7" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="D7" t="s">
-        <v>25</v>
+      <c r="D7" s="15" t="s">
+        <v>144</v>
       </c>
       <c r="E7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G7" s="15" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I7" s="19" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B8" s="15" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C8" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="15" t="s">
-        <v>145</v>
-      </c>
       <c r="E8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F8" s="15" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C9" s="15" t="s">
         <v>17</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
@@ -1247,7 +1241,7 @@
         <v>21</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
@@ -1260,28 +1254,28 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B14" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
@@ -1292,7 +1286,7 @@
         <v>14</v>
       </c>
       <c r="D15" s="20" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E15" t="s">
         <v>14</v>
@@ -1352,7 +1346,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B1" s="10" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C1" s="10"/>
       <c r="D1" s="10"/>
@@ -1360,19 +1354,19 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B2" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="C2" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="D2" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>60</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>61</v>
       </c>
       <c r="F2" s="5"/>
     </row>
@@ -1381,16 +1375,16 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D3">
         <v>20</v>
       </c>
       <c r="E3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -1398,10 +1392,10 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D4">
         <v>50</v>
@@ -1412,10 +1406,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D5">
         <v>50</v>
@@ -1426,16 +1420,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D6">
         <v>100</v>
       </c>
       <c r="E6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -1443,10 +1437,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D7">
         <v>100</v>
@@ -1457,10 +1451,10 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D8">
         <v>15</v>
@@ -1471,10 +1465,10 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D9">
         <v>5</v>
@@ -1485,10 +1479,10 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D10">
         <v>15</v>
@@ -1499,10 +1493,10 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C11" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D11">
         <v>100</v>
@@ -1513,10 +1507,10 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C12" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D12">
         <v>1</v>
@@ -1527,10 +1521,10 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -1538,15 +1532,15 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B17" s="10" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C17" s="10"/>
       <c r="D17" s="10"/>
@@ -1554,19 +1548,19 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B18" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="C18" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="D18" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="E18" s="2" t="s">
         <v>60</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
@@ -1574,16 +1568,16 @@
         <v>1</v>
       </c>
       <c r="B19" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C19" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D19">
         <v>20</v>
       </c>
       <c r="E19" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
@@ -1591,16 +1585,16 @@
         <v>2</v>
       </c>
       <c r="B20" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C20" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D20">
         <v>20</v>
       </c>
       <c r="E20" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
@@ -1608,10 +1602,10 @@
         <v>3</v>
       </c>
       <c r="B21" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C21" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
@@ -1619,10 +1613,10 @@
         <v>4</v>
       </c>
       <c r="B22" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D22">
         <v>10</v>
@@ -1633,10 +1627,10 @@
         <v>5</v>
       </c>
       <c r="B23" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C23" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D23">
         <v>5</v>
@@ -1647,10 +1641,10 @@
         <v>6</v>
       </c>
       <c r="B24" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C24" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D24">
         <v>200</v>
@@ -1661,10 +1655,10 @@
         <v>7</v>
       </c>
       <c r="B25" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C25" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D25">
         <v>50</v>
@@ -1675,10 +1669,10 @@
         <v>8</v>
       </c>
       <c r="B26" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C26" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D26">
         <v>15</v>
@@ -1689,10 +1683,10 @@
         <v>9</v>
       </c>
       <c r="B27" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C27" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D27">
         <v>15</v>
@@ -1703,10 +1697,10 @@
         <v>10</v>
       </c>
       <c r="B28" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C28" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D28">
         <v>50</v>
@@ -1717,10 +1711,10 @@
         <v>11</v>
       </c>
       <c r="B29" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C29" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D29">
         <v>15</v>
@@ -1731,10 +1725,10 @@
         <v>12</v>
       </c>
       <c r="B30" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C30" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D30">
         <v>15</v>
@@ -1745,10 +1739,10 @@
         <v>13</v>
       </c>
       <c r="B31" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C31" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D31">
         <v>50</v>
@@ -1759,10 +1753,10 @@
         <v>14</v>
       </c>
       <c r="B32" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C32" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D32">
         <v>20</v>
@@ -1775,7 +1769,7 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B35" s="10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C35" s="10"/>
       <c r="D35" s="10"/>
@@ -1783,19 +1777,19 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B36" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="B36" s="7" t="s">
+      <c r="C36" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="C36" s="7" t="s">
+      <c r="D36" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D36" s="2" t="s">
+      <c r="E36" s="2" t="s">
         <v>60</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
@@ -1803,16 +1797,16 @@
         <v>1</v>
       </c>
       <c r="B37" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C37" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D37">
         <v>20</v>
       </c>
       <c r="E37" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
@@ -1820,16 +1814,16 @@
         <v>2</v>
       </c>
       <c r="B38" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C38" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D38">
         <v>20</v>
       </c>
       <c r="E38" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
@@ -1837,10 +1831,10 @@
         <v>3</v>
       </c>
       <c r="B39" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C39" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D39">
         <v>50</v>
@@ -1851,10 +1845,10 @@
         <v>4</v>
       </c>
       <c r="B40" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C40" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D40">
         <v>50</v>
@@ -1865,10 +1859,10 @@
         <v>5</v>
       </c>
       <c r="B41" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C41" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
@@ -1876,10 +1870,10 @@
         <v>6</v>
       </c>
       <c r="B42" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C42" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D42">
         <v>5</v>
@@ -1890,10 +1884,10 @@
         <v>7</v>
       </c>
       <c r="B43" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C43" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D43">
         <v>200</v>
@@ -1904,10 +1898,10 @@
         <v>8</v>
       </c>
       <c r="B44" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C44" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D44">
         <v>100</v>
@@ -1915,7 +1909,7 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B47" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C47" s="10"/>
       <c r="D47" s="10"/>
@@ -1923,19 +1917,19 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B48" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="B48" s="7" t="s">
+      <c r="C48" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="C48" s="7" t="s">
+      <c r="D48" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D48" s="2" t="s">
+      <c r="E48" s="2" t="s">
         <v>60</v>
-      </c>
-      <c r="E48" s="2" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.2">
@@ -1943,16 +1937,16 @@
         <v>1</v>
       </c>
       <c r="B49" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C49" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D49">
         <v>20</v>
       </c>
       <c r="E49" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.2">
@@ -1960,16 +1954,16 @@
         <v>2</v>
       </c>
       <c r="B50" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C50" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D50">
         <v>20</v>
       </c>
       <c r="E50" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.2">
@@ -1977,10 +1971,10 @@
         <v>3</v>
       </c>
       <c r="B51" t="s">
+        <v>127</v>
+      </c>
+      <c r="C51" t="s">
         <v>128</v>
-      </c>
-      <c r="C51" t="s">
-        <v>129</v>
       </c>
       <c r="D51">
         <v>50</v>
@@ -1991,10 +1985,10 @@
         <v>4</v>
       </c>
       <c r="B52" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C52" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.2">
@@ -2002,15 +1996,15 @@
         <v>5</v>
       </c>
       <c r="B53" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C53" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B56" s="10" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C56" s="10"/>
       <c r="D56" s="10"/>
@@ -2018,19 +2012,19 @@
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A57" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B57" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="B57" s="7" t="s">
+      <c r="C57" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="C57" s="7" t="s">
+      <c r="D57" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D57" s="2" t="s">
+      <c r="E57" s="2" t="s">
         <v>60</v>
-      </c>
-      <c r="E57" s="2" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.2">
@@ -2038,16 +2032,16 @@
         <v>1</v>
       </c>
       <c r="B58" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C58" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D58">
         <v>20</v>
       </c>
       <c r="E58" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.2">
@@ -2055,16 +2049,16 @@
         <v>2</v>
       </c>
       <c r="B59" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C59" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D59">
         <v>20</v>
       </c>
       <c r="E59" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.2">
@@ -2072,10 +2066,10 @@
         <v>3</v>
       </c>
       <c r="B60" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C60" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D60">
         <v>50</v>
@@ -2086,10 +2080,10 @@
         <v>4</v>
       </c>
       <c r="B61" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C61" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D61">
         <v>50</v>
@@ -2100,10 +2094,10 @@
         <v>5</v>
       </c>
       <c r="B62" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C62" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D62">
         <v>200</v>
@@ -2114,10 +2108,10 @@
         <v>6</v>
       </c>
       <c r="B63" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C63" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D63">
         <v>100</v>
@@ -2125,7 +2119,7 @@
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B65" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C65" s="10"/>
       <c r="D65" s="10"/>
@@ -2133,19 +2127,19 @@
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B66" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="B66" s="7" t="s">
+      <c r="C66" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="C66" s="7" t="s">
+      <c r="D66" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D66" s="2" t="s">
+      <c r="E66" s="2" t="s">
         <v>60</v>
-      </c>
-      <c r="E66" s="2" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.2">
@@ -2153,16 +2147,16 @@
         <v>1</v>
       </c>
       <c r="B67" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C67" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D67">
         <v>20</v>
       </c>
       <c r="E67" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.2">
@@ -2170,16 +2164,16 @@
         <v>2</v>
       </c>
       <c r="B68" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C68" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D68">
         <v>50</v>
       </c>
       <c r="E68" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.2">
@@ -2187,10 +2181,10 @@
         <v>3</v>
       </c>
       <c r="B69" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C69" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D69">
         <v>50</v>
@@ -2201,10 +2195,10 @@
         <v>4</v>
       </c>
       <c r="B70" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C70" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D70">
         <v>50</v>
@@ -2215,10 +2209,10 @@
         <v>5</v>
       </c>
       <c r="B71" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C71" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D71">
         <v>200</v>
@@ -2229,10 +2223,10 @@
         <v>6</v>
       </c>
       <c r="B72" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C72" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D72">
         <v>20</v>
@@ -2243,10 +2237,10 @@
         <v>7</v>
       </c>
       <c r="B73" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C73" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.2">
@@ -2254,15 +2248,15 @@
         <v>8</v>
       </c>
       <c r="B74" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C74" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B77" s="10" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C77" s="10"/>
       <c r="D77" s="10"/>
@@ -2270,19 +2264,19 @@
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A78" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B78" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="B78" s="7" t="s">
+      <c r="C78" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="C78" s="7" t="s">
+      <c r="D78" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D78" s="2" t="s">
+      <c r="E78" s="2" t="s">
         <v>60</v>
-      </c>
-      <c r="E78" s="2" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.2">
@@ -2290,16 +2284,16 @@
         <v>1</v>
       </c>
       <c r="B79" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C79" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D79">
         <v>20</v>
       </c>
       <c r="E79" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.2">
@@ -2307,16 +2301,16 @@
         <v>2</v>
       </c>
       <c r="B80" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C80" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D80">
         <v>20</v>
       </c>
       <c r="E80" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.2">
@@ -2324,16 +2318,16 @@
         <v>3</v>
       </c>
       <c r="B81" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C81" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D81">
         <v>20</v>
       </c>
       <c r="E81" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.2">
@@ -2341,10 +2335,10 @@
         <v>4</v>
       </c>
       <c r="B82" t="s">
+        <v>81</v>
+      </c>
+      <c r="C82" t="s">
         <v>82</v>
-      </c>
-      <c r="C82" t="s">
-        <v>83</v>
       </c>
       <c r="D82">
         <v>15</v>
@@ -2355,10 +2349,10 @@
         <v>5</v>
       </c>
       <c r="B83" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C83" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D83">
         <v>20</v>
@@ -2369,10 +2363,10 @@
         <v>6</v>
       </c>
       <c r="B84" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C84" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D84">
         <v>200</v>
@@ -2383,10 +2377,10 @@
         <v>7</v>
       </c>
       <c r="B85" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C85" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D85">
         <v>20</v>
@@ -2397,10 +2391,10 @@
         <v>8</v>
       </c>
       <c r="B86" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C86" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.2">
@@ -2408,15 +2402,15 @@
         <v>9</v>
       </c>
       <c r="B87" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C87" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B90" s="10" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C90" s="10"/>
       <c r="D90" s="10"/>
@@ -2424,19 +2418,19 @@
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A91" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B91" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="B91" s="7" t="s">
+      <c r="C91" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="C91" s="7" t="s">
+      <c r="D91" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D91" s="2" t="s">
+      <c r="E91" s="2" t="s">
         <v>60</v>
-      </c>
-      <c r="E91" s="2" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.2">
@@ -2444,16 +2438,16 @@
         <v>1</v>
       </c>
       <c r="B92" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C92" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D92">
         <v>20</v>
       </c>
       <c r="E92" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.2">
@@ -2461,16 +2455,16 @@
         <v>2</v>
       </c>
       <c r="B93" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C93" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D93">
         <v>20</v>
       </c>
       <c r="E93" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.2">
@@ -2478,16 +2472,16 @@
         <v>3</v>
       </c>
       <c r="B94" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C94" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D94">
         <v>20</v>
       </c>
       <c r="E94" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.2">
@@ -2495,10 +2489,10 @@
         <v>4</v>
       </c>
       <c r="B95" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C95" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D95">
         <v>100</v>
@@ -2509,10 +2503,10 @@
         <v>5</v>
       </c>
       <c r="B96" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C96" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D96">
         <v>500</v>
@@ -2523,10 +2517,10 @@
         <v>6</v>
       </c>
       <c r="B97" t="s">
+        <v>95</v>
+      </c>
+      <c r="C97" t="s">
         <v>96</v>
-      </c>
-      <c r="C97" t="s">
-        <v>97</v>
       </c>
       <c r="D97">
         <v>1000</v>
@@ -2537,10 +2531,10 @@
         <v>7</v>
       </c>
       <c r="B98" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C98" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D98">
         <v>1000</v>
@@ -2551,10 +2545,10 @@
         <v>8</v>
       </c>
       <c r="B99" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C99" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.2">
@@ -2562,15 +2556,15 @@
         <v>9</v>
       </c>
       <c r="B100" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C100" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B103" s="10" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C103" s="10"/>
       <c r="D103" s="10"/>
@@ -2578,19 +2572,19 @@
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A104" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B104" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="B104" s="7" t="s">
+      <c r="C104" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="C104" s="7" t="s">
+      <c r="D104" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D104" s="2" t="s">
+      <c r="E104" s="2" t="s">
         <v>60</v>
-      </c>
-      <c r="E104" s="2" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.2">
@@ -2598,16 +2592,16 @@
         <v>1</v>
       </c>
       <c r="B105" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C105" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D105">
         <v>20</v>
       </c>
       <c r="E105" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.2">
@@ -2615,16 +2609,16 @@
         <v>2</v>
       </c>
       <c r="B106" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C106" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D106">
         <v>20</v>
       </c>
       <c r="E106" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.2">
@@ -2632,16 +2626,16 @@
         <v>3</v>
       </c>
       <c r="B107" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C107" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D107">
         <v>20</v>
       </c>
       <c r="E107" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.2">
@@ -2649,7 +2643,7 @@
         <v>4</v>
       </c>
       <c r="B108" s="13" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C108" s="14"/>
     </row>
@@ -2674,10 +2668,10 @@
         <v>5</v>
       </c>
       <c r="B113" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C113" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D113">
         <v>500</v>
@@ -2688,10 +2682,10 @@
         <v>6</v>
       </c>
       <c r="B114" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C114" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D114">
         <v>1000</v>
@@ -2699,7 +2693,7 @@
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B117" s="10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C117" s="10"/>
       <c r="D117" s="10"/>
@@ -2707,19 +2701,19 @@
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A118" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B118" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="B118" s="7" t="s">
+      <c r="C118" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="C118" s="7" t="s">
+      <c r="D118" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D118" s="2" t="s">
+      <c r="E118" s="2" t="s">
         <v>60</v>
-      </c>
-      <c r="E118" s="2" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.2">
@@ -2727,16 +2721,16 @@
         <v>1</v>
       </c>
       <c r="B119" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C119" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D119">
         <v>20</v>
       </c>
       <c r="E119" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.2">
@@ -2744,16 +2738,16 @@
         <v>2</v>
       </c>
       <c r="B120" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C120" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D120">
         <v>20</v>
       </c>
       <c r="E120" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.2">
@@ -2761,10 +2755,10 @@
         <v>3</v>
       </c>
       <c r="B121" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C121" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D121">
         <v>50</v>
@@ -2775,10 +2769,10 @@
         <v>4</v>
       </c>
       <c r="B122" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C122" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D122">
         <v>3</v>
@@ -2789,10 +2783,10 @@
         <v>5</v>
       </c>
       <c r="B123" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C123" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.2">
@@ -2800,7 +2794,7 @@
         <v>6</v>
       </c>
       <c r="B124" s="13" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C124" s="14"/>
     </row>
@@ -2814,7 +2808,7 @@
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B129" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C129" s="10"/>
       <c r="D129" s="10"/>
@@ -2822,19 +2816,19 @@
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A130" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B130" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="B130" s="7" t="s">
+      <c r="C130" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="C130" s="7" t="s">
+      <c r="D130" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D130" s="2" t="s">
+      <c r="E130" s="2" t="s">
         <v>60</v>
-      </c>
-      <c r="E130" s="2" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.2">
@@ -2842,16 +2836,16 @@
         <v>1</v>
       </c>
       <c r="B131" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C131" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D131">
         <v>20</v>
       </c>
       <c r="E131" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.2">
@@ -2859,16 +2853,16 @@
         <v>2</v>
       </c>
       <c r="B132" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C132" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D132">
         <v>20</v>
       </c>
       <c r="E132" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -2901,7 +2895,7 @@
   <sheetData>
     <row r="3" spans="1:24" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B3" s="8"/>
       <c r="C3" s="8"/>
@@ -2914,7 +2908,7 @@
       <c r="J3" s="8"/>
       <c r="K3" s="8"/>
       <c r="M3" s="9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="N3" s="9"/>
       <c r="O3" s="9"/>
@@ -3611,7 +3605,7 @@
     </row>
     <row r="33" spans="1:24" ht="24" x14ac:dyDescent="0.3">
       <c r="A33" s="18" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B33" s="18"/>
       <c r="C33" s="18"/>
@@ -3637,7 +3631,7 @@
         <v>1</v>
       </c>
       <c r="B34" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="M34" s="9"/>
       <c r="N34" s="9"/>
@@ -3657,7 +3651,7 @@
         <v>2</v>
       </c>
       <c r="B35" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="M35" s="9"/>
       <c r="N35" s="9"/>
@@ -3677,7 +3671,7 @@
         <v>3</v>
       </c>
       <c r="B36" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="M36" s="9"/>
       <c r="N36" s="9"/>
@@ -3697,7 +3691,7 @@
         <v>4</v>
       </c>
       <c r="B37" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="M37" s="9"/>
       <c r="N37" s="9"/>
@@ -3717,7 +3711,7 @@
         <v>5</v>
       </c>
       <c r="B38" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="M38" s="9"/>
       <c r="N38" s="9"/>
@@ -3737,7 +3731,7 @@
         <v>6</v>
       </c>
       <c r="B39" s="15" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C39" s="16"/>
       <c r="D39" s="16"/>
@@ -3760,7 +3754,7 @@
         <v>7</v>
       </c>
       <c r="B40" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C40" s="16"/>
       <c r="M40" s="9"/>
@@ -3781,7 +3775,7 @@
         <v>8</v>
       </c>
       <c r="B41" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="M41" s="9"/>
       <c r="N41" s="9"/>
@@ -3801,7 +3795,7 @@
         <v>9</v>
       </c>
       <c r="B42" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="43" spans="1:24" x14ac:dyDescent="0.2">
@@ -3809,7 +3803,7 @@
         <v>10</v>
       </c>
       <c r="B43" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add lab technician dashboard
</commit_message>
<xml_diff>
--- a/CareOS-Hospital_ERP_System.xlsx
+++ b/CareOS-Hospital_ERP_System.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hetlimbani/Desktop/Self_Learning/CareOS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D11A3F93-F5F8-BF44-8E0F-F59B412B0A37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{522D67A7-B086-334E-8635-ED4BB63490AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19420" xr2:uid="{3BCF7A51-5C29-EE4C-8BC3-93CAF12DE1EA}"/>
   </bookViews>
@@ -1111,7 +1111,7 @@
       <c r="E4" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="15" t="s">
         <v>13</v>
       </c>
       <c r="G4" s="15" t="s">
@@ -3630,7 +3630,7 @@
       <c r="A34">
         <v>1</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B34" s="15" t="s">
         <v>111</v>
       </c>
       <c r="M34" s="9"/>
@@ -3650,7 +3650,7 @@
       <c r="A35">
         <v>2</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B35" s="15" t="s">
         <v>112</v>
       </c>
       <c r="M35" s="9"/>

</xml_diff>

<commit_message>
Add billing in recpetionist role
</commit_message>
<xml_diff>
--- a/CareOS-Hospital_ERP_System.xlsx
+++ b/CareOS-Hospital_ERP_System.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hetlimbani/Desktop/Self_Learning/CareOS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{522D67A7-B086-334E-8635-ED4BB63490AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C55DCE11-66E0-A84D-95F4-52ADF83FD973}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19420" xr2:uid="{3BCF7A51-5C29-EE4C-8BC3-93CAF12DE1EA}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19420" activeTab="1" xr2:uid="{3BCF7A51-5C29-EE4C-8BC3-93CAF12DE1EA}"/>
   </bookViews>
   <sheets>
     <sheet name="ERP System" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="173">
   <si>
     <t>Total Roles</t>
   </si>
@@ -295,32 +295,10 @@
     <t>diagnosis</t>
   </si>
   <si>
-    <t>prescription</t>
-  </si>
-  <si>
     <t>notes</t>
   </si>
   <si>
     <t>update_at</t>
-  </si>
-  <si>
-    <t>medicines:[{
-            medicine:String, dosage:String,
-            days:Number }  ]</t>
-  </si>
-  <si>
-    <t>test_name</t>
-  </si>
-  <si>
-    <t>sample_collected</t>
-  </si>
-  <si>
-    <t>report</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> reportStatus:{
-        type:String,
-        default:"pending"  }</t>
   </si>
   <si>
     <t>12. Ambulance Schema
@@ -373,30 +351,15 @@
 export default mongoose.model("EmergencyRequest",EmergencyRequestSchema);</t>
   </si>
   <si>
-    <t>Medical History Table Schema</t>
-  </si>
-  <si>
     <t>result</t>
   </si>
   <si>
-    <t>text</t>
-  </si>
-  <si>
-    <t>Prescription Table Schema</t>
-  </si>
-  <si>
     <t>birth_date</t>
   </si>
   <si>
     <t>experince_startdate</t>
   </si>
   <si>
-    <t>Laboratory Table Schema</t>
-  </si>
-  <si>
-    <t>Billing Table Schema</t>
-  </si>
-  <si>
     <t>emergency_contact_name1</t>
   </si>
   <si>
@@ -530,6 +493,117 @@
   </si>
   <si>
     <t>Edit lab report functionality after adding new  lab report by nurse or doctor in lab technician role</t>
+  </si>
+  <si>
+    <t>Prescription  Collection Schema</t>
+  </si>
+  <si>
+    <t>appoitnemnt_id</t>
+  </si>
+  <si>
+    <t>patientEmail</t>
+  </si>
+  <si>
+    <t>doctorEmail</t>
+  </si>
+  <si>
+    <t>doctorName</t>
+  </si>
+  <si>
+    <t>prescriptionName</t>
+  </si>
+  <si>
+    <t>medicines</t>
+  </si>
+  <si>
+    <t>labReports</t>
+  </si>
+  <si>
+    <t>Medicines Collection Schema</t>
+  </si>
+  <si>
+    <t>barcode</t>
+  </si>
+  <si>
+    <t>medicine_name</t>
+  </si>
+  <si>
+    <t>company</t>
+  </si>
+  <si>
+    <t>category</t>
+  </si>
+  <si>
+    <t>composition</t>
+  </si>
+  <si>
+    <t>price</t>
+  </si>
+  <si>
+    <t>quantity</t>
+  </si>
+  <si>
+    <t>manufacture_date</t>
+  </si>
+  <si>
+    <t>expiry_date</t>
+  </si>
+  <si>
+    <t>medicine_usecase</t>
+  </si>
+  <si>
+    <t>Lab Reports Collection Schema</t>
+  </si>
+  <si>
+    <t>report_code</t>
+  </si>
+  <si>
+    <t>report_name</t>
+  </si>
+  <si>
+    <t>sample_type</t>
+  </si>
+  <si>
+    <t>tat_hours</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>Medicine Histories Collection Schema</t>
+  </si>
+  <si>
+    <t>prescriptionId</t>
+  </si>
+  <si>
+    <t>appointmentId</t>
+  </si>
+  <si>
+    <t>dispensedMedicines</t>
+  </si>
+  <si>
+    <t>isPaymentCompleted</t>
+  </si>
+  <si>
+    <t>patientId</t>
+  </si>
+  <si>
+    <t>pharmacistEmail</t>
+  </si>
+  <si>
+    <t>skippedMedicines</t>
+  </si>
+  <si>
+    <t>createdAt</t>
+  </si>
+  <si>
+    <t>updatedAt</t>
+  </si>
+  <si>
+    <t>dispensedAt</t>
+  </si>
+  <si>
+    <t>boolean</t>
   </si>
 </sst>
 </file>
@@ -643,7 +717,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -659,6 +733,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -669,22 +746,28 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1038,36 +1121,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="G1" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="12" t="s">
+      <c r="H1" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="12" t="s">
+      <c r="I1" s="13" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="I2" s="11"/>
+      <c r="I2" s="12"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
@@ -1099,28 +1182,28 @@
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="14" t="s">
         <v>9</v>
       </c>
       <c r="C4" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="21" t="s">
+      <c r="E4" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="F4" s="15" t="s">
+      <c r="F4" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="15" t="s">
+      <c r="G4" s="14" t="s">
         <v>13</v>
       </c>
       <c r="H4" t="s">
         <v>36</v>
       </c>
-      <c r="I4" s="19" t="s">
+      <c r="I4" s="20" t="s">
         <v>42</v>
       </c>
     </row>
@@ -1128,91 +1211,91 @@
       <c r="B5" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="15" t="s">
+      <c r="C5" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="15" t="s">
+      <c r="D5" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="E5" s="15" t="s">
+      <c r="E5" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="F5" s="15" t="s">
+      <c r="F5" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="G5" s="15" t="s">
+      <c r="G5" s="14" t="s">
         <v>33</v>
       </c>
       <c r="H5" t="s">
         <v>37</v>
       </c>
-      <c r="I5" s="19" t="s">
+      <c r="I5" s="20" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B6" s="15" t="s">
+      <c r="B6" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="15" t="s">
+      <c r="C6" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="15" t="s">
-        <v>145</v>
-      </c>
-      <c r="E6" s="15" t="s">
-        <v>120</v>
-      </c>
-      <c r="F6" s="15" t="s">
+      <c r="D6" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="E6" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="F6" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="G6" s="15" t="s">
+      <c r="G6" s="14" t="s">
         <v>34</v>
       </c>
       <c r="H6" t="s">
         <v>38</v>
       </c>
-      <c r="I6" s="19" t="s">
+      <c r="I6" s="20" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B7" s="15" t="s">
-        <v>114</v>
-      </c>
-      <c r="C7" s="15" t="s">
+      <c r="B7" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="C7" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="15" t="s">
-        <v>144</v>
+      <c r="D7" s="14" t="s">
+        <v>133</v>
       </c>
       <c r="E7" t="s">
         <v>26</v>
       </c>
-      <c r="F7" s="15" t="s">
+      <c r="F7" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="G7" s="15" t="s">
+      <c r="G7" s="14" t="s">
         <v>35</v>
       </c>
       <c r="H7" t="s">
         <v>39</v>
       </c>
-      <c r="I7" s="19" t="s">
+      <c r="I7" s="20" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B8" s="15" t="s">
+      <c r="B8" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="C8" s="15" t="s">
+      <c r="C8" s="14" t="s">
         <v>19</v>
       </c>
       <c r="E8" t="s">
         <v>49</v>
       </c>
-      <c r="F8" s="15" t="s">
+      <c r="F8" s="14" t="s">
         <v>31</v>
       </c>
       <c r="H8" t="s">
@@ -1223,10 +1306,10 @@
       <c r="B9" t="s">
         <v>49</v>
       </c>
-      <c r="C9" s="15" t="s">
+      <c r="C9" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="15" t="s">
+      <c r="F9" s="14" t="s">
         <v>32</v>
       </c>
       <c r="H9" t="s">
@@ -1234,23 +1317,23 @@
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B10" s="15" t="s">
+      <c r="B10" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="C10" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="F10" s="15" t="s">
+      <c r="F10" s="14" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C11" s="15" t="s">
+      <c r="C11" s="14" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C12" s="22"/>
+      <c r="C12" s="23"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B14" s="3" t="s">
@@ -1285,7 +1368,7 @@
       <c r="C15" t="s">
         <v>14</v>
       </c>
-      <c r="D15" s="20" t="s">
+      <c r="D15" s="21" t="s">
         <v>25</v>
       </c>
       <c r="E15" t="s">
@@ -1300,7 +1383,7 @@
       <c r="H15" t="s">
         <v>14</v>
       </c>
-      <c r="I15" s="17" t="s">
+      <c r="I15" s="16" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1334,7 +1417,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5186853C-8F41-E14D-BD0A-415B9ACDCBCD}">
-  <dimension ref="A1:F132"/>
+  <dimension ref="A1:F149"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3.33203125" bestFit="1" customWidth="1"/>
@@ -1345,12 +1428,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B1" s="10" t="s">
-        <v>130</v>
-      </c>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
+      <c r="B1" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
@@ -1465,7 +1548,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>122</v>
+        <v>111</v>
       </c>
       <c r="C9" t="s">
         <v>55</v>
@@ -1507,7 +1590,7 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>123</v>
+        <v>112</v>
       </c>
       <c r="C12" t="s">
         <v>54</v>
@@ -1539,12 +1622,12 @@
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B17" s="10" t="s">
-        <v>131</v>
-      </c>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
+      <c r="B17" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="C17" s="11"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
@@ -1602,7 +1685,7 @@
         <v>3</v>
       </c>
       <c r="B21" t="s">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="C21" t="s">
         <v>82</v>
@@ -1655,7 +1738,7 @@
         <v>7</v>
       </c>
       <c r="B25" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="C25" t="s">
         <v>55</v>
@@ -1669,7 +1752,7 @@
         <v>8</v>
       </c>
       <c r="B26" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
       <c r="C26" t="s">
         <v>55</v>
@@ -1683,7 +1766,7 @@
         <v>9</v>
       </c>
       <c r="B27" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="C27" t="s">
         <v>55</v>
@@ -1697,7 +1780,7 @@
         <v>10</v>
       </c>
       <c r="B28" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="C28" t="s">
         <v>55</v>
@@ -1711,7 +1794,7 @@
         <v>11</v>
       </c>
       <c r="B29" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="C29" t="s">
         <v>55</v>
@@ -1725,7 +1808,7 @@
         <v>12</v>
       </c>
       <c r="B30" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="C30" t="s">
         <v>55</v>
@@ -1739,7 +1822,7 @@
         <v>13</v>
       </c>
       <c r="B31" t="s">
-        <v>108</v>
+        <v>97</v>
       </c>
       <c r="C31" t="s">
         <v>55</v>
@@ -1753,7 +1836,7 @@
         <v>14</v>
       </c>
       <c r="B32" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="C32" t="s">
         <v>66</v>
@@ -1768,12 +1851,12 @@
       <c r="C34" s="6"/>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B35" s="10" t="s">
-        <v>132</v>
-      </c>
-      <c r="C35" s="10"/>
-      <c r="D35" s="10"/>
-      <c r="E35" s="10"/>
+      <c r="B35" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="C35" s="11"/>
+      <c r="D35" s="11"/>
+      <c r="E35" s="11"/>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
@@ -1859,7 +1942,7 @@
         <v>5</v>
       </c>
       <c r="B41" t="s">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="C41" t="s">
         <v>82</v>
@@ -1870,7 +1953,7 @@
         <v>6</v>
       </c>
       <c r="B42" t="s">
-        <v>126</v>
+        <v>115</v>
       </c>
       <c r="C42" t="s">
         <v>73</v>
@@ -1884,7 +1967,7 @@
         <v>7</v>
       </c>
       <c r="B43" t="s">
-        <v>124</v>
+        <v>113</v>
       </c>
       <c r="C43" t="s">
         <v>55</v>
@@ -1898,7 +1981,7 @@
         <v>8</v>
       </c>
       <c r="B44" t="s">
-        <v>125</v>
+        <v>114</v>
       </c>
       <c r="C44" t="s">
         <v>55</v>
@@ -1908,12 +1991,12 @@
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B47" s="10" t="s">
-        <v>129</v>
-      </c>
-      <c r="C47" s="10"/>
-      <c r="D47" s="10"/>
-      <c r="E47" s="10"/>
+      <c r="B47" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="C47" s="11"/>
+      <c r="D47" s="11"/>
+      <c r="E47" s="11"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
@@ -1971,10 +2054,10 @@
         <v>3</v>
       </c>
       <c r="B51" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="C51" t="s">
-        <v>128</v>
+        <v>117</v>
       </c>
       <c r="D51">
         <v>50</v>
@@ -2003,12 +2086,12 @@
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B56" s="10" t="s">
-        <v>134</v>
-      </c>
-      <c r="C56" s="10"/>
-      <c r="D56" s="10"/>
-      <c r="E56" s="10"/>
+      <c r="B56" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="C56" s="11"/>
+      <c r="D56" s="11"/>
+      <c r="E56" s="11"/>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A57" s="2" t="s">
@@ -2080,10 +2163,10 @@
         <v>4</v>
       </c>
       <c r="B61" t="s">
-        <v>133</v>
+        <v>122</v>
       </c>
       <c r="C61" t="s">
-        <v>128</v>
+        <v>117</v>
       </c>
       <c r="D61">
         <v>50</v>
@@ -2108,7 +2191,7 @@
         <v>6</v>
       </c>
       <c r="B63" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C63" t="s">
         <v>67</v>
@@ -2118,12 +2201,12 @@
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B65" s="10" t="s">
-        <v>140</v>
-      </c>
-      <c r="C65" s="10"/>
-      <c r="D65" s="10"/>
-      <c r="E65" s="10"/>
+      <c r="B65" s="11" t="s">
+        <v>129</v>
+      </c>
+      <c r="C65" s="11"/>
+      <c r="D65" s="11"/>
+      <c r="E65" s="11"/>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
@@ -2164,7 +2247,7 @@
         <v>2</v>
       </c>
       <c r="B68" t="s">
-        <v>141</v>
+        <v>130</v>
       </c>
       <c r="C68" t="s">
         <v>55</v>
@@ -2181,7 +2264,7 @@
         <v>3</v>
       </c>
       <c r="B69" t="s">
-        <v>142</v>
+        <v>131</v>
       </c>
       <c r="C69" t="s">
         <v>55</v>
@@ -2209,7 +2292,7 @@
         <v>5</v>
       </c>
       <c r="B71" t="s">
-        <v>143</v>
+        <v>132</v>
       </c>
       <c r="C71" t="s">
         <v>55</v>
@@ -2223,10 +2306,10 @@
         <v>6</v>
       </c>
       <c r="B72" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="C72" t="s">
-        <v>128</v>
+        <v>117</v>
       </c>
       <c r="D72">
         <v>20</v>
@@ -2255,12 +2338,12 @@
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B77" s="10" t="s">
-        <v>139</v>
-      </c>
-      <c r="C77" s="10"/>
-      <c r="D77" s="10"/>
-      <c r="E77" s="10"/>
+      <c r="B77" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="C77" s="11"/>
+      <c r="D77" s="11"/>
+      <c r="E77" s="11"/>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A78" s="2" t="s">
@@ -2349,10 +2432,10 @@
         <v>5</v>
       </c>
       <c r="B83" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="C83" t="s">
-        <v>138</v>
+        <v>127</v>
       </c>
       <c r="D83">
         <v>20</v>
@@ -2363,7 +2446,7 @@
         <v>6</v>
       </c>
       <c r="B84" t="s">
-        <v>136</v>
+        <v>125</v>
       </c>
       <c r="C84" t="s">
         <v>55</v>
@@ -2377,7 +2460,7 @@
         <v>7</v>
       </c>
       <c r="B85" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="C85" t="s">
         <v>55</v>
@@ -2402,19 +2485,19 @@
         <v>9</v>
       </c>
       <c r="B87" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C87" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B90" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="C90" s="10"/>
-      <c r="D90" s="10"/>
-      <c r="E90" s="10"/>
+      <c r="B90" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="C90" s="11"/>
+      <c r="D90" s="11"/>
+      <c r="E90" s="11"/>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A91" s="2" t="s">
@@ -2455,7 +2538,7 @@
         <v>2</v>
       </c>
       <c r="B93" t="s">
-        <v>76</v>
+        <v>137</v>
       </c>
       <c r="C93" t="s">
         <v>66</v>
@@ -2472,7 +2555,7 @@
         <v>3</v>
       </c>
       <c r="B94" t="s">
-        <v>77</v>
+        <v>138</v>
       </c>
       <c r="C94" t="s">
         <v>66</v>
@@ -2489,13 +2572,16 @@
         <v>4</v>
       </c>
       <c r="B95" t="s">
-        <v>83</v>
+        <v>139</v>
       </c>
       <c r="C95" t="s">
         <v>55</v>
       </c>
       <c r="D95">
         <v>100</v>
+      </c>
+      <c r="E95" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.2">
@@ -2503,7 +2589,7 @@
         <v>5</v>
       </c>
       <c r="B96" t="s">
-        <v>84</v>
+        <v>140</v>
       </c>
       <c r="C96" t="s">
         <v>55</v>
@@ -2517,13 +2603,13 @@
         <v>6</v>
       </c>
       <c r="B97" t="s">
-        <v>95</v>
+        <v>141</v>
       </c>
       <c r="C97" t="s">
-        <v>96</v>
+        <v>55</v>
       </c>
       <c r="D97">
-        <v>1000</v>
+        <v>100</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.2">
@@ -2531,10 +2617,10 @@
         <v>7</v>
       </c>
       <c r="B98" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C98" t="s">
-        <v>96</v>
+        <v>55</v>
       </c>
       <c r="D98">
         <v>1000</v>
@@ -2545,10 +2631,13 @@
         <v>8</v>
       </c>
       <c r="B99" t="s">
-        <v>52</v>
+        <v>84</v>
       </c>
       <c r="C99" t="s">
-        <v>67</v>
+        <v>55</v>
+      </c>
+      <c r="D99">
+        <v>5000</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.2">
@@ -2556,119 +2645,152 @@
         <v>9</v>
       </c>
       <c r="B100" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C100" t="s">
+        <v>55</v>
+      </c>
+      <c r="D100">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A101">
+        <v>10</v>
+      </c>
+      <c r="B101" t="s">
+        <v>142</v>
+      </c>
+      <c r="C101" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A102">
+        <v>11</v>
+      </c>
+      <c r="B102" t="s">
+        <v>143</v>
+      </c>
+      <c r="C102" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A103">
+        <v>12</v>
+      </c>
+      <c r="B103" t="s">
+        <v>52</v>
+      </c>
+      <c r="C103" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B103" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="C103" s="10"/>
-      <c r="D103" s="10"/>
-      <c r="E103" s="10"/>
-    </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A104" s="2" t="s">
+      <c r="A104">
+        <v>13</v>
+      </c>
+      <c r="B104" t="s">
+        <v>85</v>
+      </c>
+      <c r="C104" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B107" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="C107" s="11"/>
+      <c r="D107" s="11"/>
+      <c r="E107" s="11"/>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A108" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B104" s="7" t="s">
+      <c r="B108" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="C104" s="7" t="s">
+      <c r="C108" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="D104" s="2" t="s">
+      <c r="D108" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="E104" s="2" t="s">
+      <c r="E108" s="2" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A105">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A109">
         <v>1</v>
       </c>
-      <c r="B105" t="s">
+      <c r="B109" t="s">
         <v>51</v>
       </c>
-      <c r="C105" t="s">
+      <c r="C109" t="s">
         <v>66</v>
       </c>
-      <c r="D105">
+      <c r="D109">
         <v>20</v>
       </c>
-      <c r="E105" t="s">
+      <c r="E109" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A106">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A110">
         <v>2</v>
       </c>
-      <c r="B106" t="s">
-        <v>76</v>
-      </c>
-      <c r="C106" t="s">
+      <c r="B110" t="s">
+        <v>145</v>
+      </c>
+      <c r="C110" t="s">
         <v>66</v>
       </c>
-      <c r="D106">
+      <c r="D110">
         <v>20</v>
       </c>
-      <c r="E106" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A107">
+      <c r="E110" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A111">
         <v>3</v>
       </c>
-      <c r="B107" t="s">
-        <v>77</v>
-      </c>
-      <c r="C107" t="s">
+      <c r="B111" t="s">
+        <v>146</v>
+      </c>
+      <c r="C111" t="s">
         <v>66</v>
       </c>
-      <c r="D107">
+      <c r="D111">
         <v>20</v>
       </c>
-      <c r="E107" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A108">
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A112">
         <v>4</v>
       </c>
-      <c r="B108" s="13" t="s">
-        <v>87</v>
-      </c>
-      <c r="C108" s="14"/>
-    </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B109" s="14"/>
-      <c r="C109" s="14"/>
-    </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B110" s="14"/>
-      <c r="C110" s="14"/>
-    </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B111" s="14"/>
-      <c r="C111" s="14"/>
-    </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B112" s="14"/>
-      <c r="C112" s="14"/>
+      <c r="B112" t="s">
+        <v>147</v>
+      </c>
+      <c r="C112" t="s">
+        <v>55</v>
+      </c>
+      <c r="D112">
+        <v>200</v>
+      </c>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A113">
         <v>5</v>
       </c>
       <c r="B113" t="s">
-        <v>84</v>
+        <v>148</v>
       </c>
       <c r="C113" t="s">
         <v>55</v>
@@ -2682,204 +2804,459 @@
         <v>6</v>
       </c>
       <c r="B114" t="s">
-        <v>85</v>
+        <v>149</v>
       </c>
       <c r="C114" t="s">
         <v>55</v>
       </c>
       <c r="D114">
-        <v>1000</v>
+        <v>500</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A115">
+        <v>7</v>
+      </c>
+      <c r="B115" t="s">
+        <v>150</v>
+      </c>
+      <c r="C115" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A116">
+        <v>8</v>
+      </c>
+      <c r="B116" t="s">
+        <v>151</v>
+      </c>
+      <c r="C116" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B117" s="10" t="s">
-        <v>100</v>
-      </c>
-      <c r="C117" s="10"/>
-      <c r="D117" s="10"/>
-      <c r="E117" s="10"/>
+      <c r="A117">
+        <v>9</v>
+      </c>
+      <c r="B117" t="s">
+        <v>152</v>
+      </c>
+      <c r="C117" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A118" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="B118" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="C118" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D118" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="E118" s="2" t="s">
-        <v>60</v>
+      <c r="A118">
+        <v>10</v>
+      </c>
+      <c r="B118" t="s">
+        <v>153</v>
+      </c>
+      <c r="C118" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A119">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="B119" t="s">
-        <v>51</v>
+        <v>154</v>
       </c>
       <c r="C119" t="s">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="D119">
-        <v>20</v>
-      </c>
-      <c r="E119" t="s">
-        <v>78</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A120">
+        <v>12</v>
+      </c>
+      <c r="B120" t="s">
+        <v>74</v>
+      </c>
+      <c r="C120" t="s">
+        <v>55</v>
+      </c>
+      <c r="D120">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="123" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B123" s="11" t="s">
+        <v>155</v>
+      </c>
+      <c r="C123" s="11"/>
+      <c r="D123" s="11"/>
+      <c r="E123" s="11"/>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A124" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B124" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="C124" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="D124" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E124" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A125">
+        <v>1</v>
+      </c>
+      <c r="B125" t="s">
+        <v>51</v>
+      </c>
+      <c r="C125" t="s">
+        <v>66</v>
+      </c>
+      <c r="D125">
+        <v>20</v>
+      </c>
+      <c r="E125" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A126">
         <v>2</v>
       </c>
-      <c r="B120" t="s">
-        <v>76</v>
-      </c>
-      <c r="C120" t="s">
+      <c r="B126" t="s">
+        <v>156</v>
+      </c>
+      <c r="C126" t="s">
+        <v>55</v>
+      </c>
+      <c r="D126">
+        <v>20</v>
+      </c>
+      <c r="E126" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="127" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A127">
+        <v>3</v>
+      </c>
+      <c r="B127" t="s">
+        <v>157</v>
+      </c>
+      <c r="C127" t="s">
+        <v>55</v>
+      </c>
+      <c r="D127">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="128" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A128">
+        <v>4</v>
+      </c>
+      <c r="B128" t="s">
+        <v>148</v>
+      </c>
+      <c r="C128" t="s">
+        <v>55</v>
+      </c>
+      <c r="D128">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A129">
+        <v>5</v>
+      </c>
+      <c r="B129" t="s">
+        <v>158</v>
+      </c>
+      <c r="C129" t="s">
+        <v>55</v>
+      </c>
+      <c r="D129">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="A130">
+        <v>6</v>
+      </c>
+      <c r="B130" s="18" t="s">
+        <v>150</v>
+      </c>
+      <c r="C130" s="19" t="s">
+        <v>73</v>
+      </c>
+      <c r="D130" s="25" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A131">
+        <v>7</v>
+      </c>
+      <c r="B131" s="19" t="s">
+        <v>159</v>
+      </c>
+      <c r="C131" s="19" t="s">
+        <v>73</v>
+      </c>
+      <c r="D131" s="25" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A132">
+        <v>8</v>
+      </c>
+      <c r="B132" s="19" t="s">
+        <v>160</v>
+      </c>
+      <c r="C132" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="D132" s="25" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A133" s="25">
+        <v>9</v>
+      </c>
+      <c r="B133" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="C133" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D133" s="25" t="s">
+        <v>55</v>
+      </c>
+      <c r="E133" s="24"/>
+      <c r="F133" s="24"/>
+    </row>
+    <row r="134" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A134" s="24"/>
+      <c r="B134" s="8"/>
+      <c r="C134" s="8"/>
+      <c r="D134" s="24"/>
+      <c r="E134" s="24"/>
+      <c r="F134" s="24"/>
+    </row>
+    <row r="135" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A135" s="24"/>
+      <c r="B135" s="8"/>
+      <c r="C135" s="8"/>
+      <c r="D135" s="24"/>
+      <c r="E135" s="24"/>
+      <c r="F135" s="24"/>
+    </row>
+    <row r="136" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B136" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="C136" s="11"/>
+      <c r="D136" s="11"/>
+      <c r="E136" s="11"/>
+    </row>
+    <row r="137" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A137" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B137" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="C137" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="D137" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E137" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A138">
+        <v>1</v>
+      </c>
+      <c r="B138" t="s">
+        <v>51</v>
+      </c>
+      <c r="C138" t="s">
         <v>66</v>
       </c>
-      <c r="D120">
+      <c r="D138">
         <v>20</v>
       </c>
-      <c r="E120" t="s">
+      <c r="E138" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="139" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A139">
+        <v>2</v>
+      </c>
+      <c r="B139" t="s">
+        <v>162</v>
+      </c>
+      <c r="C139" t="s">
+        <v>66</v>
+      </c>
+      <c r="D139">
+        <v>20</v>
+      </c>
+      <c r="E139" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A121">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A140">
         <v>3</v>
       </c>
-      <c r="B121" t="s">
-        <v>88</v>
-      </c>
-      <c r="C121" t="s">
-        <v>55</v>
-      </c>
-      <c r="D121">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A122">
+      <c r="B140" t="s">
+        <v>163</v>
+      </c>
+      <c r="C140" t="s">
+        <v>66</v>
+      </c>
+      <c r="D140">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="141" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A141">
         <v>4</v>
       </c>
-      <c r="B122" t="s">
-        <v>89</v>
-      </c>
-      <c r="C122" t="s">
-        <v>54</v>
-      </c>
-      <c r="D122">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A123">
+      <c r="B141" t="s">
+        <v>164</v>
+      </c>
+      <c r="C141" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="142" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A142">
         <v>5</v>
       </c>
-      <c r="B123" t="s">
-        <v>90</v>
-      </c>
-      <c r="C123" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A124">
+      <c r="B142" t="s">
+        <v>165</v>
+      </c>
+      <c r="C142" t="s">
+        <v>172</v>
+      </c>
+      <c r="D142">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="143" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A143">
         <v>6</v>
       </c>
-      <c r="B124" s="13" t="s">
-        <v>91</v>
-      </c>
-      <c r="C124" s="14"/>
-    </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B125" s="14"/>
-      <c r="C125" s="14"/>
-    </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B126" s="14"/>
-      <c r="C126" s="14"/>
-    </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B129" s="10" t="s">
-        <v>101</v>
-      </c>
-      <c r="C129" s="10"/>
-      <c r="D129" s="10"/>
-      <c r="E129" s="10"/>
-    </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A130" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="B130" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="C130" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D130" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="E130" s="2" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A131">
-        <v>1</v>
-      </c>
-      <c r="B131" t="s">
-        <v>51</v>
-      </c>
-      <c r="C131" t="s">
+      <c r="B143" t="s">
+        <v>138</v>
+      </c>
+      <c r="C143" t="s">
+        <v>55</v>
+      </c>
+      <c r="D143">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="144" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A144">
+        <v>7</v>
+      </c>
+      <c r="B144" t="s">
+        <v>166</v>
+      </c>
+      <c r="C144" t="s">
         <v>66</v>
       </c>
-      <c r="D131">
+      <c r="D144">
         <v>20</v>
       </c>
-      <c r="E131" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A132">
-        <v>2</v>
-      </c>
-      <c r="B132" t="s">
-        <v>76</v>
-      </c>
-      <c r="C132" t="s">
-        <v>66</v>
-      </c>
-      <c r="D132">
-        <v>20</v>
-      </c>
-      <c r="E132" t="s">
-        <v>79</v>
+    </row>
+    <row r="145" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A145">
+        <v>8</v>
+      </c>
+      <c r="B145" t="s">
+        <v>167</v>
+      </c>
+      <c r="C145" t="s">
+        <v>55</v>
+      </c>
+      <c r="D145">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="146" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A146">
+        <v>9</v>
+      </c>
+      <c r="B146" t="s">
+        <v>168</v>
+      </c>
+      <c r="C146" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="147" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A147">
+        <v>10</v>
+      </c>
+      <c r="B147" t="s">
+        <v>169</v>
+      </c>
+      <c r="C147" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="148" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A148">
+        <v>11</v>
+      </c>
+      <c r="B148" t="s">
+        <v>171</v>
+      </c>
+      <c r="C148" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="149" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A149">
+        <v>12</v>
+      </c>
+      <c r="B149" t="s">
+        <v>170</v>
+      </c>
+      <c r="C149" t="s">
+        <v>67</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="11">
     <mergeCell ref="B47:E47"/>
     <mergeCell ref="B56:E56"/>
     <mergeCell ref="B65:E65"/>
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="B17:E17"/>
     <mergeCell ref="B35:E35"/>
-    <mergeCell ref="B124:C126"/>
-    <mergeCell ref="B129:E129"/>
+    <mergeCell ref="B136:E136"/>
     <mergeCell ref="B77:E77"/>
     <mergeCell ref="B90:E90"/>
-    <mergeCell ref="B103:E103"/>
-    <mergeCell ref="B108:C112"/>
-    <mergeCell ref="B117:E117"/>
+    <mergeCell ref="B107:E107"/>
+    <mergeCell ref="B123:E123"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2894,908 +3271,908 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:24" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8"/>
-      <c r="J3" s="8"/>
-      <c r="K3" s="8"/>
-      <c r="M3" s="9" t="s">
-        <v>93</v>
-      </c>
-      <c r="N3" s="9"/>
-      <c r="O3" s="9"/>
-      <c r="P3" s="9"/>
-      <c r="Q3" s="9"/>
-      <c r="R3" s="9"/>
-      <c r="S3" s="9"/>
-      <c r="T3" s="9"/>
-      <c r="U3" s="9"/>
-      <c r="V3" s="9"/>
-      <c r="W3" s="9"/>
-      <c r="X3" s="9"/>
+      <c r="A3" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+      <c r="M3" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="N3" s="10"/>
+      <c r="O3" s="10"/>
+      <c r="P3" s="10"/>
+      <c r="Q3" s="10"/>
+      <c r="R3" s="10"/>
+      <c r="S3" s="10"/>
+      <c r="T3" s="10"/>
+      <c r="U3" s="10"/>
+      <c r="V3" s="10"/>
+      <c r="W3" s="10"/>
+      <c r="X3" s="10"/>
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A4" s="8"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
-      <c r="H4" s="8"/>
-      <c r="I4" s="8"/>
-      <c r="J4" s="8"/>
-      <c r="K4" s="8"/>
-      <c r="M4" s="9"/>
-      <c r="N4" s="9"/>
-      <c r="O4" s="9"/>
-      <c r="P4" s="9"/>
-      <c r="Q4" s="9"/>
-      <c r="R4" s="9"/>
-      <c r="S4" s="9"/>
-      <c r="T4" s="9"/>
-      <c r="U4" s="9"/>
-      <c r="V4" s="9"/>
-      <c r="W4" s="9"/>
-      <c r="X4" s="9"/>
+      <c r="A4" s="9"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
+      <c r="I4" s="9"/>
+      <c r="J4" s="9"/>
+      <c r="K4" s="9"/>
+      <c r="M4" s="10"/>
+      <c r="N4" s="10"/>
+      <c r="O4" s="10"/>
+      <c r="P4" s="10"/>
+      <c r="Q4" s="10"/>
+      <c r="R4" s="10"/>
+      <c r="S4" s="10"/>
+      <c r="T4" s="10"/>
+      <c r="U4" s="10"/>
+      <c r="V4" s="10"/>
+      <c r="W4" s="10"/>
+      <c r="X4" s="10"/>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A5" s="8"/>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="8"/>
-      <c r="G5" s="8"/>
-      <c r="H5" s="8"/>
-      <c r="I5" s="8"/>
-      <c r="J5" s="8"/>
-      <c r="K5" s="8"/>
-      <c r="M5" s="9"/>
-      <c r="N5" s="9"/>
-      <c r="O5" s="9"/>
-      <c r="P5" s="9"/>
-      <c r="Q5" s="9"/>
-      <c r="R5" s="9"/>
-      <c r="S5" s="9"/>
-      <c r="T5" s="9"/>
-      <c r="U5" s="9"/>
-      <c r="V5" s="9"/>
-      <c r="W5" s="9"/>
-      <c r="X5" s="9"/>
+      <c r="A5" s="9"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="M5" s="10"/>
+      <c r="N5" s="10"/>
+      <c r="O5" s="10"/>
+      <c r="P5" s="10"/>
+      <c r="Q5" s="10"/>
+      <c r="R5" s="10"/>
+      <c r="S5" s="10"/>
+      <c r="T5" s="10"/>
+      <c r="U5" s="10"/>
+      <c r="V5" s="10"/>
+      <c r="W5" s="10"/>
+      <c r="X5" s="10"/>
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A6" s="8"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
-      <c r="I6" s="8"/>
-      <c r="J6" s="8"/>
-      <c r="K6" s="8"/>
-      <c r="M6" s="9"/>
-      <c r="N6" s="9"/>
-      <c r="O6" s="9"/>
-      <c r="P6" s="9"/>
-      <c r="Q6" s="9"/>
-      <c r="R6" s="9"/>
-      <c r="S6" s="9"/>
-      <c r="T6" s="9"/>
-      <c r="U6" s="9"/>
-      <c r="V6" s="9"/>
-      <c r="W6" s="9"/>
-      <c r="X6" s="9"/>
+      <c r="A6" s="9"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="9"/>
+      <c r="K6" s="9"/>
+      <c r="M6" s="10"/>
+      <c r="N6" s="10"/>
+      <c r="O6" s="10"/>
+      <c r="P6" s="10"/>
+      <c r="Q6" s="10"/>
+      <c r="R6" s="10"/>
+      <c r="S6" s="10"/>
+      <c r="T6" s="10"/>
+      <c r="U6" s="10"/>
+      <c r="V6" s="10"/>
+      <c r="W6" s="10"/>
+      <c r="X6" s="10"/>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A7" s="8"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="8"/>
-      <c r="M7" s="9"/>
-      <c r="N7" s="9"/>
-      <c r="O7" s="9"/>
-      <c r="P7" s="9"/>
-      <c r="Q7" s="9"/>
-      <c r="R7" s="9"/>
-      <c r="S7" s="9"/>
-      <c r="T7" s="9"/>
-      <c r="U7" s="9"/>
-      <c r="V7" s="9"/>
-      <c r="W7" s="9"/>
-      <c r="X7" s="9"/>
+      <c r="A7" s="9"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
+      <c r="M7" s="10"/>
+      <c r="N7" s="10"/>
+      <c r="O7" s="10"/>
+      <c r="P7" s="10"/>
+      <c r="Q7" s="10"/>
+      <c r="R7" s="10"/>
+      <c r="S7" s="10"/>
+      <c r="T7" s="10"/>
+      <c r="U7" s="10"/>
+      <c r="V7" s="10"/>
+      <c r="W7" s="10"/>
+      <c r="X7" s="10"/>
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A8" s="8"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
-      <c r="I8" s="8"/>
-      <c r="J8" s="8"/>
-      <c r="K8" s="8"/>
-      <c r="M8" s="9"/>
-      <c r="N8" s="9"/>
-      <c r="O8" s="9"/>
-      <c r="P8" s="9"/>
-      <c r="Q8" s="9"/>
-      <c r="R8" s="9"/>
-      <c r="S8" s="9"/>
-      <c r="T8" s="9"/>
-      <c r="U8" s="9"/>
-      <c r="V8" s="9"/>
-      <c r="W8" s="9"/>
-      <c r="X8" s="9"/>
+      <c r="A8" s="9"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="9"/>
+      <c r="I8" s="9"/>
+      <c r="J8" s="9"/>
+      <c r="K8" s="9"/>
+      <c r="M8" s="10"/>
+      <c r="N8" s="10"/>
+      <c r="O8" s="10"/>
+      <c r="P8" s="10"/>
+      <c r="Q8" s="10"/>
+      <c r="R8" s="10"/>
+      <c r="S8" s="10"/>
+      <c r="T8" s="10"/>
+      <c r="U8" s="10"/>
+      <c r="V8" s="10"/>
+      <c r="W8" s="10"/>
+      <c r="X8" s="10"/>
     </row>
     <row r="9" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A9" s="8"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
-      <c r="I9" s="8"/>
-      <c r="J9" s="8"/>
-      <c r="K9" s="8"/>
-      <c r="M9" s="9"/>
-      <c r="N9" s="9"/>
-      <c r="O9" s="9"/>
-      <c r="P9" s="9"/>
-      <c r="Q9" s="9"/>
-      <c r="R9" s="9"/>
-      <c r="S9" s="9"/>
-      <c r="T9" s="9"/>
-      <c r="U9" s="9"/>
-      <c r="V9" s="9"/>
-      <c r="W9" s="9"/>
-      <c r="X9" s="9"/>
+      <c r="A9" s="9"/>
+      <c r="B9" s="9"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="9"/>
+      <c r="I9" s="9"/>
+      <c r="J9" s="9"/>
+      <c r="K9" s="9"/>
+      <c r="M9" s="10"/>
+      <c r="N9" s="10"/>
+      <c r="O9" s="10"/>
+      <c r="P9" s="10"/>
+      <c r="Q9" s="10"/>
+      <c r="R9" s="10"/>
+      <c r="S9" s="10"/>
+      <c r="T9" s="10"/>
+      <c r="U9" s="10"/>
+      <c r="V9" s="10"/>
+      <c r="W9" s="10"/>
+      <c r="X9" s="10"/>
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A10" s="8"/>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
-      <c r="H10" s="8"/>
-      <c r="I10" s="8"/>
-      <c r="J10" s="8"/>
-      <c r="K10" s="8"/>
-      <c r="M10" s="9"/>
-      <c r="N10" s="9"/>
-      <c r="O10" s="9"/>
-      <c r="P10" s="9"/>
-      <c r="Q10" s="9"/>
-      <c r="R10" s="9"/>
-      <c r="S10" s="9"/>
-      <c r="T10" s="9"/>
-      <c r="U10" s="9"/>
-      <c r="V10" s="9"/>
-      <c r="W10" s="9"/>
-      <c r="X10" s="9"/>
+      <c r="A10" s="9"/>
+      <c r="B10" s="9"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
+      <c r="H10" s="9"/>
+      <c r="I10" s="9"/>
+      <c r="J10" s="9"/>
+      <c r="K10" s="9"/>
+      <c r="M10" s="10"/>
+      <c r="N10" s="10"/>
+      <c r="O10" s="10"/>
+      <c r="P10" s="10"/>
+      <c r="Q10" s="10"/>
+      <c r="R10" s="10"/>
+      <c r="S10" s="10"/>
+      <c r="T10" s="10"/>
+      <c r="U10" s="10"/>
+      <c r="V10" s="10"/>
+      <c r="W10" s="10"/>
+      <c r="X10" s="10"/>
     </row>
     <row r="11" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A11" s="8"/>
-      <c r="B11" s="8"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
-      <c r="H11" s="8"/>
-      <c r="I11" s="8"/>
-      <c r="J11" s="8"/>
-      <c r="K11" s="8"/>
-      <c r="M11" s="9"/>
-      <c r="N11" s="9"/>
-      <c r="O11" s="9"/>
-      <c r="P11" s="9"/>
-      <c r="Q11" s="9"/>
-      <c r="R11" s="9"/>
-      <c r="S11" s="9"/>
-      <c r="T11" s="9"/>
-      <c r="U11" s="9"/>
-      <c r="V11" s="9"/>
-      <c r="W11" s="9"/>
-      <c r="X11" s="9"/>
+      <c r="A11" s="9"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="9"/>
+      <c r="I11" s="9"/>
+      <c r="J11" s="9"/>
+      <c r="K11" s="9"/>
+      <c r="M11" s="10"/>
+      <c r="N11" s="10"/>
+      <c r="O11" s="10"/>
+      <c r="P11" s="10"/>
+      <c r="Q11" s="10"/>
+      <c r="R11" s="10"/>
+      <c r="S11" s="10"/>
+      <c r="T11" s="10"/>
+      <c r="U11" s="10"/>
+      <c r="V11" s="10"/>
+      <c r="W11" s="10"/>
+      <c r="X11" s="10"/>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A12" s="8"/>
-      <c r="B12" s="8"/>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="8"/>
-      <c r="G12" s="8"/>
-      <c r="H12" s="8"/>
-      <c r="I12" s="8"/>
-      <c r="J12" s="8"/>
-      <c r="K12" s="8"/>
-      <c r="M12" s="9"/>
-      <c r="N12" s="9"/>
-      <c r="O12" s="9"/>
-      <c r="P12" s="9"/>
-      <c r="Q12" s="9"/>
-      <c r="R12" s="9"/>
-      <c r="S12" s="9"/>
-      <c r="T12" s="9"/>
-      <c r="U12" s="9"/>
-      <c r="V12" s="9"/>
-      <c r="W12" s="9"/>
-      <c r="X12" s="9"/>
+      <c r="A12" s="9"/>
+      <c r="B12" s="9"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
+      <c r="H12" s="9"/>
+      <c r="I12" s="9"/>
+      <c r="J12" s="9"/>
+      <c r="K12" s="9"/>
+      <c r="M12" s="10"/>
+      <c r="N12" s="10"/>
+      <c r="O12" s="10"/>
+      <c r="P12" s="10"/>
+      <c r="Q12" s="10"/>
+      <c r="R12" s="10"/>
+      <c r="S12" s="10"/>
+      <c r="T12" s="10"/>
+      <c r="U12" s="10"/>
+      <c r="V12" s="10"/>
+      <c r="W12" s="10"/>
+      <c r="X12" s="10"/>
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A13" s="8"/>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
-      <c r="H13" s="8"/>
-      <c r="I13" s="8"/>
-      <c r="J13" s="8"/>
-      <c r="K13" s="8"/>
-      <c r="M13" s="9"/>
-      <c r="N13" s="9"/>
-      <c r="O13" s="9"/>
-      <c r="P13" s="9"/>
-      <c r="Q13" s="9"/>
-      <c r="R13" s="9"/>
-      <c r="S13" s="9"/>
-      <c r="T13" s="9"/>
-      <c r="U13" s="9"/>
-      <c r="V13" s="9"/>
-      <c r="W13" s="9"/>
-      <c r="X13" s="9"/>
+      <c r="A13" s="9"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="9"/>
+      <c r="I13" s="9"/>
+      <c r="J13" s="9"/>
+      <c r="K13" s="9"/>
+      <c r="M13" s="10"/>
+      <c r="N13" s="10"/>
+      <c r="O13" s="10"/>
+      <c r="P13" s="10"/>
+      <c r="Q13" s="10"/>
+      <c r="R13" s="10"/>
+      <c r="S13" s="10"/>
+      <c r="T13" s="10"/>
+      <c r="U13" s="10"/>
+      <c r="V13" s="10"/>
+      <c r="W13" s="10"/>
+      <c r="X13" s="10"/>
     </row>
     <row r="14" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A14" s="8"/>
-      <c r="B14" s="8"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="8"/>
-      <c r="F14" s="8"/>
-      <c r="G14" s="8"/>
-      <c r="H14" s="8"/>
-      <c r="I14" s="8"/>
-      <c r="J14" s="8"/>
-      <c r="K14" s="8"/>
-      <c r="M14" s="9"/>
-      <c r="N14" s="9"/>
-      <c r="O14" s="9"/>
-      <c r="P14" s="9"/>
-      <c r="Q14" s="9"/>
-      <c r="R14" s="9"/>
-      <c r="S14" s="9"/>
-      <c r="T14" s="9"/>
-      <c r="U14" s="9"/>
-      <c r="V14" s="9"/>
-      <c r="W14" s="9"/>
-      <c r="X14" s="9"/>
+      <c r="A14" s="9"/>
+      <c r="B14" s="9"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
+      <c r="H14" s="9"/>
+      <c r="I14" s="9"/>
+      <c r="J14" s="9"/>
+      <c r="K14" s="9"/>
+      <c r="M14" s="10"/>
+      <c r="N14" s="10"/>
+      <c r="O14" s="10"/>
+      <c r="P14" s="10"/>
+      <c r="Q14" s="10"/>
+      <c r="R14" s="10"/>
+      <c r="S14" s="10"/>
+      <c r="T14" s="10"/>
+      <c r="U14" s="10"/>
+      <c r="V14" s="10"/>
+      <c r="W14" s="10"/>
+      <c r="X14" s="10"/>
     </row>
     <row r="15" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A15" s="8"/>
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8"/>
-      <c r="F15" s="8"/>
-      <c r="G15" s="8"/>
-      <c r="H15" s="8"/>
-      <c r="I15" s="8"/>
-      <c r="J15" s="8"/>
-      <c r="K15" s="8"/>
-      <c r="M15" s="9"/>
-      <c r="N15" s="9"/>
-      <c r="O15" s="9"/>
-      <c r="P15" s="9"/>
-      <c r="Q15" s="9"/>
-      <c r="R15" s="9"/>
-      <c r="S15" s="9"/>
-      <c r="T15" s="9"/>
-      <c r="U15" s="9"/>
-      <c r="V15" s="9"/>
-      <c r="W15" s="9"/>
-      <c r="X15" s="9"/>
+      <c r="A15" s="9"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="9"/>
+      <c r="H15" s="9"/>
+      <c r="I15" s="9"/>
+      <c r="J15" s="9"/>
+      <c r="K15" s="9"/>
+      <c r="M15" s="10"/>
+      <c r="N15" s="10"/>
+      <c r="O15" s="10"/>
+      <c r="P15" s="10"/>
+      <c r="Q15" s="10"/>
+      <c r="R15" s="10"/>
+      <c r="S15" s="10"/>
+      <c r="T15" s="10"/>
+      <c r="U15" s="10"/>
+      <c r="V15" s="10"/>
+      <c r="W15" s="10"/>
+      <c r="X15" s="10"/>
     </row>
     <row r="16" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A16" s="8"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
-      <c r="H16" s="8"/>
-      <c r="I16" s="8"/>
-      <c r="J16" s="8"/>
-      <c r="K16" s="8"/>
-      <c r="M16" s="9"/>
-      <c r="N16" s="9"/>
-      <c r="O16" s="9"/>
-      <c r="P16" s="9"/>
-      <c r="Q16" s="9"/>
-      <c r="R16" s="9"/>
-      <c r="S16" s="9"/>
-      <c r="T16" s="9"/>
-      <c r="U16" s="9"/>
-      <c r="V16" s="9"/>
-      <c r="W16" s="9"/>
-      <c r="X16" s="9"/>
+      <c r="A16" s="9"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="9"/>
+      <c r="I16" s="9"/>
+      <c r="J16" s="9"/>
+      <c r="K16" s="9"/>
+      <c r="M16" s="10"/>
+      <c r="N16" s="10"/>
+      <c r="O16" s="10"/>
+      <c r="P16" s="10"/>
+      <c r="Q16" s="10"/>
+      <c r="R16" s="10"/>
+      <c r="S16" s="10"/>
+      <c r="T16" s="10"/>
+      <c r="U16" s="10"/>
+      <c r="V16" s="10"/>
+      <c r="W16" s="10"/>
+      <c r="X16" s="10"/>
     </row>
     <row r="17" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A17" s="8"/>
-      <c r="B17" s="8"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="8"/>
-      <c r="F17" s="8"/>
-      <c r="G17" s="8"/>
-      <c r="H17" s="8"/>
-      <c r="I17" s="8"/>
-      <c r="J17" s="8"/>
-      <c r="K17" s="8"/>
-      <c r="M17" s="9"/>
-      <c r="N17" s="9"/>
-      <c r="O17" s="9"/>
-      <c r="P17" s="9"/>
-      <c r="Q17" s="9"/>
-      <c r="R17" s="9"/>
-      <c r="S17" s="9"/>
-      <c r="T17" s="9"/>
-      <c r="U17" s="9"/>
-      <c r="V17" s="9"/>
-      <c r="W17" s="9"/>
-      <c r="X17" s="9"/>
+      <c r="A17" s="9"/>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
+      <c r="G17" s="9"/>
+      <c r="H17" s="9"/>
+      <c r="I17" s="9"/>
+      <c r="J17" s="9"/>
+      <c r="K17" s="9"/>
+      <c r="M17" s="10"/>
+      <c r="N17" s="10"/>
+      <c r="O17" s="10"/>
+      <c r="P17" s="10"/>
+      <c r="Q17" s="10"/>
+      <c r="R17" s="10"/>
+      <c r="S17" s="10"/>
+      <c r="T17" s="10"/>
+      <c r="U17" s="10"/>
+      <c r="V17" s="10"/>
+      <c r="W17" s="10"/>
+      <c r="X17" s="10"/>
     </row>
     <row r="18" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A18" s="8"/>
-      <c r="B18" s="8"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="8"/>
-      <c r="G18" s="8"/>
-      <c r="H18" s="8"/>
-      <c r="I18" s="8"/>
-      <c r="J18" s="8"/>
-      <c r="K18" s="8"/>
-      <c r="M18" s="9"/>
-      <c r="N18" s="9"/>
-      <c r="O18" s="9"/>
-      <c r="P18" s="9"/>
-      <c r="Q18" s="9"/>
-      <c r="R18" s="9"/>
-      <c r="S18" s="9"/>
-      <c r="T18" s="9"/>
-      <c r="U18" s="9"/>
-      <c r="V18" s="9"/>
-      <c r="W18" s="9"/>
-      <c r="X18" s="9"/>
+      <c r="A18" s="9"/>
+      <c r="B18" s="9"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
+      <c r="G18" s="9"/>
+      <c r="H18" s="9"/>
+      <c r="I18" s="9"/>
+      <c r="J18" s="9"/>
+      <c r="K18" s="9"/>
+      <c r="M18" s="10"/>
+      <c r="N18" s="10"/>
+      <c r="O18" s="10"/>
+      <c r="P18" s="10"/>
+      <c r="Q18" s="10"/>
+      <c r="R18" s="10"/>
+      <c r="S18" s="10"/>
+      <c r="T18" s="10"/>
+      <c r="U18" s="10"/>
+      <c r="V18" s="10"/>
+      <c r="W18" s="10"/>
+      <c r="X18" s="10"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A19" s="8"/>
-      <c r="B19" s="8"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="8"/>
-      <c r="G19" s="8"/>
-      <c r="H19" s="8"/>
-      <c r="I19" s="8"/>
-      <c r="J19" s="8"/>
-      <c r="K19" s="8"/>
-      <c r="M19" s="9"/>
-      <c r="N19" s="9"/>
-      <c r="O19" s="9"/>
-      <c r="P19" s="9"/>
-      <c r="Q19" s="9"/>
-      <c r="R19" s="9"/>
-      <c r="S19" s="9"/>
-      <c r="T19" s="9"/>
-      <c r="U19" s="9"/>
-      <c r="V19" s="9"/>
-      <c r="W19" s="9"/>
-      <c r="X19" s="9"/>
+      <c r="A19" s="9"/>
+      <c r="B19" s="9"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="9"/>
+      <c r="H19" s="9"/>
+      <c r="I19" s="9"/>
+      <c r="J19" s="9"/>
+      <c r="K19" s="9"/>
+      <c r="M19" s="10"/>
+      <c r="N19" s="10"/>
+      <c r="O19" s="10"/>
+      <c r="P19" s="10"/>
+      <c r="Q19" s="10"/>
+      <c r="R19" s="10"/>
+      <c r="S19" s="10"/>
+      <c r="T19" s="10"/>
+      <c r="U19" s="10"/>
+      <c r="V19" s="10"/>
+      <c r="W19" s="10"/>
+      <c r="X19" s="10"/>
     </row>
     <row r="20" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A20" s="8"/>
-      <c r="B20" s="8"/>
-      <c r="C20" s="8"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="8"/>
-      <c r="F20" s="8"/>
-      <c r="G20" s="8"/>
-      <c r="H20" s="8"/>
-      <c r="I20" s="8"/>
-      <c r="J20" s="8"/>
-      <c r="K20" s="8"/>
-      <c r="M20" s="9"/>
-      <c r="N20" s="9"/>
-      <c r="O20" s="9"/>
-      <c r="P20" s="9"/>
-      <c r="Q20" s="9"/>
-      <c r="R20" s="9"/>
-      <c r="S20" s="9"/>
-      <c r="T20" s="9"/>
-      <c r="U20" s="9"/>
-      <c r="V20" s="9"/>
-      <c r="W20" s="9"/>
-      <c r="X20" s="9"/>
+      <c r="A20" s="9"/>
+      <c r="B20" s="9"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="9"/>
+      <c r="G20" s="9"/>
+      <c r="H20" s="9"/>
+      <c r="I20" s="9"/>
+      <c r="J20" s="9"/>
+      <c r="K20" s="9"/>
+      <c r="M20" s="10"/>
+      <c r="N20" s="10"/>
+      <c r="O20" s="10"/>
+      <c r="P20" s="10"/>
+      <c r="Q20" s="10"/>
+      <c r="R20" s="10"/>
+      <c r="S20" s="10"/>
+      <c r="T20" s="10"/>
+      <c r="U20" s="10"/>
+      <c r="V20" s="10"/>
+      <c r="W20" s="10"/>
+      <c r="X20" s="10"/>
     </row>
     <row r="21" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A21" s="8"/>
-      <c r="B21" s="8"/>
-      <c r="C21" s="8"/>
-      <c r="D21" s="8"/>
-      <c r="E21" s="8"/>
-      <c r="F21" s="8"/>
-      <c r="G21" s="8"/>
-      <c r="H21" s="8"/>
-      <c r="I21" s="8"/>
-      <c r="J21" s="8"/>
-      <c r="K21" s="8"/>
-      <c r="M21" s="9"/>
-      <c r="N21" s="9"/>
-      <c r="O21" s="9"/>
-      <c r="P21" s="9"/>
-      <c r="Q21" s="9"/>
-      <c r="R21" s="9"/>
-      <c r="S21" s="9"/>
-      <c r="T21" s="9"/>
-      <c r="U21" s="9"/>
-      <c r="V21" s="9"/>
-      <c r="W21" s="9"/>
-      <c r="X21" s="9"/>
+      <c r="A21" s="9"/>
+      <c r="B21" s="9"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="9"/>
+      <c r="H21" s="9"/>
+      <c r="I21" s="9"/>
+      <c r="J21" s="9"/>
+      <c r="K21" s="9"/>
+      <c r="M21" s="10"/>
+      <c r="N21" s="10"/>
+      <c r="O21" s="10"/>
+      <c r="P21" s="10"/>
+      <c r="Q21" s="10"/>
+      <c r="R21" s="10"/>
+      <c r="S21" s="10"/>
+      <c r="T21" s="10"/>
+      <c r="U21" s="10"/>
+      <c r="V21" s="10"/>
+      <c r="W21" s="10"/>
+      <c r="X21" s="10"/>
     </row>
     <row r="22" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A22" s="8"/>
-      <c r="B22" s="8"/>
-      <c r="C22" s="8"/>
-      <c r="D22" s="8"/>
-      <c r="E22" s="8"/>
-      <c r="F22" s="8"/>
-      <c r="G22" s="8"/>
-      <c r="H22" s="8"/>
-      <c r="I22" s="8"/>
-      <c r="J22" s="8"/>
-      <c r="K22" s="8"/>
-      <c r="M22" s="9"/>
-      <c r="N22" s="9"/>
-      <c r="O22" s="9"/>
-      <c r="P22" s="9"/>
-      <c r="Q22" s="9"/>
-      <c r="R22" s="9"/>
-      <c r="S22" s="9"/>
-      <c r="T22" s="9"/>
-      <c r="U22" s="9"/>
-      <c r="V22" s="9"/>
-      <c r="W22" s="9"/>
-      <c r="X22" s="9"/>
+      <c r="A22" s="9"/>
+      <c r="B22" s="9"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
+      <c r="I22" s="9"/>
+      <c r="J22" s="9"/>
+      <c r="K22" s="9"/>
+      <c r="M22" s="10"/>
+      <c r="N22" s="10"/>
+      <c r="O22" s="10"/>
+      <c r="P22" s="10"/>
+      <c r="Q22" s="10"/>
+      <c r="R22" s="10"/>
+      <c r="S22" s="10"/>
+      <c r="T22" s="10"/>
+      <c r="U22" s="10"/>
+      <c r="V22" s="10"/>
+      <c r="W22" s="10"/>
+      <c r="X22" s="10"/>
     </row>
     <row r="23" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A23" s="8"/>
-      <c r="B23" s="8"/>
-      <c r="C23" s="8"/>
-      <c r="D23" s="8"/>
-      <c r="E23" s="8"/>
-      <c r="F23" s="8"/>
-      <c r="G23" s="8"/>
-      <c r="H23" s="8"/>
-      <c r="I23" s="8"/>
-      <c r="J23" s="8"/>
-      <c r="K23" s="8"/>
-      <c r="M23" s="9"/>
-      <c r="N23" s="9"/>
-      <c r="O23" s="9"/>
-      <c r="P23" s="9"/>
-      <c r="Q23" s="9"/>
-      <c r="R23" s="9"/>
-      <c r="S23" s="9"/>
-      <c r="T23" s="9"/>
-      <c r="U23" s="9"/>
-      <c r="V23" s="9"/>
-      <c r="W23" s="9"/>
-      <c r="X23" s="9"/>
+      <c r="A23" s="9"/>
+      <c r="B23" s="9"/>
+      <c r="C23" s="9"/>
+      <c r="D23" s="9"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
+      <c r="G23" s="9"/>
+      <c r="H23" s="9"/>
+      <c r="I23" s="9"/>
+      <c r="J23" s="9"/>
+      <c r="K23" s="9"/>
+      <c r="M23" s="10"/>
+      <c r="N23" s="10"/>
+      <c r="O23" s="10"/>
+      <c r="P23" s="10"/>
+      <c r="Q23" s="10"/>
+      <c r="R23" s="10"/>
+      <c r="S23" s="10"/>
+      <c r="T23" s="10"/>
+      <c r="U23" s="10"/>
+      <c r="V23" s="10"/>
+      <c r="W23" s="10"/>
+      <c r="X23" s="10"/>
     </row>
     <row r="24" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A24" s="8"/>
-      <c r="B24" s="8"/>
-      <c r="C24" s="8"/>
-      <c r="D24" s="8"/>
-      <c r="E24" s="8"/>
-      <c r="F24" s="8"/>
-      <c r="G24" s="8"/>
-      <c r="H24" s="8"/>
-      <c r="I24" s="8"/>
-      <c r="J24" s="8"/>
-      <c r="K24" s="8"/>
-      <c r="M24" s="9"/>
-      <c r="N24" s="9"/>
-      <c r="O24" s="9"/>
-      <c r="P24" s="9"/>
-      <c r="Q24" s="9"/>
-      <c r="R24" s="9"/>
-      <c r="S24" s="9"/>
-      <c r="T24" s="9"/>
-      <c r="U24" s="9"/>
-      <c r="V24" s="9"/>
-      <c r="W24" s="9"/>
-      <c r="X24" s="9"/>
+      <c r="A24" s="9"/>
+      <c r="B24" s="9"/>
+      <c r="C24" s="9"/>
+      <c r="D24" s="9"/>
+      <c r="E24" s="9"/>
+      <c r="F24" s="9"/>
+      <c r="G24" s="9"/>
+      <c r="H24" s="9"/>
+      <c r="I24" s="9"/>
+      <c r="J24" s="9"/>
+      <c r="K24" s="9"/>
+      <c r="M24" s="10"/>
+      <c r="N24" s="10"/>
+      <c r="O24" s="10"/>
+      <c r="P24" s="10"/>
+      <c r="Q24" s="10"/>
+      <c r="R24" s="10"/>
+      <c r="S24" s="10"/>
+      <c r="T24" s="10"/>
+      <c r="U24" s="10"/>
+      <c r="V24" s="10"/>
+      <c r="W24" s="10"/>
+      <c r="X24" s="10"/>
     </row>
     <row r="25" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A25" s="8"/>
-      <c r="B25" s="8"/>
-      <c r="C25" s="8"/>
-      <c r="D25" s="8"/>
-      <c r="E25" s="8"/>
-      <c r="F25" s="8"/>
-      <c r="G25" s="8"/>
-      <c r="H25" s="8"/>
-      <c r="I25" s="8"/>
-      <c r="J25" s="8"/>
-      <c r="K25" s="8"/>
-      <c r="M25" s="9"/>
-      <c r="N25" s="9"/>
-      <c r="O25" s="9"/>
-      <c r="P25" s="9"/>
-      <c r="Q25" s="9"/>
-      <c r="R25" s="9"/>
-      <c r="S25" s="9"/>
-      <c r="T25" s="9"/>
-      <c r="U25" s="9"/>
-      <c r="V25" s="9"/>
-      <c r="W25" s="9"/>
-      <c r="X25" s="9"/>
+      <c r="A25" s="9"/>
+      <c r="B25" s="9"/>
+      <c r="C25" s="9"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="9"/>
+      <c r="F25" s="9"/>
+      <c r="G25" s="9"/>
+      <c r="H25" s="9"/>
+      <c r="I25" s="9"/>
+      <c r="J25" s="9"/>
+      <c r="K25" s="9"/>
+      <c r="M25" s="10"/>
+      <c r="N25" s="10"/>
+      <c r="O25" s="10"/>
+      <c r="P25" s="10"/>
+      <c r="Q25" s="10"/>
+      <c r="R25" s="10"/>
+      <c r="S25" s="10"/>
+      <c r="T25" s="10"/>
+      <c r="U25" s="10"/>
+      <c r="V25" s="10"/>
+      <c r="W25" s="10"/>
+      <c r="X25" s="10"/>
     </row>
     <row r="26" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A26" s="8"/>
-      <c r="B26" s="8"/>
-      <c r="C26" s="8"/>
-      <c r="D26" s="8"/>
-      <c r="E26" s="8"/>
-      <c r="F26" s="8"/>
-      <c r="G26" s="8"/>
-      <c r="H26" s="8"/>
-      <c r="I26" s="8"/>
-      <c r="J26" s="8"/>
-      <c r="K26" s="8"/>
-      <c r="M26" s="9"/>
-      <c r="N26" s="9"/>
-      <c r="O26" s="9"/>
-      <c r="P26" s="9"/>
-      <c r="Q26" s="9"/>
-      <c r="R26" s="9"/>
-      <c r="S26" s="9"/>
-      <c r="T26" s="9"/>
-      <c r="U26" s="9"/>
-      <c r="V26" s="9"/>
-      <c r="W26" s="9"/>
-      <c r="X26" s="9"/>
+      <c r="A26" s="9"/>
+      <c r="B26" s="9"/>
+      <c r="C26" s="9"/>
+      <c r="D26" s="9"/>
+      <c r="E26" s="9"/>
+      <c r="F26" s="9"/>
+      <c r="G26" s="9"/>
+      <c r="H26" s="9"/>
+      <c r="I26" s="9"/>
+      <c r="J26" s="9"/>
+      <c r="K26" s="9"/>
+      <c r="M26" s="10"/>
+      <c r="N26" s="10"/>
+      <c r="O26" s="10"/>
+      <c r="P26" s="10"/>
+      <c r="Q26" s="10"/>
+      <c r="R26" s="10"/>
+      <c r="S26" s="10"/>
+      <c r="T26" s="10"/>
+      <c r="U26" s="10"/>
+      <c r="V26" s="10"/>
+      <c r="W26" s="10"/>
+      <c r="X26" s="10"/>
     </row>
     <row r="27" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A27" s="8"/>
-      <c r="B27" s="8"/>
-      <c r="C27" s="8"/>
-      <c r="D27" s="8"/>
-      <c r="E27" s="8"/>
-      <c r="F27" s="8"/>
-      <c r="G27" s="8"/>
-      <c r="H27" s="8"/>
-      <c r="I27" s="8"/>
-      <c r="J27" s="8"/>
-      <c r="K27" s="8"/>
-      <c r="M27" s="9"/>
-      <c r="N27" s="9"/>
-      <c r="O27" s="9"/>
-      <c r="P27" s="9"/>
-      <c r="Q27" s="9"/>
-      <c r="R27" s="9"/>
-      <c r="S27" s="9"/>
-      <c r="T27" s="9"/>
-      <c r="U27" s="9"/>
-      <c r="V27" s="9"/>
-      <c r="W27" s="9"/>
-      <c r="X27" s="9"/>
+      <c r="A27" s="9"/>
+      <c r="B27" s="9"/>
+      <c r="C27" s="9"/>
+      <c r="D27" s="9"/>
+      <c r="E27" s="9"/>
+      <c r="F27" s="9"/>
+      <c r="G27" s="9"/>
+      <c r="H27" s="9"/>
+      <c r="I27" s="9"/>
+      <c r="J27" s="9"/>
+      <c r="K27" s="9"/>
+      <c r="M27" s="10"/>
+      <c r="N27" s="10"/>
+      <c r="O27" s="10"/>
+      <c r="P27" s="10"/>
+      <c r="Q27" s="10"/>
+      <c r="R27" s="10"/>
+      <c r="S27" s="10"/>
+      <c r="T27" s="10"/>
+      <c r="U27" s="10"/>
+      <c r="V27" s="10"/>
+      <c r="W27" s="10"/>
+      <c r="X27" s="10"/>
     </row>
     <row r="28" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A28" s="8"/>
-      <c r="B28" s="8"/>
-      <c r="C28" s="8"/>
-      <c r="D28" s="8"/>
-      <c r="E28" s="8"/>
-      <c r="F28" s="8"/>
-      <c r="G28" s="8"/>
-      <c r="H28" s="8"/>
-      <c r="I28" s="8"/>
-      <c r="J28" s="8"/>
-      <c r="K28" s="8"/>
-      <c r="M28" s="9"/>
-      <c r="N28" s="9"/>
-      <c r="O28" s="9"/>
-      <c r="P28" s="9"/>
-      <c r="Q28" s="9"/>
-      <c r="R28" s="9"/>
-      <c r="S28" s="9"/>
-      <c r="T28" s="9"/>
-      <c r="U28" s="9"/>
-      <c r="V28" s="9"/>
-      <c r="W28" s="9"/>
-      <c r="X28" s="9"/>
+      <c r="A28" s="9"/>
+      <c r="B28" s="9"/>
+      <c r="C28" s="9"/>
+      <c r="D28" s="9"/>
+      <c r="E28" s="9"/>
+      <c r="F28" s="9"/>
+      <c r="G28" s="9"/>
+      <c r="H28" s="9"/>
+      <c r="I28" s="9"/>
+      <c r="J28" s="9"/>
+      <c r="K28" s="9"/>
+      <c r="M28" s="10"/>
+      <c r="N28" s="10"/>
+      <c r="O28" s="10"/>
+      <c r="P28" s="10"/>
+      <c r="Q28" s="10"/>
+      <c r="R28" s="10"/>
+      <c r="S28" s="10"/>
+      <c r="T28" s="10"/>
+      <c r="U28" s="10"/>
+      <c r="V28" s="10"/>
+      <c r="W28" s="10"/>
+      <c r="X28" s="10"/>
     </row>
     <row r="29" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="M29" s="9"/>
-      <c r="N29" s="9"/>
-      <c r="O29" s="9"/>
-      <c r="P29" s="9"/>
-      <c r="Q29" s="9"/>
-      <c r="R29" s="9"/>
-      <c r="S29" s="9"/>
-      <c r="T29" s="9"/>
-      <c r="U29" s="9"/>
-      <c r="V29" s="9"/>
-      <c r="W29" s="9"/>
-      <c r="X29" s="9"/>
+      <c r="M29" s="10"/>
+      <c r="N29" s="10"/>
+      <c r="O29" s="10"/>
+      <c r="P29" s="10"/>
+      <c r="Q29" s="10"/>
+      <c r="R29" s="10"/>
+      <c r="S29" s="10"/>
+      <c r="T29" s="10"/>
+      <c r="U29" s="10"/>
+      <c r="V29" s="10"/>
+      <c r="W29" s="10"/>
+      <c r="X29" s="10"/>
     </row>
     <row r="30" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="M30" s="9"/>
-      <c r="N30" s="9"/>
-      <c r="O30" s="9"/>
-      <c r="P30" s="9"/>
-      <c r="Q30" s="9"/>
-      <c r="R30" s="9"/>
-      <c r="S30" s="9"/>
-      <c r="T30" s="9"/>
-      <c r="U30" s="9"/>
-      <c r="V30" s="9"/>
-      <c r="W30" s="9"/>
-      <c r="X30" s="9"/>
+      <c r="M30" s="10"/>
+      <c r="N30" s="10"/>
+      <c r="O30" s="10"/>
+      <c r="P30" s="10"/>
+      <c r="Q30" s="10"/>
+      <c r="R30" s="10"/>
+      <c r="S30" s="10"/>
+      <c r="T30" s="10"/>
+      <c r="U30" s="10"/>
+      <c r="V30" s="10"/>
+      <c r="W30" s="10"/>
+      <c r="X30" s="10"/>
     </row>
     <row r="31" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="M31" s="9"/>
-      <c r="N31" s="9"/>
-      <c r="O31" s="9"/>
-      <c r="P31" s="9"/>
-      <c r="Q31" s="9"/>
-      <c r="R31" s="9"/>
-      <c r="S31" s="9"/>
-      <c r="T31" s="9"/>
-      <c r="U31" s="9"/>
-      <c r="V31" s="9"/>
-      <c r="W31" s="9"/>
-      <c r="X31" s="9"/>
+      <c r="M31" s="10"/>
+      <c r="N31" s="10"/>
+      <c r="O31" s="10"/>
+      <c r="P31" s="10"/>
+      <c r="Q31" s="10"/>
+      <c r="R31" s="10"/>
+      <c r="S31" s="10"/>
+      <c r="T31" s="10"/>
+      <c r="U31" s="10"/>
+      <c r="V31" s="10"/>
+      <c r="W31" s="10"/>
+      <c r="X31" s="10"/>
     </row>
     <row r="32" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="M32" s="9"/>
-      <c r="N32" s="9"/>
-      <c r="O32" s="9"/>
-      <c r="P32" s="9"/>
-      <c r="Q32" s="9"/>
-      <c r="R32" s="9"/>
-      <c r="S32" s="9"/>
-      <c r="T32" s="9"/>
-      <c r="U32" s="9"/>
-      <c r="V32" s="9"/>
-      <c r="W32" s="9"/>
-      <c r="X32" s="9"/>
+      <c r="M32" s="10"/>
+      <c r="N32" s="10"/>
+      <c r="O32" s="10"/>
+      <c r="P32" s="10"/>
+      <c r="Q32" s="10"/>
+      <c r="R32" s="10"/>
+      <c r="S32" s="10"/>
+      <c r="T32" s="10"/>
+      <c r="U32" s="10"/>
+      <c r="V32" s="10"/>
+      <c r="W32" s="10"/>
+      <c r="X32" s="10"/>
     </row>
     <row r="33" spans="1:24" ht="24" x14ac:dyDescent="0.3">
-      <c r="A33" s="18" t="s">
-        <v>110</v>
-      </c>
-      <c r="B33" s="18"/>
-      <c r="C33" s="18"/>
-      <c r="D33" s="18"/>
-      <c r="E33" s="18"/>
-      <c r="F33" s="18"/>
-      <c r="G33" s="18"/>
-      <c r="M33" s="9"/>
-      <c r="N33" s="9"/>
-      <c r="O33" s="9"/>
-      <c r="P33" s="9"/>
-      <c r="Q33" s="9"/>
-      <c r="R33" s="9"/>
-      <c r="S33" s="9"/>
-      <c r="T33" s="9"/>
-      <c r="U33" s="9"/>
-      <c r="V33" s="9"/>
-      <c r="W33" s="9"/>
-      <c r="X33" s="9"/>
+      <c r="A33" s="17" t="s">
+        <v>99</v>
+      </c>
+      <c r="B33" s="17"/>
+      <c r="C33" s="17"/>
+      <c r="D33" s="17"/>
+      <c r="E33" s="17"/>
+      <c r="F33" s="17"/>
+      <c r="G33" s="17"/>
+      <c r="M33" s="10"/>
+      <c r="N33" s="10"/>
+      <c r="O33" s="10"/>
+      <c r="P33" s="10"/>
+      <c r="Q33" s="10"/>
+      <c r="R33" s="10"/>
+      <c r="S33" s="10"/>
+      <c r="T33" s="10"/>
+      <c r="U33" s="10"/>
+      <c r="V33" s="10"/>
+      <c r="W33" s="10"/>
+      <c r="X33" s="10"/>
     </row>
     <row r="34" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>1</v>
       </c>
-      <c r="B34" s="15" t="s">
-        <v>111</v>
-      </c>
-      <c r="M34" s="9"/>
-      <c r="N34" s="9"/>
-      <c r="O34" s="9"/>
-      <c r="P34" s="9"/>
-      <c r="Q34" s="9"/>
-      <c r="R34" s="9"/>
-      <c r="S34" s="9"/>
-      <c r="T34" s="9"/>
-      <c r="U34" s="9"/>
-      <c r="V34" s="9"/>
-      <c r="W34" s="9"/>
-      <c r="X34" s="9"/>
+      <c r="B34" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="M34" s="10"/>
+      <c r="N34" s="10"/>
+      <c r="O34" s="10"/>
+      <c r="P34" s="10"/>
+      <c r="Q34" s="10"/>
+      <c r="R34" s="10"/>
+      <c r="S34" s="10"/>
+      <c r="T34" s="10"/>
+      <c r="U34" s="10"/>
+      <c r="V34" s="10"/>
+      <c r="W34" s="10"/>
+      <c r="X34" s="10"/>
     </row>
     <row r="35" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>2</v>
       </c>
-      <c r="B35" s="15" t="s">
-        <v>112</v>
-      </c>
-      <c r="M35" s="9"/>
-      <c r="N35" s="9"/>
-      <c r="O35" s="9"/>
-      <c r="P35" s="9"/>
-      <c r="Q35" s="9"/>
-      <c r="R35" s="9"/>
-      <c r="S35" s="9"/>
-      <c r="T35" s="9"/>
-      <c r="U35" s="9"/>
-      <c r="V35" s="9"/>
-      <c r="W35" s="9"/>
-      <c r="X35" s="9"/>
+      <c r="B35" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="M35" s="10"/>
+      <c r="N35" s="10"/>
+      <c r="O35" s="10"/>
+      <c r="P35" s="10"/>
+      <c r="Q35" s="10"/>
+      <c r="R35" s="10"/>
+      <c r="S35" s="10"/>
+      <c r="T35" s="10"/>
+      <c r="U35" s="10"/>
+      <c r="V35" s="10"/>
+      <c r="W35" s="10"/>
+      <c r="X35" s="10"/>
     </row>
     <row r="36" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>3</v>
       </c>
       <c r="B36" t="s">
-        <v>113</v>
-      </c>
-      <c r="M36" s="9"/>
-      <c r="N36" s="9"/>
-      <c r="O36" s="9"/>
-      <c r="P36" s="9"/>
-      <c r="Q36" s="9"/>
-      <c r="R36" s="9"/>
-      <c r="S36" s="9"/>
-      <c r="T36" s="9"/>
-      <c r="U36" s="9"/>
-      <c r="V36" s="9"/>
-      <c r="W36" s="9"/>
-      <c r="X36" s="9"/>
+        <v>102</v>
+      </c>
+      <c r="M36" s="10"/>
+      <c r="N36" s="10"/>
+      <c r="O36" s="10"/>
+      <c r="P36" s="10"/>
+      <c r="Q36" s="10"/>
+      <c r="R36" s="10"/>
+      <c r="S36" s="10"/>
+      <c r="T36" s="10"/>
+      <c r="U36" s="10"/>
+      <c r="V36" s="10"/>
+      <c r="W36" s="10"/>
+      <c r="X36" s="10"/>
     </row>
     <row r="37" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>4</v>
       </c>
       <c r="B37" t="s">
-        <v>115</v>
-      </c>
-      <c r="M37" s="9"/>
-      <c r="N37" s="9"/>
-      <c r="O37" s="9"/>
-      <c r="P37" s="9"/>
-      <c r="Q37" s="9"/>
-      <c r="R37" s="9"/>
-      <c r="S37" s="9"/>
-      <c r="T37" s="9"/>
-      <c r="U37" s="9"/>
-      <c r="V37" s="9"/>
-      <c r="W37" s="9"/>
-      <c r="X37" s="9"/>
+        <v>104</v>
+      </c>
+      <c r="M37" s="10"/>
+      <c r="N37" s="10"/>
+      <c r="O37" s="10"/>
+      <c r="P37" s="10"/>
+      <c r="Q37" s="10"/>
+      <c r="R37" s="10"/>
+      <c r="S37" s="10"/>
+      <c r="T37" s="10"/>
+      <c r="U37" s="10"/>
+      <c r="V37" s="10"/>
+      <c r="W37" s="10"/>
+      <c r="X37" s="10"/>
     </row>
     <row r="38" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>5</v>
       </c>
       <c r="B38" t="s">
-        <v>116</v>
-      </c>
-      <c r="M38" s="9"/>
-      <c r="N38" s="9"/>
-      <c r="O38" s="9"/>
-      <c r="P38" s="9"/>
-      <c r="Q38" s="9"/>
-      <c r="R38" s="9"/>
-      <c r="S38" s="9"/>
-      <c r="T38" s="9"/>
-      <c r="U38" s="9"/>
-      <c r="V38" s="9"/>
-      <c r="W38" s="9"/>
-      <c r="X38" s="9"/>
+        <v>105</v>
+      </c>
+      <c r="M38" s="10"/>
+      <c r="N38" s="10"/>
+      <c r="O38" s="10"/>
+      <c r="P38" s="10"/>
+      <c r="Q38" s="10"/>
+      <c r="R38" s="10"/>
+      <c r="S38" s="10"/>
+      <c r="T38" s="10"/>
+      <c r="U38" s="10"/>
+      <c r="V38" s="10"/>
+      <c r="W38" s="10"/>
+      <c r="X38" s="10"/>
     </row>
     <row r="39" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>6</v>
       </c>
-      <c r="B39" s="15" t="s">
-        <v>117</v>
-      </c>
-      <c r="C39" s="16"/>
-      <c r="D39" s="16"/>
-      <c r="E39" s="16"/>
-      <c r="M39" s="9"/>
-      <c r="N39" s="9"/>
-      <c r="O39" s="9"/>
-      <c r="P39" s="9"/>
-      <c r="Q39" s="9"/>
-      <c r="R39" s="9"/>
-      <c r="S39" s="9"/>
-      <c r="T39" s="9"/>
-      <c r="U39" s="9"/>
-      <c r="V39" s="9"/>
-      <c r="W39" s="9"/>
-      <c r="X39" s="9"/>
+      <c r="B39" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="C39" s="15"/>
+      <c r="D39" s="15"/>
+      <c r="E39" s="15"/>
+      <c r="M39" s="10"/>
+      <c r="N39" s="10"/>
+      <c r="O39" s="10"/>
+      <c r="P39" s="10"/>
+      <c r="Q39" s="10"/>
+      <c r="R39" s="10"/>
+      <c r="S39" s="10"/>
+      <c r="T39" s="10"/>
+      <c r="U39" s="10"/>
+      <c r="V39" s="10"/>
+      <c r="W39" s="10"/>
+      <c r="X39" s="10"/>
     </row>
     <row r="40" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>7</v>
       </c>
-      <c r="B40" s="15" t="s">
-        <v>118</v>
-      </c>
-      <c r="C40" s="16"/>
-      <c r="M40" s="9"/>
-      <c r="N40" s="9"/>
-      <c r="O40" s="9"/>
-      <c r="P40" s="9"/>
-      <c r="Q40" s="9"/>
-      <c r="R40" s="9"/>
-      <c r="S40" s="9"/>
-      <c r="T40" s="9"/>
-      <c r="U40" s="9"/>
-      <c r="V40" s="9"/>
-      <c r="W40" s="9"/>
-      <c r="X40" s="9"/>
+      <c r="B40" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="C40" s="15"/>
+      <c r="M40" s="10"/>
+      <c r="N40" s="10"/>
+      <c r="O40" s="10"/>
+      <c r="P40" s="10"/>
+      <c r="Q40" s="10"/>
+      <c r="R40" s="10"/>
+      <c r="S40" s="10"/>
+      <c r="T40" s="10"/>
+      <c r="U40" s="10"/>
+      <c r="V40" s="10"/>
+      <c r="W40" s="10"/>
+      <c r="X40" s="10"/>
     </row>
     <row r="41" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>8</v>
       </c>
       <c r="B41" t="s">
-        <v>119</v>
-      </c>
-      <c r="M41" s="9"/>
-      <c r="N41" s="9"/>
-      <c r="O41" s="9"/>
-      <c r="P41" s="9"/>
-      <c r="Q41" s="9"/>
-      <c r="R41" s="9"/>
-      <c r="S41" s="9"/>
-      <c r="T41" s="9"/>
-      <c r="U41" s="9"/>
-      <c r="V41" s="9"/>
-      <c r="W41" s="9"/>
-      <c r="X41" s="9"/>
+        <v>108</v>
+      </c>
+      <c r="M41" s="10"/>
+      <c r="N41" s="10"/>
+      <c r="O41" s="10"/>
+      <c r="P41" s="10"/>
+      <c r="Q41" s="10"/>
+      <c r="R41" s="10"/>
+      <c r="S41" s="10"/>
+      <c r="T41" s="10"/>
+      <c r="U41" s="10"/>
+      <c r="V41" s="10"/>
+      <c r="W41" s="10"/>
+      <c r="X41" s="10"/>
     </row>
     <row r="42" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>9</v>
       </c>
       <c r="B42" t="s">
-        <v>121</v>
+        <v>110</v>
       </c>
     </row>
     <row r="43" spans="1:24" x14ac:dyDescent="0.2">
@@ -3803,7 +4180,7 @@
         <v>10</v>
       </c>
       <c r="B43" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add doctor dashboard in frontend
</commit_message>
<xml_diff>
--- a/CareOS-Hospital_ERP_System.xlsx
+++ b/CareOS-Hospital_ERP_System.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hetlimbani/Desktop/Self_Learning/CareOS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{660731CF-F229-9C4A-A209-D89E306E117A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC734C12-BE7D-E641-8748-CEAF5C4C6E40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19420" activeTab="1" xr2:uid="{3BCF7A51-5C29-EE4C-8BC3-93CAF12DE1EA}"/>
+    <workbookView xWindow="-20" yWindow="680" windowWidth="34200" windowHeight="19420" xr2:uid="{3BCF7A51-5C29-EE4C-8BC3-93CAF12DE1EA}"/>
   </bookViews>
   <sheets>
     <sheet name="ERP System" sheetId="1" r:id="rId1"/>
     <sheet name="Schema" sheetId="2" r:id="rId2"/>
     <sheet name="Usefull" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="183">
   <si>
     <t>Total Roles</t>
   </si>
@@ -64,9 +64,6 @@
     <t>Hospital Admin</t>
   </si>
   <si>
-    <t>Ambulance Operator</t>
-  </si>
-  <si>
     <t>Features</t>
   </si>
   <si>
@@ -103,9 +100,6 @@
     <t>Lab Report Review</t>
   </si>
   <si>
-    <t>Doctor Notes</t>
-  </si>
-  <si>
     <t>Ward Dashboard</t>
   </si>
   <si>
@@ -167,18 +161,6 @@
   </si>
   <si>
     <t>Permissions</t>
-  </si>
-  <si>
-    <t>Emergency Requests</t>
-  </si>
-  <si>
-    <t>GPS Tracking</t>
-  </si>
-  <si>
-    <t>Driver Assignment</t>
-  </si>
-  <si>
-    <t>Route Tracking</t>
   </si>
   <si>
     <t>Must to Have</t>
@@ -658,7 +640,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -677,13 +659,6 @@
       <sz val="12"/>
       <color rgb="FFFF0000"/>
       <name val="Aptos Narrow (Body)"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FFFFFF00"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -765,11 +740,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -777,7 +752,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -789,15 +764,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -806,10 +780,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1155,7 +1128,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08157DB4-050D-DB49-BEDF-9CEE3097D5D6}">
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.5" customWidth="1"/>
@@ -1165,294 +1138,263 @@
     <col min="6" max="6" width="18.5" customWidth="1"/>
     <col min="7" max="7" width="24" customWidth="1"/>
     <col min="8" max="8" width="22.1640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="26.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+    <row r="1" spans="1:8" ht="19" x14ac:dyDescent="0.25">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
-        <v>50</v>
-      </c>
-      <c r="C1" s="13" t="s">
+      <c r="B1" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="C1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="F1" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="G1" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="13" t="s">
+      <c r="H1" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="13" t="s">
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="I2" s="12"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="B3" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B4" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B4" s="14" t="s">
+      <c r="C4" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" s="20" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="H4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="G5" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="H5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B6" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="F6" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="G6" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="H6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B7" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>127</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="F7" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="G7" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="H7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B8" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="E8" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="F8" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="H8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B9" t="s">
+        <v>43</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="F9" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="H9" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B10" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C10" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="F10" s="13" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="C11" s="13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="C12" s="21"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B14" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B15" t="s">
+        <v>10</v>
+      </c>
+      <c r="C15" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D15" s="19" t="s">
+        <v>23</v>
+      </c>
+      <c r="E15" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="G15" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="H15" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B16" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D16" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="22" t="s">
-        <v>15</v>
-      </c>
-      <c r="F4" s="14" t="s">
+    </row>
+    <row r="17" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B17" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="14" t="s">
+      <c r="C17" s="4"/>
+      <c r="D17" s="13" t="s">
         <v>13</v>
-      </c>
-      <c r="H4" t="s">
-        <v>36</v>
-      </c>
-      <c r="I4" s="20" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="E5" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="G5" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="H5" t="s">
-        <v>37</v>
-      </c>
-      <c r="I5" s="20" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B6" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6" s="14" t="s">
-        <v>134</v>
-      </c>
-      <c r="E6" s="14" t="s">
-        <v>109</v>
-      </c>
-      <c r="F6" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="G6" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="H6" t="s">
-        <v>38</v>
-      </c>
-      <c r="I6" s="20" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B7" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="C7" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D7" s="14" t="s">
-        <v>133</v>
-      </c>
-      <c r="E7" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="F7" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="G7" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="H7" t="s">
-        <v>39</v>
-      </c>
-      <c r="I7" s="20" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B8" s="14" t="s">
-        <v>48</v>
-      </c>
-      <c r="C8" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="E8" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="F8" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="H8" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B9" t="s">
-        <v>49</v>
-      </c>
-      <c r="C9" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="F9" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="H9" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B10" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="F10" s="14" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C11" s="14" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C12" s="23"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B14" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="I14" s="3" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B15" t="s">
-        <v>11</v>
-      </c>
-      <c r="C15" t="s">
-        <v>14</v>
-      </c>
-      <c r="D15" s="21" t="s">
-        <v>25</v>
-      </c>
-      <c r="E15" t="s">
-        <v>14</v>
-      </c>
-      <c r="F15" t="s">
-        <v>14</v>
-      </c>
-      <c r="G15" t="s">
-        <v>14</v>
-      </c>
-      <c r="H15" t="s">
-        <v>14</v>
-      </c>
-      <c r="I15" s="16" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B16" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C16" t="s">
-        <v>20</v>
-      </c>
-      <c r="D16" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B17" t="s">
-        <v>14</v>
-      </c>
-      <c r="C17" s="4"/>
-      <c r="D17" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.2">
@@ -1477,7 +1419,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B1" s="11" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="C1" s="11"/>
       <c r="D1" s="11"/>
@@ -1485,19 +1427,19 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="F2" s="5"/>
     </row>
@@ -1506,16 +1448,16 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C3" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D3">
         <v>20</v>
       </c>
       <c r="E3" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -1523,10 +1465,10 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="C4" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D4">
         <v>50</v>
@@ -1537,10 +1479,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="C5" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D5">
         <v>50</v>
@@ -1551,16 +1493,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="C6" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D6">
         <v>100</v>
       </c>
       <c r="E6" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -1568,10 +1510,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="C7" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D7">
         <v>100</v>
@@ -1582,10 +1524,10 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="C8" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D8">
         <v>15</v>
@@ -1596,10 +1538,10 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="C9" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D9">
         <v>5</v>
@@ -1610,10 +1552,10 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="C10" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D10">
         <v>15</v>
@@ -1624,10 +1566,10 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="C11" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D11">
         <v>100</v>
@@ -1638,10 +1580,10 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="C12" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="D12">
         <v>1</v>
@@ -1652,10 +1594,10 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="C13" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -1663,15 +1605,15 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="C14" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B17" s="11" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="C17" s="11"/>
       <c r="D17" s="11"/>
@@ -1679,19 +1621,19 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
@@ -1699,16 +1641,16 @@
         <v>1</v>
       </c>
       <c r="B19" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C19" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D19">
         <v>20</v>
       </c>
       <c r="E19" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
@@ -1716,16 +1658,16 @@
         <v>2</v>
       </c>
       <c r="B20" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="C20" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D20">
         <v>20</v>
       </c>
       <c r="E20" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
@@ -1733,10 +1675,10 @@
         <v>3</v>
       </c>
       <c r="B21" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="C21" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
@@ -1744,10 +1686,10 @@
         <v>4</v>
       </c>
       <c r="B22" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="C22" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D22">
         <v>10</v>
@@ -1758,10 +1700,10 @@
         <v>5</v>
       </c>
       <c r="B23" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="C23" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D23">
         <v>5</v>
@@ -1772,10 +1714,10 @@
         <v>6</v>
       </c>
       <c r="B24" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="C24" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D24">
         <v>200</v>
@@ -1786,10 +1728,10 @@
         <v>7</v>
       </c>
       <c r="B25" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="C25" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D25">
         <v>50</v>
@@ -1800,10 +1742,10 @@
         <v>8</v>
       </c>
       <c r="B26" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="C26" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D26">
         <v>15</v>
@@ -1814,10 +1756,10 @@
         <v>9</v>
       </c>
       <c r="B27" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="C27" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D27">
         <v>15</v>
@@ -1828,10 +1770,10 @@
         <v>10</v>
       </c>
       <c r="B28" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="C28" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D28">
         <v>50</v>
@@ -1842,10 +1784,10 @@
         <v>11</v>
       </c>
       <c r="B29" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="C29" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D29">
         <v>15</v>
@@ -1856,10 +1798,10 @@
         <v>12</v>
       </c>
       <c r="B30" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="C30" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D30">
         <v>15</v>
@@ -1870,10 +1812,10 @@
         <v>13</v>
       </c>
       <c r="B31" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="C31" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D31">
         <v>50</v>
@@ -1884,10 +1826,10 @@
         <v>14</v>
       </c>
       <c r="B32" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="C32" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D32">
         <v>20</v>
@@ -1900,7 +1842,7 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B35" s="11" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="C35" s="11"/>
       <c r="D35" s="11"/>
@@ -1908,19 +1850,19 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
@@ -1928,16 +1870,16 @@
         <v>1</v>
       </c>
       <c r="B37" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C37" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D37">
         <v>20</v>
       </c>
       <c r="E37" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
@@ -1945,16 +1887,16 @@
         <v>2</v>
       </c>
       <c r="B38" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="C38" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D38">
         <v>20</v>
       </c>
       <c r="E38" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
@@ -1962,10 +1904,10 @@
         <v>3</v>
       </c>
       <c r="B39" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="C39" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D39">
         <v>50</v>
@@ -1976,10 +1918,10 @@
         <v>4</v>
       </c>
       <c r="B40" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="C40" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D40">
         <v>50</v>
@@ -1990,10 +1932,10 @@
         <v>5</v>
       </c>
       <c r="B41" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="C41" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
@@ -2001,10 +1943,10 @@
         <v>6</v>
       </c>
       <c r="B42" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="C42" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="D42">
         <v>5</v>
@@ -2015,10 +1957,10 @@
         <v>7</v>
       </c>
       <c r="B43" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="C43" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D43">
         <v>200</v>
@@ -2029,10 +1971,10 @@
         <v>8</v>
       </c>
       <c r="B44" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="C44" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D44">
         <v>100</v>
@@ -2040,7 +1982,7 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B47" s="11" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="C47" s="11"/>
       <c r="D47" s="11"/>
@@ -2048,19 +1990,19 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.2">
@@ -2068,16 +2010,16 @@
         <v>1</v>
       </c>
       <c r="B49" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C49" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D49">
         <v>20</v>
       </c>
       <c r="E49" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.2">
@@ -2085,16 +2027,16 @@
         <v>2</v>
       </c>
       <c r="B50" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="C50" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D50">
         <v>20</v>
       </c>
       <c r="E50" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.2">
@@ -2102,10 +2044,10 @@
         <v>3</v>
       </c>
       <c r="B51" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="C51" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D51">
         <v>50</v>
@@ -2116,10 +2058,10 @@
         <v>4</v>
       </c>
       <c r="B52" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="C52" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.2">
@@ -2127,15 +2069,15 @@
         <v>5</v>
       </c>
       <c r="B53" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="C53" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B56" s="11" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="C56" s="11"/>
       <c r="D56" s="11"/>
@@ -2143,19 +2085,19 @@
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A57" s="2" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="B57" s="7" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.2">
@@ -2163,16 +2105,16 @@
         <v>1</v>
       </c>
       <c r="B58" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C58" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D58">
         <v>20</v>
       </c>
       <c r="E58" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.2">
@@ -2180,16 +2122,16 @@
         <v>2</v>
       </c>
       <c r="B59" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="C59" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D59">
         <v>20</v>
       </c>
       <c r="E59" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.2">
@@ -2197,10 +2139,10 @@
         <v>3</v>
       </c>
       <c r="B60" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="C60" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="D60">
         <v>50</v>
@@ -2211,10 +2153,10 @@
         <v>4</v>
       </c>
       <c r="B61" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="C61" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D61">
         <v>50</v>
@@ -2225,10 +2167,10 @@
         <v>5</v>
       </c>
       <c r="B62" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="C62" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="D62">
         <v>200</v>
@@ -2239,10 +2181,10 @@
         <v>6</v>
       </c>
       <c r="B63" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="C63" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="D63">
         <v>100</v>
@@ -2250,7 +2192,7 @@
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B65" s="11" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="C65" s="11"/>
       <c r="D65" s="11"/>
@@ -2258,19 +2200,19 @@
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="B66" s="7" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="C66" s="7" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.2">
@@ -2278,16 +2220,16 @@
         <v>1</v>
       </c>
       <c r="B67" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C67" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D67">
         <v>20</v>
       </c>
       <c r="E67" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.2">
@@ -2295,16 +2237,16 @@
         <v>2</v>
       </c>
       <c r="B68" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="C68" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D68">
         <v>50</v>
       </c>
       <c r="E68" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.2">
@@ -2312,10 +2254,10 @@
         <v>3</v>
       </c>
       <c r="B69" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="C69" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D69">
         <v>50</v>
@@ -2326,10 +2268,10 @@
         <v>4</v>
       </c>
       <c r="B70" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="C70" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D70">
         <v>50</v>
@@ -2340,10 +2282,10 @@
         <v>5</v>
       </c>
       <c r="B71" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="C71" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D71">
         <v>200</v>
@@ -2354,10 +2296,10 @@
         <v>6</v>
       </c>
       <c r="B72" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="C72" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D72">
         <v>20</v>
@@ -2368,10 +2310,10 @@
         <v>7</v>
       </c>
       <c r="B73" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="C73" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.2">
@@ -2379,15 +2321,15 @@
         <v>8</v>
       </c>
       <c r="B74" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="C74" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B77" s="11" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="C77" s="11"/>
       <c r="D77" s="11"/>
@@ -2395,19 +2337,19 @@
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A78" s="2" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="B78" s="7" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="C78" s="7" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.2">
@@ -2415,16 +2357,16 @@
         <v>1</v>
       </c>
       <c r="B79" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C79" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D79">
         <v>20</v>
       </c>
       <c r="E79" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.2">
@@ -2432,16 +2374,16 @@
         <v>2</v>
       </c>
       <c r="B80" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="C80" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D80">
         <v>20</v>
       </c>
       <c r="E80" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.2">
@@ -2449,16 +2391,16 @@
         <v>3</v>
       </c>
       <c r="B81" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="C81" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D81">
         <v>20</v>
       </c>
       <c r="E81" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.2">
@@ -2466,10 +2408,10 @@
         <v>4</v>
       </c>
       <c r="B82" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="C82" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="D82">
         <v>15</v>
@@ -2480,10 +2422,10 @@
         <v>5</v>
       </c>
       <c r="B83" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="C83" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="D83">
         <v>20</v>
@@ -2494,10 +2436,10 @@
         <v>6</v>
       </c>
       <c r="B84" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="C84" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D84">
         <v>200</v>
@@ -2508,10 +2450,10 @@
         <v>7</v>
       </c>
       <c r="B85" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="C85" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D85">
         <v>20</v>
@@ -2522,10 +2464,10 @@
         <v>8</v>
       </c>
       <c r="B86" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="C86" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.2">
@@ -2533,15 +2475,15 @@
         <v>9</v>
       </c>
       <c r="B87" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="C87" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B90" s="11" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="C90" s="11"/>
       <c r="D90" s="11"/>
@@ -2549,19 +2491,19 @@
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A91" s="2" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="B91" s="7" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="C91" s="7" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.2">
@@ -2569,16 +2511,16 @@
         <v>1</v>
       </c>
       <c r="B92" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C92" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D92">
         <v>20</v>
       </c>
       <c r="E92" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.2">
@@ -2586,16 +2528,16 @@
         <v>2</v>
       </c>
       <c r="B93" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="C93" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D93">
         <v>20</v>
       </c>
       <c r="E93" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.2">
@@ -2603,16 +2545,16 @@
         <v>3</v>
       </c>
       <c r="B94" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="C94" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D94">
         <v>20</v>
       </c>
       <c r="E94" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.2">
@@ -2620,16 +2562,16 @@
         <v>4</v>
       </c>
       <c r="B95" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="C95" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D95">
         <v>100</v>
       </c>
       <c r="E95" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.2">
@@ -2637,10 +2579,10 @@
         <v>5</v>
       </c>
       <c r="B96" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="C96" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D96">
         <v>500</v>
@@ -2651,10 +2593,10 @@
         <v>6</v>
       </c>
       <c r="B97" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="C97" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D97">
         <v>100</v>
@@ -2665,10 +2607,10 @@
         <v>7</v>
       </c>
       <c r="B98" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="C98" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D98">
         <v>1000</v>
@@ -2679,10 +2621,10 @@
         <v>8</v>
       </c>
       <c r="B99" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="C99" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D99">
         <v>5000</v>
@@ -2693,10 +2635,10 @@
         <v>9</v>
       </c>
       <c r="B100" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="C100" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D100">
         <v>5000</v>
@@ -2707,10 +2649,10 @@
         <v>10</v>
       </c>
       <c r="B101" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="C101" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.2">
@@ -2718,10 +2660,10 @@
         <v>11</v>
       </c>
       <c r="B102" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="C102" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.2">
@@ -2729,10 +2671,10 @@
         <v>12</v>
       </c>
       <c r="B103" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="C103" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.2">
@@ -2740,15 +2682,15 @@
         <v>13</v>
       </c>
       <c r="B104" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="C104" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B107" s="11" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="C107" s="11"/>
       <c r="D107" s="11"/>
@@ -2756,19 +2698,19 @@
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A108" s="2" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="B108" s="7" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="C108" s="7" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="E108" s="2" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.2">
@@ -2776,16 +2718,16 @@
         <v>1</v>
       </c>
       <c r="B109" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C109" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D109">
         <v>20</v>
       </c>
       <c r="E109" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.2">
@@ -2793,16 +2735,16 @@
         <v>2</v>
       </c>
       <c r="B110" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="C110" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D110">
         <v>20</v>
       </c>
-      <c r="E110" s="16" t="s">
-        <v>80</v>
+      <c r="E110" s="15" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.2">
@@ -2810,16 +2752,16 @@
         <v>3</v>
       </c>
       <c r="B111" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="C111" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D111">
         <v>20</v>
       </c>
       <c r="E111" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.2">
@@ -2827,10 +2769,10 @@
         <v>4</v>
       </c>
       <c r="B112" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="C112" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D112">
         <v>200</v>
@@ -2841,10 +2783,10 @@
         <v>5</v>
       </c>
       <c r="B113" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="C113" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D113">
         <v>500</v>
@@ -2855,10 +2797,10 @@
         <v>6</v>
       </c>
       <c r="B114" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="C114" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D114">
         <v>500</v>
@@ -2869,10 +2811,10 @@
         <v>7</v>
       </c>
       <c r="B115" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="C115" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.2">
@@ -2880,10 +2822,10 @@
         <v>8</v>
       </c>
       <c r="B116" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="C116" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.2">
@@ -2891,10 +2833,10 @@
         <v>9</v>
       </c>
       <c r="B117" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="C117" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.2">
@@ -2902,10 +2844,10 @@
         <v>10</v>
       </c>
       <c r="B118" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="C118" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.2">
@@ -2913,10 +2855,10 @@
         <v>11</v>
       </c>
       <c r="B119" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="C119" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D119">
         <v>2000</v>
@@ -2927,10 +2869,10 @@
         <v>12</v>
       </c>
       <c r="B120" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="C120" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D120">
         <v>200</v>
@@ -2938,7 +2880,7 @@
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B123" s="11" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="C123" s="11"/>
       <c r="D123" s="11"/>
@@ -2946,19 +2888,19 @@
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A124" s="2" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="B124" s="7" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="C124" s="7" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="D124" s="2" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="E124" s="2" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.2">
@@ -2966,16 +2908,16 @@
         <v>1</v>
       </c>
       <c r="B125" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C125" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D125">
         <v>20</v>
       </c>
       <c r="E125" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.2">
@@ -2983,16 +2925,16 @@
         <v>2</v>
       </c>
       <c r="B126" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="C126" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D126">
         <v>20</v>
       </c>
       <c r="E126" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.2">
@@ -3000,10 +2942,10 @@
         <v>3</v>
       </c>
       <c r="B127" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="C127" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D127">
         <v>100</v>
@@ -3014,10 +2956,10 @@
         <v>4</v>
       </c>
       <c r="B128" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="C128" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D128">
         <v>200</v>
@@ -3028,10 +2970,10 @@
         <v>5</v>
       </c>
       <c r="B129" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="C129" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D129">
         <v>200</v>
@@ -3041,79 +2983,79 @@
       <c r="A130">
         <v>6</v>
       </c>
-      <c r="B130" s="18" t="s">
-        <v>150</v>
-      </c>
-      <c r="C130" s="19" t="s">
-        <v>73</v>
-      </c>
-      <c r="D130" s="25" t="s">
-        <v>73</v>
+      <c r="B130" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="C130" s="18" t="s">
+        <v>67</v>
+      </c>
+      <c r="D130" s="23" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A131">
         <v>7</v>
       </c>
-      <c r="B131" s="19" t="s">
-        <v>159</v>
-      </c>
-      <c r="C131" s="19" t="s">
-        <v>73</v>
-      </c>
-      <c r="D131" s="25" t="s">
-        <v>73</v>
+      <c r="B131" s="18" t="s">
+        <v>153</v>
+      </c>
+      <c r="C131" s="18" t="s">
+        <v>67</v>
+      </c>
+      <c r="D131" s="23" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A132">
         <v>8</v>
       </c>
-      <c r="B132" s="19" t="s">
-        <v>160</v>
-      </c>
-      <c r="C132" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="D132" s="25" t="s">
-        <v>55</v>
+      <c r="B132" s="18" t="s">
+        <v>154</v>
+      </c>
+      <c r="C132" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="D132" s="23" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A133" s="25">
+      <c r="A133" s="23">
         <v>9</v>
       </c>
       <c r="B133" s="8" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="C133" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="D133" s="25" t="s">
-        <v>55</v>
-      </c>
-      <c r="E133" s="24"/>
-      <c r="F133" s="24"/>
+        <v>49</v>
+      </c>
+      <c r="D133" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="E133" s="22"/>
+      <c r="F133" s="22"/>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A134" s="24"/>
+      <c r="A134" s="22"/>
       <c r="B134" s="8"/>
       <c r="C134" s="8"/>
-      <c r="D134" s="24"/>
-      <c r="E134" s="24"/>
-      <c r="F134" s="24"/>
+      <c r="D134" s="22"/>
+      <c r="E134" s="22"/>
+      <c r="F134" s="22"/>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A135" s="24"/>
+      <c r="A135" s="22"/>
       <c r="B135" s="8"/>
       <c r="C135" s="8"/>
-      <c r="D135" s="24"/>
-      <c r="E135" s="24"/>
-      <c r="F135" s="24"/>
+      <c r="D135" s="22"/>
+      <c r="E135" s="22"/>
+      <c r="F135" s="22"/>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B136" s="11" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="C136" s="11"/>
       <c r="D136" s="11"/>
@@ -3121,19 +3063,19 @@
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A137" s="2" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="B137" s="7" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="C137" s="7" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="D137" s="2" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="E137" s="2" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.2">
@@ -3141,16 +3083,16 @@
         <v>1</v>
       </c>
       <c r="B138" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C138" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D138">
         <v>20</v>
       </c>
       <c r="E138" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.2">
@@ -3158,16 +3100,16 @@
         <v>2</v>
       </c>
       <c r="B139" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="C139" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D139">
         <v>20</v>
       </c>
       <c r="E139" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.2">
@@ -3175,16 +3117,16 @@
         <v>3</v>
       </c>
       <c r="B140" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="C140" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D140">
         <v>20</v>
       </c>
       <c r="E140" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.2">
@@ -3192,10 +3134,10 @@
         <v>4</v>
       </c>
       <c r="B141" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="C141" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.2">
@@ -3203,10 +3145,10 @@
         <v>5</v>
       </c>
       <c r="B142" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="C142" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="D142">
         <v>7</v>
@@ -3217,10 +3159,10 @@
         <v>6</v>
       </c>
       <c r="B143" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="C143" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D143">
         <v>100</v>
@@ -3231,16 +3173,16 @@
         <v>7</v>
       </c>
       <c r="B144" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="C144" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D144">
         <v>20</v>
       </c>
       <c r="E144" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.2">
@@ -3248,10 +3190,10 @@
         <v>8</v>
       </c>
       <c r="B145" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="C145" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D145">
         <v>100</v>
@@ -3262,10 +3204,10 @@
         <v>9</v>
       </c>
       <c r="B146" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="C146" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.2">
@@ -3273,10 +3215,10 @@
         <v>10</v>
       </c>
       <c r="B147" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="C147" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.2">
@@ -3284,10 +3226,10 @@
         <v>11</v>
       </c>
       <c r="B148" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="C148" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.2">
@@ -3295,15 +3237,15 @@
         <v>12</v>
       </c>
       <c r="B149" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="C149" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B152" s="11" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="C152" s="11"/>
       <c r="D152" s="11"/>
@@ -3311,19 +3253,19 @@
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A153" s="2" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="B153" s="7" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="C153" s="7" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="D153" s="2" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="E153" s="2" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.2">
@@ -3331,16 +3273,16 @@
         <v>1</v>
       </c>
       <c r="B154" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C154" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D154">
         <v>20</v>
       </c>
       <c r="E154" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.2">
@@ -3348,16 +3290,16 @@
         <v>2</v>
       </c>
       <c r="B155" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="C155" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D155">
         <v>20</v>
       </c>
       <c r="E155" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
     </row>
     <row r="156" spans="1:5" x14ac:dyDescent="0.2">
@@ -3365,16 +3307,16 @@
         <v>3</v>
       </c>
       <c r="B156" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="C156" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D156">
         <v>20</v>
       </c>
       <c r="E156" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
     </row>
     <row r="157" spans="1:5" x14ac:dyDescent="0.2">
@@ -3382,16 +3324,16 @@
         <v>4</v>
       </c>
       <c r="B157" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="C157" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D157">
         <v>20</v>
       </c>
       <c r="E157" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
     </row>
     <row r="158" spans="1:5" x14ac:dyDescent="0.2">
@@ -3399,16 +3341,16 @@
         <v>5</v>
       </c>
       <c r="B158" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="C158" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D158">
         <v>20</v>
       </c>
       <c r="E158" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
     </row>
     <row r="159" spans="1:5" x14ac:dyDescent="0.2">
@@ -3416,10 +3358,10 @@
         <v>6</v>
       </c>
       <c r="B159" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="C159" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D159">
         <v>500</v>
@@ -3430,10 +3372,10 @@
         <v>7</v>
       </c>
       <c r="B160" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="C160" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D160">
         <v>100</v>
@@ -3444,10 +3386,10 @@
         <v>8</v>
       </c>
       <c r="B161" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="C161" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
     </row>
     <row r="162" spans="1:5" x14ac:dyDescent="0.2">
@@ -3455,10 +3397,10 @@
         <v>9</v>
       </c>
       <c r="B162" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="C162" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="D162">
         <v>7</v>
@@ -3469,10 +3411,10 @@
         <v>10</v>
       </c>
       <c r="B163" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="C163" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="D163">
         <v>7</v>
@@ -3483,18 +3425,18 @@
         <v>11</v>
       </c>
       <c r="B164" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="C164" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B165" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="C165" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D165">
         <v>2000</v>
@@ -3502,10 +3444,10 @@
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B166" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="C166" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D166">
         <v>2000</v>
@@ -3516,10 +3458,10 @@
         <v>12</v>
       </c>
       <c r="B167" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="C167" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
     </row>
     <row r="168" spans="1:5" x14ac:dyDescent="0.2">
@@ -3527,10 +3469,10 @@
         <v>13</v>
       </c>
       <c r="B168" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="C168" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
     </row>
     <row r="169" spans="1:5" x14ac:dyDescent="0.2">
@@ -3538,15 +3480,15 @@
         <v>14</v>
       </c>
       <c r="B169" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="C169" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B172" s="11" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="C172" s="11"/>
       <c r="D172" s="11"/>
@@ -3554,19 +3496,19 @@
     </row>
     <row r="173" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A173" s="2" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="B173" s="7" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="C173" s="7" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="D173" s="2" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="E173" s="2" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
     </row>
     <row r="174" spans="1:5" x14ac:dyDescent="0.2">
@@ -3574,16 +3516,16 @@
         <v>1</v>
       </c>
       <c r="B174" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C174" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D174">
         <v>20</v>
       </c>
       <c r="E174" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
     </row>
     <row r="175" spans="1:5" x14ac:dyDescent="0.2">
@@ -3591,16 +3533,16 @@
         <v>2</v>
       </c>
       <c r="B175" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="C175" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D175">
         <v>20</v>
       </c>
       <c r="E175" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
     </row>
     <row r="176" spans="1:5" x14ac:dyDescent="0.2">
@@ -3608,16 +3550,16 @@
         <v>3</v>
       </c>
       <c r="B176" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="C176" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D176">
         <v>20</v>
       </c>
       <c r="E176" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
     </row>
     <row r="177" spans="1:5" x14ac:dyDescent="0.2">
@@ -3625,16 +3567,16 @@
         <v>4</v>
       </c>
       <c r="B177" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="C177" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D177">
         <v>20</v>
       </c>
       <c r="E177" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
     </row>
     <row r="178" spans="1:5" x14ac:dyDescent="0.2">
@@ -3642,10 +3584,10 @@
         <v>5</v>
       </c>
       <c r="B178" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="C178" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D178">
         <v>7</v>
@@ -3656,10 +3598,10 @@
         <v>6</v>
       </c>
       <c r="B179" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="C179" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D179">
         <v>100</v>
@@ -3670,10 +3612,10 @@
         <v>7</v>
       </c>
       <c r="B180" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="C180" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D180">
         <v>20</v>
@@ -3684,10 +3626,10 @@
         <v>8</v>
       </c>
       <c r="B181" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="C181" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D181">
         <v>100</v>
@@ -3698,10 +3640,10 @@
         <v>9</v>
       </c>
       <c r="B182" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="C182" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="D182">
         <v>7</v>
@@ -3712,10 +3654,10 @@
         <v>10</v>
       </c>
       <c r="B183" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="C183" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D183">
         <v>20</v>
@@ -3726,13 +3668,13 @@
         <v>11</v>
       </c>
       <c r="B184" t="s">
+        <v>176</v>
+      </c>
+      <c r="C184" t="s">
+        <v>61</v>
+      </c>
+      <c r="D184" t="s">
         <v>182</v>
-      </c>
-      <c r="C184" t="s">
-        <v>67</v>
-      </c>
-      <c r="D184" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="185" spans="1:5" x14ac:dyDescent="0.2">
@@ -3740,10 +3682,10 @@
         <v>12</v>
       </c>
       <c r="B185" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="C185" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
     </row>
     <row r="186" spans="1:5" x14ac:dyDescent="0.2">
@@ -3751,10 +3693,10 @@
         <v>13</v>
       </c>
       <c r="B186" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="C186" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -3787,7 +3729,7 @@
   <sheetData>
     <row r="3" spans="1:24" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="9" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="B3" s="9"/>
       <c r="C3" s="9"/>
@@ -3800,7 +3742,7 @@
       <c r="J3" s="9"/>
       <c r="K3" s="9"/>
       <c r="M3" s="10" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="N3" s="10"/>
       <c r="O3" s="10"/>
@@ -4496,15 +4438,15 @@
       <c r="X32" s="10"/>
     </row>
     <row r="33" spans="1:24" ht="24" x14ac:dyDescent="0.3">
-      <c r="A33" s="17" t="s">
-        <v>99</v>
-      </c>
-      <c r="B33" s="17"/>
-      <c r="C33" s="17"/>
-      <c r="D33" s="17"/>
-      <c r="E33" s="17"/>
-      <c r="F33" s="17"/>
-      <c r="G33" s="17"/>
+      <c r="A33" s="16" t="s">
+        <v>93</v>
+      </c>
+      <c r="B33" s="16"/>
+      <c r="C33" s="16"/>
+      <c r="D33" s="16"/>
+      <c r="E33" s="16"/>
+      <c r="F33" s="16"/>
+      <c r="G33" s="16"/>
       <c r="M33" s="10"/>
       <c r="N33" s="10"/>
       <c r="O33" s="10"/>
@@ -4522,8 +4464,8 @@
       <c r="A34">
         <v>1</v>
       </c>
-      <c r="B34" s="14" t="s">
-        <v>100</v>
+      <c r="B34" s="13" t="s">
+        <v>94</v>
       </c>
       <c r="M34" s="10"/>
       <c r="N34" s="10"/>
@@ -4542,8 +4484,8 @@
       <c r="A35">
         <v>2</v>
       </c>
-      <c r="B35" s="14" t="s">
-        <v>101</v>
+      <c r="B35" s="13" t="s">
+        <v>95</v>
       </c>
       <c r="M35" s="10"/>
       <c r="N35" s="10"/>
@@ -4563,7 +4505,7 @@
         <v>3</v>
       </c>
       <c r="B36" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="M36" s="10"/>
       <c r="N36" s="10"/>
@@ -4583,7 +4525,7 @@
         <v>4</v>
       </c>
       <c r="B37" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="M37" s="10"/>
       <c r="N37" s="10"/>
@@ -4603,7 +4545,7 @@
         <v>5</v>
       </c>
       <c r="B38" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="M38" s="10"/>
       <c r="N38" s="10"/>
@@ -4622,12 +4564,12 @@
       <c r="A39">
         <v>6</v>
       </c>
-      <c r="B39" s="14" t="s">
-        <v>106</v>
-      </c>
-      <c r="C39" s="15"/>
-      <c r="D39" s="15"/>
-      <c r="E39" s="15"/>
+      <c r="B39" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="C39" s="14"/>
+      <c r="D39" s="14"/>
+      <c r="E39" s="14"/>
       <c r="M39" s="10"/>
       <c r="N39" s="10"/>
       <c r="O39" s="10"/>
@@ -4645,10 +4587,10 @@
       <c r="A40">
         <v>7</v>
       </c>
-      <c r="B40" s="14" t="s">
-        <v>107</v>
-      </c>
-      <c r="C40" s="15"/>
+      <c r="B40" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="C40" s="14"/>
       <c r="M40" s="10"/>
       <c r="N40" s="10"/>
       <c r="O40" s="10"/>
@@ -4667,7 +4609,7 @@
         <v>8</v>
       </c>
       <c r="B41" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="M41" s="10"/>
       <c r="N41" s="10"/>
@@ -4687,7 +4629,7 @@
         <v>9</v>
       </c>
       <c r="B42" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
     </row>
     <row r="43" spans="1:24" x14ac:dyDescent="0.2">
@@ -4695,7 +4637,7 @@
         <v>10</v>
       </c>
       <c r="B43" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add billing history functionality in patient role
</commit_message>
<xml_diff>
--- a/CareOS-Hospital_ERP_System.xlsx
+++ b/CareOS-Hospital_ERP_System.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hetlimbani/Desktop/Self_Learning/CareOS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC734C12-BE7D-E641-8748-CEAF5C4C6E40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D961B95B-FBA4-2B4E-ABBE-F8AD747F7BFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="680" windowWidth="34200" windowHeight="19420" xr2:uid="{3BCF7A51-5C29-EE4C-8BC3-93CAF12DE1EA}"/>
+    <workbookView xWindow="-20" yWindow="680" windowWidth="34200" windowHeight="19420" activeTab="1" xr2:uid="{3BCF7A51-5C29-EE4C-8BC3-93CAF12DE1EA}"/>
   </bookViews>
   <sheets>
     <sheet name="ERP System" sheetId="1" r:id="rId1"/>
     <sheet name="Schema" sheetId="2" r:id="rId2"/>
-    <sheet name="Usefull" sheetId="3" r:id="rId3"/>
+    <sheet name="Bugs" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="577" uniqueCount="200">
   <si>
     <t>Total Roles</t>
   </si>
@@ -283,56 +283,6 @@
     <t>update_at</t>
   </si>
   <si>
-    <t>12. Ambulance Schema
-import mongoose from "mongoose";
-const AmbulanceSchema = new mongoose.Schema({
-    driverName:String,
-    vehicleNumber:String,
-    currentLocation:{
-        lat:Number,
-        lng:Number
-    },
-    status:{
-        type:String,
-        enum:[
-            "available",
-            "busy",
-            "maintenance"
-        ],
-        default:"available"
-    }
-},
-{timestamps:true});
-export default mongoose.model("Ambulance",AmbulanceSchema);</t>
-  </si>
-  <si>
-    <t>13. Emergency Request Schema
-import mongoose from "mongoose";
-const EmergencyRequestSchema = new mongoose.Schema({
-    patientId:{
-        type:mongoose.Schema.Types.ObjectId,
-        ref:"Patient"
-    },
-    ambulanceId:{
-        type:mongoose.Schema.Types.ObjectId,
-        ref:"Ambulance"
-    },
-    pickupLocation:String,
-    destination:String,
-    status:{
-        type:String,
-        enum:[
-            "requested",
-            "assigned",
-            "completed"
-        ],
-        default:"requested"
-    }
-},
-{timestamps:true});
-export default mongoose.model("EmergencyRequest",EmergencyRequestSchema);</t>
-  </si>
-  <si>
     <t>result</t>
   </si>
   <si>
@@ -429,12 +379,6 @@
     <t>User Collection Schema</t>
   </si>
   <si>
-    <t>Patient  Collection Schema</t>
-  </si>
-  <si>
-    <t>Doctor Collection Schema</t>
-  </si>
-  <si>
     <t>slots</t>
   </si>
   <si>
@@ -634,13 +578,76 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>Admissions Collection Schema</t>
+  </si>
+  <si>
+    <t>patientName</t>
+  </si>
+  <si>
+    <t>nurseIds</t>
+  </si>
+  <si>
+    <t>bedId</t>
+  </si>
+  <si>
+    <t>roomType</t>
+  </si>
+  <si>
+    <t>admittedAt</t>
+  </si>
+  <si>
+    <t>dischargeEligibleAt</t>
+  </si>
+  <si>
+    <t>big_integer[]</t>
+  </si>
+  <si>
+    <t>Doctor Profile Collection Schema</t>
+  </si>
+  <si>
+    <t>Patient Profile Collection Schema</t>
+  </si>
+  <si>
+    <t>Wardbeds Collection Schema</t>
+  </si>
+  <si>
+    <t>bedNumber</t>
+  </si>
+  <si>
+    <t>currentAdmissionId</t>
+  </si>
+  <si>
+    <t>Treatment Plans Collection Schema</t>
+  </si>
+  <si>
+    <t>admissionId</t>
+  </si>
+  <si>
+    <t>treatmentHeading</t>
+  </si>
+  <si>
+    <t>totalPlanCost</t>
+  </si>
+  <si>
+    <t>scheduledDate</t>
+  </si>
+  <si>
+    <t>scheduledTime</t>
+  </si>
+  <si>
+    <t>administrationStatus</t>
+  </si>
+  <si>
+    <t>clinicalNotes</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -701,8 +708,15 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -727,6 +741,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFBFBFBF"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -740,7 +760,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -758,22 +778,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -789,6 +799,26 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1131,38 +1161,38 @@
   <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.5" customWidth="1"/>
+    <col min="1" max="1" width="11.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="22.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="32.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="27.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.5" customWidth="1"/>
-    <col min="7" max="7" width="24" customWidth="1"/>
+    <col min="6" max="6" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.1640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="22.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="G1" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="12" t="s">
+      <c r="H1" s="10" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1193,22 +1223,22 @@
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="E4" s="20" t="s">
+      <c r="D4" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="F4" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="G4" s="13" t="s">
+      <c r="G4" s="11" t="s">
         <v>12</v>
       </c>
       <c r="H4" t="s">
@@ -1219,19 +1249,19 @@
       <c r="B5" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="C5" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="D5" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="E5" s="13" t="s">
+      <c r="E5" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="F5" s="13" t="s">
+      <c r="F5" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="G5" s="13" t="s">
+      <c r="G5" s="11" t="s">
         <v>31</v>
       </c>
       <c r="H5" t="s">
@@ -1239,22 +1269,22 @@
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="13" t="s">
-        <v>128</v>
-      </c>
-      <c r="E6" s="13" t="s">
-        <v>103</v>
-      </c>
-      <c r="F6" s="13" t="s">
+      <c r="D6" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="F6" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="G6" s="13" t="s">
+      <c r="G6" s="11" t="s">
         <v>32</v>
       </c>
       <c r="H6" t="s">
@@ -1262,22 +1292,22 @@
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B7" s="13" t="s">
-        <v>97</v>
-      </c>
-      <c r="C7" s="13" t="s">
+      <c r="B7" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="C7" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="13" t="s">
-        <v>127</v>
-      </c>
-      <c r="E7" s="13" t="s">
+      <c r="D7" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="E7" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="F7" s="13" t="s">
+      <c r="F7" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="G7" s="13" t="s">
+      <c r="G7" s="11" t="s">
         <v>33</v>
       </c>
       <c r="H7" t="s">
@@ -1285,16 +1315,16 @@
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B8" s="13" t="s">
+      <c r="B8" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="E8" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="F8" s="13" t="s">
+      <c r="F8" s="11" t="s">
         <v>29</v>
       </c>
       <c r="H8" t="s">
@@ -1305,10 +1335,10 @@
       <c r="B9" t="s">
         <v>43</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="F9" s="11" t="s">
         <v>30</v>
       </c>
       <c r="H9" t="s">
@@ -1316,23 +1346,23 @@
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B10" s="13" t="s">
+      <c r="B10" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="F10" s="13" t="s">
+      <c r="F10" s="11" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="11" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="C12" s="21"/>
+      <c r="C12" s="17"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="B14" s="3" t="s">
@@ -1361,19 +1391,19 @@
       <c r="B15" t="s">
         <v>10</v>
       </c>
-      <c r="C15" s="13" t="s">
+      <c r="C15" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="D15" s="19" t="s">
+      <c r="D15" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="E15" s="13" t="s">
+      <c r="E15" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="F15" s="13" t="s">
+      <c r="F15" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="G15" s="13" t="s">
+      <c r="G15" s="11" t="s">
         <v>13</v>
       </c>
       <c r="H15" t="s">
@@ -1389,11 +1419,11 @@
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B17" s="13" t="s">
+      <c r="B17" s="11" t="s">
         <v>13</v>
       </c>
       <c r="C17" s="4"/>
-      <c r="D17" s="13" t="s">
+      <c r="D17" s="11" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1407,23 +1437,23 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5186853C-8F41-E14D-BD0A-415B9ACDCBCD}">
-  <dimension ref="A1:F186"/>
+  <dimension ref="A1:F231"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="3.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="3.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B1" s="11" t="s">
-        <v>113</v>
-      </c>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
+      <c r="B1" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
@@ -1538,7 +1568,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C9" t="s">
         <v>49</v>
@@ -1580,7 +1610,7 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C12" t="s">
         <v>48</v>
@@ -1612,12 +1642,12 @@
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B17" s="11" t="s">
-        <v>114</v>
-      </c>
-      <c r="C17" s="11"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="11"/>
+      <c r="B17" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
@@ -1675,7 +1705,7 @@
         <v>3</v>
       </c>
       <c r="B21" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C21" t="s">
         <v>76</v>
@@ -1728,7 +1758,7 @@
         <v>7</v>
       </c>
       <c r="B25" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C25" t="s">
         <v>49</v>
@@ -1742,7 +1772,7 @@
         <v>8</v>
       </c>
       <c r="B26" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C26" t="s">
         <v>49</v>
@@ -1756,7 +1786,7 @@
         <v>9</v>
       </c>
       <c r="B27" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C27" t="s">
         <v>49</v>
@@ -1770,7 +1800,7 @@
         <v>10</v>
       </c>
       <c r="B28" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C28" t="s">
         <v>49</v>
@@ -1784,7 +1814,7 @@
         <v>11</v>
       </c>
       <c r="B29" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C29" t="s">
         <v>49</v>
@@ -1798,7 +1828,7 @@
         <v>12</v>
       </c>
       <c r="B30" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C30" t="s">
         <v>49</v>
@@ -1812,7 +1842,7 @@
         <v>13</v>
       </c>
       <c r="B31" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C31" t="s">
         <v>49</v>
@@ -1826,7 +1856,7 @@
         <v>14</v>
       </c>
       <c r="B32" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C32" t="s">
         <v>60</v>
@@ -1841,12 +1871,12 @@
       <c r="C34" s="6"/>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B35" s="11" t="s">
-        <v>115</v>
-      </c>
-      <c r="C35" s="11"/>
-      <c r="D35" s="11"/>
-      <c r="E35" s="11"/>
+      <c r="B35" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="C35" s="9"/>
+      <c r="D35" s="9"/>
+      <c r="E35" s="9"/>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
@@ -1932,7 +1962,7 @@
         <v>5</v>
       </c>
       <c r="B41" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C41" t="s">
         <v>76</v>
@@ -1943,7 +1973,7 @@
         <v>6</v>
       </c>
       <c r="B42" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C42" t="s">
         <v>67</v>
@@ -1957,7 +1987,7 @@
         <v>7</v>
       </c>
       <c r="B43" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C43" t="s">
         <v>49</v>
@@ -1971,7 +2001,7 @@
         <v>8</v>
       </c>
       <c r="B44" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C44" t="s">
         <v>49</v>
@@ -1981,12 +2011,12 @@
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B47" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="C47" s="11"/>
-      <c r="D47" s="11"/>
-      <c r="E47" s="11"/>
+      <c r="B47" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="C47" s="9"/>
+      <c r="D47" s="9"/>
+      <c r="E47" s="9"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
@@ -2044,10 +2074,10 @@
         <v>3</v>
       </c>
       <c r="B51" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C51" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D51">
         <v>50</v>
@@ -2076,12 +2106,12 @@
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B56" s="11" t="s">
-        <v>117</v>
-      </c>
-      <c r="C56" s="11"/>
-      <c r="D56" s="11"/>
-      <c r="E56" s="11"/>
+      <c r="B56" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="C56" s="9"/>
+      <c r="D56" s="9"/>
+      <c r="E56" s="9"/>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A57" s="2" t="s">
@@ -2153,10 +2183,10 @@
         <v>4</v>
       </c>
       <c r="B61" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="C61" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D61">
         <v>50</v>
@@ -2191,12 +2221,12 @@
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B65" s="11" t="s">
-        <v>123</v>
-      </c>
-      <c r="C65" s="11"/>
-      <c r="D65" s="11"/>
-      <c r="E65" s="11"/>
+      <c r="B65" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="C65" s="9"/>
+      <c r="D65" s="9"/>
+      <c r="E65" s="9"/>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
@@ -2237,7 +2267,7 @@
         <v>2</v>
       </c>
       <c r="B68" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="C68" t="s">
         <v>49</v>
@@ -2254,7 +2284,7 @@
         <v>3</v>
       </c>
       <c r="B69" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="C69" t="s">
         <v>49</v>
@@ -2282,7 +2312,7 @@
         <v>5</v>
       </c>
       <c r="B71" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C71" t="s">
         <v>49</v>
@@ -2296,10 +2326,10 @@
         <v>6</v>
       </c>
       <c r="B72" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C72" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D72">
         <v>20</v>
@@ -2328,12 +2358,12 @@
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B77" s="11" t="s">
-        <v>122</v>
-      </c>
-      <c r="C77" s="11"/>
-      <c r="D77" s="11"/>
-      <c r="E77" s="11"/>
+      <c r="B77" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="C77" s="9"/>
+      <c r="D77" s="9"/>
+      <c r="E77" s="9"/>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A78" s="2" t="s">
@@ -2422,10 +2452,10 @@
         <v>5</v>
       </c>
       <c r="B83" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C83" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="D83">
         <v>20</v>
@@ -2436,7 +2466,7 @@
         <v>6</v>
       </c>
       <c r="B84" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C84" t="s">
         <v>49</v>
@@ -2450,7 +2480,7 @@
         <v>7</v>
       </c>
       <c r="B85" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C85" t="s">
         <v>49</v>
@@ -2482,12 +2512,12 @@
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B90" s="11" t="s">
-        <v>130</v>
-      </c>
-      <c r="C90" s="11"/>
-      <c r="D90" s="11"/>
-      <c r="E90" s="11"/>
+      <c r="B90" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="C90" s="9"/>
+      <c r="D90" s="9"/>
+      <c r="E90" s="9"/>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A91" s="2" t="s">
@@ -2528,7 +2558,7 @@
         <v>2</v>
       </c>
       <c r="B93" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C93" t="s">
         <v>60</v>
@@ -2545,7 +2575,7 @@
         <v>3</v>
       </c>
       <c r="B94" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="C94" t="s">
         <v>60</v>
@@ -2562,7 +2592,7 @@
         <v>4</v>
       </c>
       <c r="B95" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C95" t="s">
         <v>49</v>
@@ -2579,7 +2609,7 @@
         <v>5</v>
       </c>
       <c r="B96" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C96" t="s">
         <v>49</v>
@@ -2593,7 +2623,7 @@
         <v>6</v>
       </c>
       <c r="B97" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C97" t="s">
         <v>49</v>
@@ -2635,7 +2665,7 @@
         <v>9</v>
       </c>
       <c r="B100" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C100" t="s">
         <v>49</v>
@@ -2649,10 +2679,10 @@
         <v>10</v>
       </c>
       <c r="B101" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="C101" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.2">
@@ -2660,10 +2690,10 @@
         <v>11</v>
       </c>
       <c r="B102" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="C102" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.2">
@@ -2689,12 +2719,12 @@
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B107" s="11" t="s">
-        <v>138</v>
-      </c>
-      <c r="C107" s="11"/>
-      <c r="D107" s="11"/>
-      <c r="E107" s="11"/>
+      <c r="B107" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="C107" s="9"/>
+      <c r="D107" s="9"/>
+      <c r="E107" s="9"/>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A108" s="2" t="s">
@@ -2735,7 +2765,7 @@
         <v>2</v>
       </c>
       <c r="B110" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="C110" t="s">
         <v>60</v>
@@ -2743,7 +2773,7 @@
       <c r="D110">
         <v>20</v>
       </c>
-      <c r="E110" s="15" t="s">
+      <c r="E110" s="12" t="s">
         <v>74</v>
       </c>
     </row>
@@ -2752,7 +2782,7 @@
         <v>3</v>
       </c>
       <c r="B111" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="C111" t="s">
         <v>60</v>
@@ -2769,7 +2799,7 @@
         <v>4</v>
       </c>
       <c r="B112" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="C112" t="s">
         <v>49</v>
@@ -2783,7 +2813,7 @@
         <v>5</v>
       </c>
       <c r="B113" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="C113" t="s">
         <v>49</v>
@@ -2797,7 +2827,7 @@
         <v>6</v>
       </c>
       <c r="B114" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="C114" t="s">
         <v>49</v>
@@ -2811,7 +2841,7 @@
         <v>7</v>
       </c>
       <c r="B115" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C115" t="s">
         <v>67</v>
@@ -2822,7 +2852,7 @@
         <v>8</v>
       </c>
       <c r="B116" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="C116" t="s">
         <v>67</v>
@@ -2833,7 +2863,7 @@
         <v>9</v>
       </c>
       <c r="B117" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="C117" t="s">
         <v>76</v>
@@ -2844,7 +2874,7 @@
         <v>10</v>
       </c>
       <c r="B118" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="C118" t="s">
         <v>76</v>
@@ -2855,7 +2885,7 @@
         <v>11</v>
       </c>
       <c r="B119" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="C119" t="s">
         <v>49</v>
@@ -2879,12 +2909,12 @@
       </c>
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B123" s="11" t="s">
-        <v>149</v>
-      </c>
-      <c r="C123" s="11"/>
-      <c r="D123" s="11"/>
-      <c r="E123" s="11"/>
+      <c r="B123" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="C123" s="9"/>
+      <c r="D123" s="9"/>
+      <c r="E123" s="9"/>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A124" s="2" t="s">
@@ -2925,7 +2955,7 @@
         <v>2</v>
       </c>
       <c r="B126" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="C126" t="s">
         <v>49</v>
@@ -2942,7 +2972,7 @@
         <v>3</v>
       </c>
       <c r="B127" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C127" t="s">
         <v>49</v>
@@ -2956,7 +2986,7 @@
         <v>4</v>
       </c>
       <c r="B128" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="C128" t="s">
         <v>49</v>
@@ -2970,7 +3000,7 @@
         <v>5</v>
       </c>
       <c r="B129" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="C129" t="s">
         <v>49</v>
@@ -2983,13 +3013,13 @@
       <c r="A130">
         <v>6</v>
       </c>
-      <c r="B130" s="17" t="s">
-        <v>144</v>
-      </c>
-      <c r="C130" s="18" t="s">
+      <c r="B130" s="13" t="s">
+        <v>140</v>
+      </c>
+      <c r="C130" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="D130" s="23" t="s">
+      <c r="D130" s="19" t="s">
         <v>67</v>
       </c>
     </row>
@@ -2997,13 +3027,13 @@
       <c r="A131">
         <v>7</v>
       </c>
-      <c r="B131" s="18" t="s">
-        <v>153</v>
-      </c>
-      <c r="C131" s="18" t="s">
+      <c r="B131" s="14" t="s">
+        <v>149</v>
+      </c>
+      <c r="C131" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="D131" s="23" t="s">
+      <c r="D131" s="19" t="s">
         <v>67</v>
       </c>
     </row>
@@ -3011,18 +3041,18 @@
       <c r="A132">
         <v>8</v>
       </c>
-      <c r="B132" s="18" t="s">
-        <v>154</v>
-      </c>
-      <c r="C132" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="D132" s="23" t="s">
+      <c r="B132" s="14" t="s">
+        <v>150</v>
+      </c>
+      <c r="C132" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="D132" s="19" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A133" s="23">
+      <c r="A133" s="19">
         <v>9</v>
       </c>
       <c r="B133" s="8" t="s">
@@ -3031,35 +3061,35 @@
       <c r="C133" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="D133" s="23" t="s">
-        <v>49</v>
-      </c>
-      <c r="E133" s="22"/>
-      <c r="F133" s="22"/>
+      <c r="D133" s="19" t="s">
+        <v>49</v>
+      </c>
+      <c r="E133" s="18"/>
+      <c r="F133" s="18"/>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A134" s="22"/>
+      <c r="A134" s="18"/>
       <c r="B134" s="8"/>
       <c r="C134" s="8"/>
-      <c r="D134" s="22"/>
-      <c r="E134" s="22"/>
-      <c r="F134" s="22"/>
+      <c r="D134" s="18"/>
+      <c r="E134" s="18"/>
+      <c r="F134" s="18"/>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A135" s="22"/>
+      <c r="A135" s="18"/>
       <c r="B135" s="8"/>
       <c r="C135" s="8"/>
-      <c r="D135" s="22"/>
-      <c r="E135" s="22"/>
-      <c r="F135" s="22"/>
+      <c r="D135" s="18"/>
+      <c r="E135" s="18"/>
+      <c r="F135" s="18"/>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B136" s="11" t="s">
-        <v>155</v>
-      </c>
-      <c r="C136" s="11"/>
-      <c r="D136" s="11"/>
-      <c r="E136" s="11"/>
+      <c r="B136" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="C136" s="9"/>
+      <c r="D136" s="9"/>
+      <c r="E136" s="9"/>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A137" s="2" t="s">
@@ -3100,7 +3130,7 @@
         <v>2</v>
       </c>
       <c r="B139" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="C139" t="s">
         <v>60</v>
@@ -3117,7 +3147,7 @@
         <v>3</v>
       </c>
       <c r="B140" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="C140" t="s">
         <v>60</v>
@@ -3134,10 +3164,10 @@
         <v>4</v>
       </c>
       <c r="B141" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="C141" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.2">
@@ -3145,10 +3175,10 @@
         <v>5</v>
       </c>
       <c r="B142" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="C142" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="D142">
         <v>7</v>
@@ -3159,7 +3189,7 @@
         <v>6</v>
       </c>
       <c r="B143" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="C143" t="s">
         <v>49</v>
@@ -3173,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="B144" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="C144" t="s">
         <v>60</v>
@@ -3190,7 +3220,7 @@
         <v>8</v>
       </c>
       <c r="B145" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="C145" t="s">
         <v>49</v>
@@ -3204,10 +3234,10 @@
         <v>9</v>
       </c>
       <c r="B146" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="C146" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.2">
@@ -3215,7 +3245,7 @@
         <v>10</v>
       </c>
       <c r="B147" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="C147" t="s">
         <v>61</v>
@@ -3226,7 +3256,7 @@
         <v>11</v>
       </c>
       <c r="B148" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="C148" t="s">
         <v>61</v>
@@ -3237,19 +3267,19 @@
         <v>12</v>
       </c>
       <c r="B149" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="C149" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B152" s="11" t="s">
-        <v>167</v>
-      </c>
-      <c r="C152" s="11"/>
-      <c r="D152" s="11"/>
-      <c r="E152" s="11"/>
+      <c r="B152" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="C152" s="9"/>
+      <c r="D152" s="9"/>
+      <c r="E152" s="9"/>
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A153" s="2" t="s">
@@ -3290,7 +3320,7 @@
         <v>2</v>
       </c>
       <c r="B155" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="C155" t="s">
         <v>60</v>
@@ -3307,7 +3337,7 @@
         <v>3</v>
       </c>
       <c r="B156" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="C156" t="s">
         <v>60</v>
@@ -3324,7 +3354,7 @@
         <v>4</v>
       </c>
       <c r="B157" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="C157" t="s">
         <v>60</v>
@@ -3341,7 +3371,7 @@
         <v>5</v>
       </c>
       <c r="B158" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="C158" t="s">
         <v>60</v>
@@ -3358,10 +3388,10 @@
         <v>6</v>
       </c>
       <c r="B159" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="C159" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D159">
         <v>500</v>
@@ -3372,7 +3402,7 @@
         <v>7</v>
       </c>
       <c r="B160" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C160" t="s">
         <v>49</v>
@@ -3386,10 +3416,10 @@
         <v>8</v>
       </c>
       <c r="B161" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="C161" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="162" spans="1:5" x14ac:dyDescent="0.2">
@@ -3397,7 +3427,7 @@
         <v>9</v>
       </c>
       <c r="B162" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="C162" t="s">
         <v>67</v>
@@ -3411,10 +3441,10 @@
         <v>10</v>
       </c>
       <c r="B163" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="C163" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="D163">
         <v>7</v>
@@ -3425,15 +3455,15 @@
         <v>11</v>
       </c>
       <c r="B164" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C164" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B165" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C165" t="s">
         <v>49</v>
@@ -3444,7 +3474,7 @@
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B166" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="C166" t="s">
         <v>49</v>
@@ -3458,7 +3488,7 @@
         <v>12</v>
       </c>
       <c r="B167" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="C167" t="s">
         <v>61</v>
@@ -3469,7 +3499,7 @@
         <v>13</v>
       </c>
       <c r="B168" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="C168" t="s">
         <v>61</v>
@@ -3480,19 +3510,19 @@
         <v>14</v>
       </c>
       <c r="B169" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="C169" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B172" s="11" t="s">
-        <v>178</v>
-      </c>
-      <c r="C172" s="11"/>
-      <c r="D172" s="11"/>
-      <c r="E172" s="11"/>
+      <c r="B172" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="C172" s="9"/>
+      <c r="D172" s="9"/>
+      <c r="E172" s="9"/>
     </row>
     <row r="173" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A173" s="2" t="s">
@@ -3533,7 +3563,7 @@
         <v>2</v>
       </c>
       <c r="B175" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="C175" t="s">
         <v>60</v>
@@ -3550,7 +3580,7 @@
         <v>3</v>
       </c>
       <c r="B176" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="C176" t="s">
         <v>60</v>
@@ -3567,7 +3597,7 @@
         <v>4</v>
       </c>
       <c r="B177" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="C177" t="s">
         <v>60</v>
@@ -3584,7 +3614,7 @@
         <v>5</v>
       </c>
       <c r="B178" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="C178" t="s">
         <v>49</v>
@@ -3598,7 +3628,7 @@
         <v>6</v>
       </c>
       <c r="B179" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="C179" t="s">
         <v>49</v>
@@ -3612,10 +3642,10 @@
         <v>7</v>
       </c>
       <c r="B180" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="C180" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D180">
         <v>20</v>
@@ -3626,10 +3656,10 @@
         <v>8</v>
       </c>
       <c r="B181" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="C181" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D181">
         <v>100</v>
@@ -3640,7 +3670,7 @@
         <v>9</v>
       </c>
       <c r="B182" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="C182" t="s">
         <v>67</v>
@@ -3654,7 +3684,7 @@
         <v>10</v>
       </c>
       <c r="B183" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="C183" t="s">
         <v>49</v>
@@ -3668,13 +3698,13 @@
         <v>11</v>
       </c>
       <c r="B184" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="C184" t="s">
         <v>61</v>
       </c>
       <c r="D184" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
     </row>
     <row r="185" spans="1:5" x14ac:dyDescent="0.2">
@@ -3682,7 +3712,7 @@
         <v>12</v>
       </c>
       <c r="B185" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="C185" t="s">
         <v>61</v>
@@ -3693,16 +3723,580 @@
         <v>13</v>
       </c>
       <c r="B186" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="C186" t="s">
         <v>61</v>
       </c>
     </row>
+    <row r="189" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A189" s="12"/>
+      <c r="B189" s="26" t="s">
+        <v>189</v>
+      </c>
+      <c r="C189" s="26"/>
+      <c r="D189" s="26"/>
+      <c r="E189" s="26"/>
+    </row>
+    <row r="190" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A190" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="B190" s="22" t="s">
+        <v>51</v>
+      </c>
+      <c r="C190" s="22" t="s">
+        <v>52</v>
+      </c>
+      <c r="D190" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="E190" s="21" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="191" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A191" s="12">
+        <v>1</v>
+      </c>
+      <c r="B191" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="C191" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="D191" s="12">
+        <v>20</v>
+      </c>
+      <c r="E191" s="12" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="192" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A192" s="12">
+        <v>2</v>
+      </c>
+      <c r="B192" s="12" t="s">
+        <v>190</v>
+      </c>
+      <c r="C192" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="D192" s="12">
+        <v>15</v>
+      </c>
+      <c r="E192" s="12" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="193" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A193" s="12">
+        <v>3</v>
+      </c>
+      <c r="B193" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="C193" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="D193" s="12">
+        <v>15</v>
+      </c>
+      <c r="E193" s="12"/>
+    </row>
+    <row r="194" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A194" s="12">
+        <v>4</v>
+      </c>
+      <c r="B194" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="C194" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="D194" s="12">
+        <v>15</v>
+      </c>
+      <c r="E194" s="12"/>
+    </row>
+    <row r="195" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A195" s="12">
+        <v>5</v>
+      </c>
+      <c r="B195" s="12" t="s">
+        <v>140</v>
+      </c>
+      <c r="C195" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="D195" s="12">
+        <v>5</v>
+      </c>
+      <c r="E195" s="12"/>
+    </row>
+    <row r="196" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A196" s="12">
+        <v>6</v>
+      </c>
+      <c r="B196" s="23" t="s">
+        <v>160</v>
+      </c>
+      <c r="C196" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="D196" s="25"/>
+      <c r="E196" s="12"/>
+    </row>
+    <row r="197" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A197" s="12">
+        <v>7</v>
+      </c>
+      <c r="B197" s="24" t="s">
+        <v>191</v>
+      </c>
+      <c r="C197" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="D197" s="25">
+        <v>20</v>
+      </c>
+      <c r="E197" s="12" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="200" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B200" s="9" t="s">
+        <v>179</v>
+      </c>
+      <c r="C200" s="9"/>
+      <c r="D200" s="9"/>
+      <c r="E200" s="9"/>
+    </row>
+    <row r="201" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A201" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B201" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="C201" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="D201" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="E201" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="202" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A202">
+        <v>1</v>
+      </c>
+      <c r="B202" t="s">
+        <v>45</v>
+      </c>
+      <c r="C202" t="s">
+        <v>60</v>
+      </c>
+      <c r="D202">
+        <v>20</v>
+      </c>
+      <c r="E202" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="203" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A203">
+        <v>2</v>
+      </c>
+      <c r="B203" t="s">
+        <v>152</v>
+      </c>
+      <c r="C203" t="s">
+        <v>60</v>
+      </c>
+      <c r="D203">
+        <v>20</v>
+      </c>
+      <c r="E203" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="204" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A204">
+        <v>3</v>
+      </c>
+      <c r="B204" t="s">
+        <v>156</v>
+      </c>
+      <c r="C204" t="s">
+        <v>60</v>
+      </c>
+      <c r="D204">
+        <v>20</v>
+      </c>
+      <c r="E204" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="205" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A205">
+        <v>4</v>
+      </c>
+      <c r="B205" t="s">
+        <v>182</v>
+      </c>
+      <c r="C205" t="s">
+        <v>60</v>
+      </c>
+      <c r="D205">
+        <v>20</v>
+      </c>
+      <c r="E205" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="206" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A206">
+        <v>5</v>
+      </c>
+      <c r="B206" t="s">
+        <v>181</v>
+      </c>
+      <c r="C206" t="s">
+        <v>186</v>
+      </c>
+      <c r="D206">
+        <v>20</v>
+      </c>
+      <c r="E206" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="207" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A207">
+        <v>6</v>
+      </c>
+      <c r="B207" t="s">
+        <v>180</v>
+      </c>
+      <c r="C207" t="s">
+        <v>49</v>
+      </c>
+      <c r="D207">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="208" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A208">
+        <v>7</v>
+      </c>
+      <c r="B208" t="s">
+        <v>128</v>
+      </c>
+      <c r="C208" t="s">
+        <v>49</v>
+      </c>
+      <c r="D208">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="209" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A209">
+        <v>8</v>
+      </c>
+      <c r="B209" t="s">
+        <v>183</v>
+      </c>
+      <c r="C209" t="s">
+        <v>49</v>
+      </c>
+      <c r="D209">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="210" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A210">
+        <v>9</v>
+      </c>
+      <c r="B210" t="s">
+        <v>116</v>
+      </c>
+      <c r="C210" t="s">
+        <v>49</v>
+      </c>
+      <c r="D210">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="211" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A211">
+        <v>10</v>
+      </c>
+      <c r="B211" t="s">
+        <v>184</v>
+      </c>
+      <c r="C211" t="s">
+        <v>61</v>
+      </c>
+      <c r="D211" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="212" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A212">
+        <v>11</v>
+      </c>
+      <c r="B212" t="s">
+        <v>185</v>
+      </c>
+      <c r="C212" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="213" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A213">
+        <v>12</v>
+      </c>
+      <c r="B213" t="s">
+        <v>159</v>
+      </c>
+      <c r="C213" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="214" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A214">
+        <v>13</v>
+      </c>
+      <c r="B214" t="s">
+        <v>160</v>
+      </c>
+      <c r="C214" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="217" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B217" s="9" t="s">
+        <v>192</v>
+      </c>
+      <c r="C217" s="9"/>
+      <c r="D217" s="9"/>
+      <c r="E217" s="9"/>
+    </row>
+    <row r="218" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A218" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B218" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="C218" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="D218" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="E218" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="219" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A219">
+        <v>1</v>
+      </c>
+      <c r="B219" t="s">
+        <v>45</v>
+      </c>
+      <c r="C219" t="s">
+        <v>60</v>
+      </c>
+      <c r="D219">
+        <v>20</v>
+      </c>
+      <c r="E219" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="220" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A220">
+        <v>2</v>
+      </c>
+      <c r="B220" t="s">
+        <v>193</v>
+      </c>
+      <c r="C220" t="s">
+        <v>60</v>
+      </c>
+      <c r="D220">
+        <v>20</v>
+      </c>
+      <c r="E220" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="221" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A221">
+        <v>3</v>
+      </c>
+      <c r="B221" t="s">
+        <v>156</v>
+      </c>
+      <c r="C221" t="s">
+        <v>60</v>
+      </c>
+      <c r="D221">
+        <v>20</v>
+      </c>
+      <c r="E221" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="222" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A222">
+        <v>4</v>
+      </c>
+      <c r="B222" t="s">
+        <v>129</v>
+      </c>
+      <c r="C222" t="s">
+        <v>49</v>
+      </c>
+      <c r="D222">
+        <v>100</v>
+      </c>
+      <c r="E222" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="223" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A223">
+        <v>5</v>
+      </c>
+      <c r="B223" t="s">
+        <v>194</v>
+      </c>
+      <c r="C223" t="s">
+        <v>49</v>
+      </c>
+      <c r="D223">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="224" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A224">
+        <v>6</v>
+      </c>
+      <c r="B224" t="s">
+        <v>175</v>
+      </c>
+      <c r="C224" t="s">
+        <v>109</v>
+      </c>
+      <c r="D224">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="225" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A225">
+        <v>7</v>
+      </c>
+      <c r="B225" t="s">
+        <v>195</v>
+      </c>
+      <c r="C225" t="s">
+        <v>67</v>
+      </c>
+      <c r="D225">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="226" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A226">
+        <v>8</v>
+      </c>
+      <c r="B226" t="s">
+        <v>196</v>
+      </c>
+      <c r="C226" t="s">
+        <v>49</v>
+      </c>
+      <c r="D226">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="227" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A227">
+        <v>9</v>
+      </c>
+      <c r="B227" t="s">
+        <v>197</v>
+      </c>
+      <c r="C227" t="s">
+        <v>49</v>
+      </c>
+      <c r="D227">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="228" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A228">
+        <v>10</v>
+      </c>
+      <c r="B228" t="s">
+        <v>198</v>
+      </c>
+      <c r="C228" t="s">
+        <v>49</v>
+      </c>
+      <c r="D228">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="229" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A229">
+        <v>11</v>
+      </c>
+      <c r="B229" t="s">
+        <v>199</v>
+      </c>
+      <c r="C229" t="s">
+        <v>49</v>
+      </c>
+      <c r="D229">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="230" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A230">
+        <v>12</v>
+      </c>
+      <c r="B230" t="s">
+        <v>159</v>
+      </c>
+      <c r="C230" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="231" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A231">
+        <v>13</v>
+      </c>
+      <c r="B231" t="s">
+        <v>160</v>
+      </c>
+      <c r="C231" t="s">
+        <v>61</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="16">
+    <mergeCell ref="B217:E217"/>
     <mergeCell ref="B152:E152"/>
     <mergeCell ref="B172:E172"/>
+    <mergeCell ref="B200:E200"/>
+    <mergeCell ref="B189:E189"/>
     <mergeCell ref="B47:E47"/>
     <mergeCell ref="B56:E56"/>
     <mergeCell ref="B65:E65"/>
@@ -3721,931 +4315,101 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD54E32F-1636-154F-88FF-57ECFAEA7F4B}">
-  <dimension ref="A3:X43"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="38.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="3.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="79" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:24" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="B3" s="9"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="9"/>
-      <c r="I3" s="9"/>
-      <c r="J3" s="9"/>
-      <c r="K3" s="9"/>
-      <c r="M3" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="N3" s="10"/>
-      <c r="O3" s="10"/>
-      <c r="P3" s="10"/>
-      <c r="Q3" s="10"/>
-      <c r="R3" s="10"/>
-      <c r="S3" s="10"/>
-      <c r="T3" s="10"/>
-      <c r="U3" s="10"/>
-      <c r="V3" s="10"/>
-      <c r="W3" s="10"/>
-      <c r="X3" s="10"/>
-    </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A4" s="9"/>
-      <c r="B4" s="9"/>
-      <c r="C4" s="9"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9"/>
-      <c r="G4" s="9"/>
-      <c r="H4" s="9"/>
-      <c r="I4" s="9"/>
-      <c r="J4" s="9"/>
-      <c r="K4" s="9"/>
-      <c r="M4" s="10"/>
-      <c r="N4" s="10"/>
-      <c r="O4" s="10"/>
-      <c r="P4" s="10"/>
-      <c r="Q4" s="10"/>
-      <c r="R4" s="10"/>
-      <c r="S4" s="10"/>
-      <c r="T4" s="10"/>
-      <c r="U4" s="10"/>
-      <c r="V4" s="10"/>
-      <c r="W4" s="10"/>
-      <c r="X4" s="10"/>
-    </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A5" s="9"/>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="9"/>
-      <c r="H5" s="9"/>
-      <c r="I5" s="9"/>
-      <c r="J5" s="9"/>
-      <c r="K5" s="9"/>
-      <c r="M5" s="10"/>
-      <c r="N5" s="10"/>
-      <c r="O5" s="10"/>
-      <c r="P5" s="10"/>
-      <c r="Q5" s="10"/>
-      <c r="R5" s="10"/>
-      <c r="S5" s="10"/>
-      <c r="T5" s="10"/>
-      <c r="U5" s="10"/>
-      <c r="V5" s="10"/>
-      <c r="W5" s="10"/>
-      <c r="X5" s="10"/>
-    </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A6" s="9"/>
-      <c r="B6" s="9"/>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="9"/>
-      <c r="I6" s="9"/>
-      <c r="J6" s="9"/>
-      <c r="K6" s="9"/>
-      <c r="M6" s="10"/>
-      <c r="N6" s="10"/>
-      <c r="O6" s="10"/>
-      <c r="P6" s="10"/>
-      <c r="Q6" s="10"/>
-      <c r="R6" s="10"/>
-      <c r="S6" s="10"/>
-      <c r="T6" s="10"/>
-      <c r="U6" s="10"/>
-      <c r="V6" s="10"/>
-      <c r="W6" s="10"/>
-      <c r="X6" s="10"/>
-    </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A7" s="9"/>
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
-      <c r="M7" s="10"/>
-      <c r="N7" s="10"/>
-      <c r="O7" s="10"/>
-      <c r="P7" s="10"/>
-      <c r="Q7" s="10"/>
-      <c r="R7" s="10"/>
-      <c r="S7" s="10"/>
-      <c r="T7" s="10"/>
-      <c r="U7" s="10"/>
-      <c r="V7" s="10"/>
-      <c r="W7" s="10"/>
-      <c r="X7" s="10"/>
-    </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A8" s="9"/>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9"/>
-      <c r="K8" s="9"/>
-      <c r="M8" s="10"/>
-      <c r="N8" s="10"/>
-      <c r="O8" s="10"/>
-      <c r="P8" s="10"/>
-      <c r="Q8" s="10"/>
-      <c r="R8" s="10"/>
-      <c r="S8" s="10"/>
-      <c r="T8" s="10"/>
-      <c r="U8" s="10"/>
-      <c r="V8" s="10"/>
-      <c r="W8" s="10"/>
-      <c r="X8" s="10"/>
-    </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A9" s="9"/>
-      <c r="B9" s="9"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="9"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="9"/>
-      <c r="K9" s="9"/>
-      <c r="M9" s="10"/>
-      <c r="N9" s="10"/>
-      <c r="O9" s="10"/>
-      <c r="P9" s="10"/>
-      <c r="Q9" s="10"/>
-      <c r="R9" s="10"/>
-      <c r="S9" s="10"/>
-      <c r="T9" s="10"/>
-      <c r="U9" s="10"/>
-      <c r="V9" s="10"/>
-      <c r="W9" s="10"/>
-      <c r="X9" s="10"/>
-    </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A10" s="9"/>
-      <c r="B10" s="9"/>
-      <c r="C10" s="9"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="9"/>
-      <c r="G10" s="9"/>
-      <c r="H10" s="9"/>
-      <c r="I10" s="9"/>
-      <c r="J10" s="9"/>
-      <c r="K10" s="9"/>
-      <c r="M10" s="10"/>
-      <c r="N10" s="10"/>
-      <c r="O10" s="10"/>
-      <c r="P10" s="10"/>
-      <c r="Q10" s="10"/>
-      <c r="R10" s="10"/>
-      <c r="S10" s="10"/>
-      <c r="T10" s="10"/>
-      <c r="U10" s="10"/>
-      <c r="V10" s="10"/>
-      <c r="W10" s="10"/>
-      <c r="X10" s="10"/>
-    </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A11" s="9"/>
-      <c r="B11" s="9"/>
-      <c r="C11" s="9"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="9"/>
-      <c r="I11" s="9"/>
-      <c r="J11" s="9"/>
-      <c r="K11" s="9"/>
-      <c r="M11" s="10"/>
-      <c r="N11" s="10"/>
-      <c r="O11" s="10"/>
-      <c r="P11" s="10"/>
-      <c r="Q11" s="10"/>
-      <c r="R11" s="10"/>
-      <c r="S11" s="10"/>
-      <c r="T11" s="10"/>
-      <c r="U11" s="10"/>
-      <c r="V11" s="10"/>
-      <c r="W11" s="10"/>
-      <c r="X11" s="10"/>
-    </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A12" s="9"/>
-      <c r="B12" s="9"/>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="9"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
-      <c r="K12" s="9"/>
-      <c r="M12" s="10"/>
-      <c r="N12" s="10"/>
-      <c r="O12" s="10"/>
-      <c r="P12" s="10"/>
-      <c r="Q12" s="10"/>
-      <c r="R12" s="10"/>
-      <c r="S12" s="10"/>
-      <c r="T12" s="10"/>
-      <c r="U12" s="10"/>
-      <c r="V12" s="10"/>
-      <c r="W12" s="10"/>
-      <c r="X12" s="10"/>
-    </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A13" s="9"/>
-      <c r="B13" s="9"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="9"/>
-      <c r="I13" s="9"/>
-      <c r="J13" s="9"/>
-      <c r="K13" s="9"/>
-      <c r="M13" s="10"/>
-      <c r="N13" s="10"/>
-      <c r="O13" s="10"/>
-      <c r="P13" s="10"/>
-      <c r="Q13" s="10"/>
-      <c r="R13" s="10"/>
-      <c r="S13" s="10"/>
-      <c r="T13" s="10"/>
-      <c r="U13" s="10"/>
-      <c r="V13" s="10"/>
-      <c r="W13" s="10"/>
-      <c r="X13" s="10"/>
-    </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A14" s="9"/>
-      <c r="B14" s="9"/>
-      <c r="C14" s="9"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="9"/>
-      <c r="I14" s="9"/>
-      <c r="J14" s="9"/>
-      <c r="K14" s="9"/>
-      <c r="M14" s="10"/>
-      <c r="N14" s="10"/>
-      <c r="O14" s="10"/>
-      <c r="P14" s="10"/>
-      <c r="Q14" s="10"/>
-      <c r="R14" s="10"/>
-      <c r="S14" s="10"/>
-      <c r="T14" s="10"/>
-      <c r="U14" s="10"/>
-      <c r="V14" s="10"/>
-      <c r="W14" s="10"/>
-      <c r="X14" s="10"/>
-    </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A15" s="9"/>
-      <c r="B15" s="9"/>
-      <c r="C15" s="9"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9"/>
-      <c r="F15" s="9"/>
-      <c r="G15" s="9"/>
-      <c r="H15" s="9"/>
-      <c r="I15" s="9"/>
-      <c r="J15" s="9"/>
-      <c r="K15" s="9"/>
-      <c r="M15" s="10"/>
-      <c r="N15" s="10"/>
-      <c r="O15" s="10"/>
-      <c r="P15" s="10"/>
-      <c r="Q15" s="10"/>
-      <c r="R15" s="10"/>
-      <c r="S15" s="10"/>
-      <c r="T15" s="10"/>
-      <c r="U15" s="10"/>
-      <c r="V15" s="10"/>
-      <c r="W15" s="10"/>
-      <c r="X15" s="10"/>
-    </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A16" s="9"/>
-      <c r="B16" s="9"/>
-      <c r="C16" s="9"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
-      <c r="G16" s="9"/>
-      <c r="H16" s="9"/>
-      <c r="I16" s="9"/>
-      <c r="J16" s="9"/>
-      <c r="K16" s="9"/>
-      <c r="M16" s="10"/>
-      <c r="N16" s="10"/>
-      <c r="O16" s="10"/>
-      <c r="P16" s="10"/>
-      <c r="Q16" s="10"/>
-      <c r="R16" s="10"/>
-      <c r="S16" s="10"/>
-      <c r="T16" s="10"/>
-      <c r="U16" s="10"/>
-      <c r="V16" s="10"/>
-      <c r="W16" s="10"/>
-      <c r="X16" s="10"/>
-    </row>
-    <row r="17" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A17" s="9"/>
-      <c r="B17" s="9"/>
-      <c r="C17" s="9"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="9"/>
-      <c r="F17" s="9"/>
-      <c r="G17" s="9"/>
-      <c r="H17" s="9"/>
-      <c r="I17" s="9"/>
-      <c r="J17" s="9"/>
-      <c r="K17" s="9"/>
-      <c r="M17" s="10"/>
-      <c r="N17" s="10"/>
-      <c r="O17" s="10"/>
-      <c r="P17" s="10"/>
-      <c r="Q17" s="10"/>
-      <c r="R17" s="10"/>
-      <c r="S17" s="10"/>
-      <c r="T17" s="10"/>
-      <c r="U17" s="10"/>
-      <c r="V17" s="10"/>
-      <c r="W17" s="10"/>
-      <c r="X17" s="10"/>
-    </row>
-    <row r="18" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A18" s="9"/>
-      <c r="B18" s="9"/>
-      <c r="C18" s="9"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="9"/>
-      <c r="G18" s="9"/>
-      <c r="H18" s="9"/>
-      <c r="I18" s="9"/>
-      <c r="J18" s="9"/>
-      <c r="K18" s="9"/>
-      <c r="M18" s="10"/>
-      <c r="N18" s="10"/>
-      <c r="O18" s="10"/>
-      <c r="P18" s="10"/>
-      <c r="Q18" s="10"/>
-      <c r="R18" s="10"/>
-      <c r="S18" s="10"/>
-      <c r="T18" s="10"/>
-      <c r="U18" s="10"/>
-      <c r="V18" s="10"/>
-      <c r="W18" s="10"/>
-      <c r="X18" s="10"/>
-    </row>
-    <row r="19" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A19" s="9"/>
-      <c r="B19" s="9"/>
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="9"/>
-      <c r="H19" s="9"/>
-      <c r="I19" s="9"/>
-      <c r="J19" s="9"/>
-      <c r="K19" s="9"/>
-      <c r="M19" s="10"/>
-      <c r="N19" s="10"/>
-      <c r="O19" s="10"/>
-      <c r="P19" s="10"/>
-      <c r="Q19" s="10"/>
-      <c r="R19" s="10"/>
-      <c r="S19" s="10"/>
-      <c r="T19" s="10"/>
-      <c r="U19" s="10"/>
-      <c r="V19" s="10"/>
-      <c r="W19" s="10"/>
-      <c r="X19" s="10"/>
-    </row>
-    <row r="20" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A20" s="9"/>
-      <c r="B20" s="9"/>
-      <c r="C20" s="9"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="9"/>
-      <c r="F20" s="9"/>
-      <c r="G20" s="9"/>
-      <c r="H20" s="9"/>
-      <c r="I20" s="9"/>
-      <c r="J20" s="9"/>
-      <c r="K20" s="9"/>
-      <c r="M20" s="10"/>
-      <c r="N20" s="10"/>
-      <c r="O20" s="10"/>
-      <c r="P20" s="10"/>
-      <c r="Q20" s="10"/>
-      <c r="R20" s="10"/>
-      <c r="S20" s="10"/>
-      <c r="T20" s="10"/>
-      <c r="U20" s="10"/>
-      <c r="V20" s="10"/>
-      <c r="W20" s="10"/>
-      <c r="X20" s="10"/>
-    </row>
-    <row r="21" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A21" s="9"/>
-      <c r="B21" s="9"/>
-      <c r="C21" s="9"/>
-      <c r="D21" s="9"/>
-      <c r="E21" s="9"/>
-      <c r="F21" s="9"/>
-      <c r="G21" s="9"/>
-      <c r="H21" s="9"/>
-      <c r="I21" s="9"/>
-      <c r="J21" s="9"/>
-      <c r="K21" s="9"/>
-      <c r="M21" s="10"/>
-      <c r="N21" s="10"/>
-      <c r="O21" s="10"/>
-      <c r="P21" s="10"/>
-      <c r="Q21" s="10"/>
-      <c r="R21" s="10"/>
-      <c r="S21" s="10"/>
-      <c r="T21" s="10"/>
-      <c r="U21" s="10"/>
-      <c r="V21" s="10"/>
-      <c r="W21" s="10"/>
-      <c r="X21" s="10"/>
-    </row>
-    <row r="22" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A22" s="9"/>
-      <c r="B22" s="9"/>
-      <c r="C22" s="9"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="9"/>
-      <c r="F22" s="9"/>
-      <c r="G22" s="9"/>
-      <c r="H22" s="9"/>
-      <c r="I22" s="9"/>
-      <c r="J22" s="9"/>
-      <c r="K22" s="9"/>
-      <c r="M22" s="10"/>
-      <c r="N22" s="10"/>
-      <c r="O22" s="10"/>
-      <c r="P22" s="10"/>
-      <c r="Q22" s="10"/>
-      <c r="R22" s="10"/>
-      <c r="S22" s="10"/>
-      <c r="T22" s="10"/>
-      <c r="U22" s="10"/>
-      <c r="V22" s="10"/>
-      <c r="W22" s="10"/>
-      <c r="X22" s="10"/>
-    </row>
-    <row r="23" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A23" s="9"/>
-      <c r="B23" s="9"/>
-      <c r="C23" s="9"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="9"/>
-      <c r="F23" s="9"/>
-      <c r="G23" s="9"/>
-      <c r="H23" s="9"/>
-      <c r="I23" s="9"/>
-      <c r="J23" s="9"/>
-      <c r="K23" s="9"/>
-      <c r="M23" s="10"/>
-      <c r="N23" s="10"/>
-      <c r="O23" s="10"/>
-      <c r="P23" s="10"/>
-      <c r="Q23" s="10"/>
-      <c r="R23" s="10"/>
-      <c r="S23" s="10"/>
-      <c r="T23" s="10"/>
-      <c r="U23" s="10"/>
-      <c r="V23" s="10"/>
-      <c r="W23" s="10"/>
-      <c r="X23" s="10"/>
-    </row>
-    <row r="24" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A24" s="9"/>
-      <c r="B24" s="9"/>
-      <c r="C24" s="9"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="9"/>
-      <c r="G24" s="9"/>
-      <c r="H24" s="9"/>
-      <c r="I24" s="9"/>
-      <c r="J24" s="9"/>
-      <c r="K24" s="9"/>
-      <c r="M24" s="10"/>
-      <c r="N24" s="10"/>
-      <c r="O24" s="10"/>
-      <c r="P24" s="10"/>
-      <c r="Q24" s="10"/>
-      <c r="R24" s="10"/>
-      <c r="S24" s="10"/>
-      <c r="T24" s="10"/>
-      <c r="U24" s="10"/>
-      <c r="V24" s="10"/>
-      <c r="W24" s="10"/>
-      <c r="X24" s="10"/>
-    </row>
-    <row r="25" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A25" s="9"/>
-      <c r="B25" s="9"/>
-      <c r="C25" s="9"/>
-      <c r="D25" s="9"/>
-      <c r="E25" s="9"/>
-      <c r="F25" s="9"/>
-      <c r="G25" s="9"/>
-      <c r="H25" s="9"/>
-      <c r="I25" s="9"/>
-      <c r="J25" s="9"/>
-      <c r="K25" s="9"/>
-      <c r="M25" s="10"/>
-      <c r="N25" s="10"/>
-      <c r="O25" s="10"/>
-      <c r="P25" s="10"/>
-      <c r="Q25" s="10"/>
-      <c r="R25" s="10"/>
-      <c r="S25" s="10"/>
-      <c r="T25" s="10"/>
-      <c r="U25" s="10"/>
-      <c r="V25" s="10"/>
-      <c r="W25" s="10"/>
-      <c r="X25" s="10"/>
-    </row>
-    <row r="26" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A26" s="9"/>
-      <c r="B26" s="9"/>
-      <c r="C26" s="9"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="9"/>
-      <c r="F26" s="9"/>
-      <c r="G26" s="9"/>
-      <c r="H26" s="9"/>
-      <c r="I26" s="9"/>
-      <c r="J26" s="9"/>
-      <c r="K26" s="9"/>
-      <c r="M26" s="10"/>
-      <c r="N26" s="10"/>
-      <c r="O26" s="10"/>
-      <c r="P26" s="10"/>
-      <c r="Q26" s="10"/>
-      <c r="R26" s="10"/>
-      <c r="S26" s="10"/>
-      <c r="T26" s="10"/>
-      <c r="U26" s="10"/>
-      <c r="V26" s="10"/>
-      <c r="W26" s="10"/>
-      <c r="X26" s="10"/>
-    </row>
-    <row r="27" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A27" s="9"/>
-      <c r="B27" s="9"/>
-      <c r="C27" s="9"/>
-      <c r="D27" s="9"/>
-      <c r="E27" s="9"/>
-      <c r="F27" s="9"/>
-      <c r="G27" s="9"/>
-      <c r="H27" s="9"/>
-      <c r="I27" s="9"/>
-      <c r="J27" s="9"/>
-      <c r="K27" s="9"/>
-      <c r="M27" s="10"/>
-      <c r="N27" s="10"/>
-      <c r="O27" s="10"/>
-      <c r="P27" s="10"/>
-      <c r="Q27" s="10"/>
-      <c r="R27" s="10"/>
-      <c r="S27" s="10"/>
-      <c r="T27" s="10"/>
-      <c r="U27" s="10"/>
-      <c r="V27" s="10"/>
-      <c r="W27" s="10"/>
-      <c r="X27" s="10"/>
-    </row>
-    <row r="28" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A28" s="9"/>
-      <c r="B28" s="9"/>
-      <c r="C28" s="9"/>
-      <c r="D28" s="9"/>
-      <c r="E28" s="9"/>
-      <c r="F28" s="9"/>
-      <c r="G28" s="9"/>
-      <c r="H28" s="9"/>
-      <c r="I28" s="9"/>
-      <c r="J28" s="9"/>
-      <c r="K28" s="9"/>
-      <c r="M28" s="10"/>
-      <c r="N28" s="10"/>
-      <c r="O28" s="10"/>
-      <c r="P28" s="10"/>
-      <c r="Q28" s="10"/>
-      <c r="R28" s="10"/>
-      <c r="S28" s="10"/>
-      <c r="T28" s="10"/>
-      <c r="U28" s="10"/>
-      <c r="V28" s="10"/>
-      <c r="W28" s="10"/>
-      <c r="X28" s="10"/>
-    </row>
-    <row r="29" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="M29" s="10"/>
-      <c r="N29" s="10"/>
-      <c r="O29" s="10"/>
-      <c r="P29" s="10"/>
-      <c r="Q29" s="10"/>
-      <c r="R29" s="10"/>
-      <c r="S29" s="10"/>
-      <c r="T29" s="10"/>
-      <c r="U29" s="10"/>
-      <c r="V29" s="10"/>
-      <c r="W29" s="10"/>
-      <c r="X29" s="10"/>
-    </row>
-    <row r="30" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="M30" s="10"/>
-      <c r="N30" s="10"/>
-      <c r="O30" s="10"/>
-      <c r="P30" s="10"/>
-      <c r="Q30" s="10"/>
-      <c r="R30" s="10"/>
-      <c r="S30" s="10"/>
-      <c r="T30" s="10"/>
-      <c r="U30" s="10"/>
-      <c r="V30" s="10"/>
-      <c r="W30" s="10"/>
-      <c r="X30" s="10"/>
-    </row>
-    <row r="31" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="M31" s="10"/>
-      <c r="N31" s="10"/>
-      <c r="O31" s="10"/>
-      <c r="P31" s="10"/>
-      <c r="Q31" s="10"/>
-      <c r="R31" s="10"/>
-      <c r="S31" s="10"/>
-      <c r="T31" s="10"/>
-      <c r="U31" s="10"/>
-      <c r="V31" s="10"/>
-      <c r="W31" s="10"/>
-      <c r="X31" s="10"/>
-    </row>
-    <row r="32" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="M32" s="10"/>
-      <c r="N32" s="10"/>
-      <c r="O32" s="10"/>
-      <c r="P32" s="10"/>
-      <c r="Q32" s="10"/>
-      <c r="R32" s="10"/>
-      <c r="S32" s="10"/>
-      <c r="T32" s="10"/>
-      <c r="U32" s="10"/>
-      <c r="V32" s="10"/>
-      <c r="W32" s="10"/>
-      <c r="X32" s="10"/>
-    </row>
-    <row r="33" spans="1:24" ht="24" x14ac:dyDescent="0.3">
-      <c r="A33" s="16" t="s">
+    <row r="1" spans="1:4" ht="24" x14ac:dyDescent="0.3">
+      <c r="B1" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="B33" s="16"/>
-      <c r="C33" s="16"/>
-      <c r="D33" s="16"/>
-      <c r="E33" s="16"/>
-      <c r="F33" s="16"/>
-      <c r="G33" s="16"/>
-      <c r="M33" s="10"/>
-      <c r="N33" s="10"/>
-      <c r="O33" s="10"/>
-      <c r="P33" s="10"/>
-      <c r="Q33" s="10"/>
-      <c r="R33" s="10"/>
-      <c r="S33" s="10"/>
-      <c r="T33" s="10"/>
-      <c r="U33" s="10"/>
-      <c r="V33" s="10"/>
-      <c r="W33" s="10"/>
-      <c r="X33" s="10"/>
-    </row>
-    <row r="34" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A34">
-        <v>1</v>
-      </c>
-      <c r="B34" s="13" t="s">
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
         <v>94</v>
       </c>
-      <c r="M34" s="10"/>
-      <c r="N34" s="10"/>
-      <c r="O34" s="10"/>
-      <c r="P34" s="10"/>
-      <c r="Q34" s="10"/>
-      <c r="R34" s="10"/>
-      <c r="S34" s="10"/>
-      <c r="T34" s="10"/>
-      <c r="U34" s="10"/>
-      <c r="V34" s="10"/>
-      <c r="W34" s="10"/>
-      <c r="X34" s="10"/>
-    </row>
-    <row r="35" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A35">
-        <v>2</v>
-      </c>
-      <c r="B35" s="13" t="s">
-        <v>95</v>
-      </c>
-      <c r="M35" s="10"/>
-      <c r="N35" s="10"/>
-      <c r="O35" s="10"/>
-      <c r="P35" s="10"/>
-      <c r="Q35" s="10"/>
-      <c r="R35" s="10"/>
-      <c r="S35" s="10"/>
-      <c r="T35" s="10"/>
-      <c r="U35" s="10"/>
-      <c r="V35" s="10"/>
-      <c r="W35" s="10"/>
-      <c r="X35" s="10"/>
-    </row>
-    <row r="36" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A36">
-        <v>3</v>
-      </c>
-      <c r="B36" t="s">
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
         <v>96</v>
       </c>
-      <c r="M36" s="10"/>
-      <c r="N36" s="10"/>
-      <c r="O36" s="10"/>
-      <c r="P36" s="10"/>
-      <c r="Q36" s="10"/>
-      <c r="R36" s="10"/>
-      <c r="S36" s="10"/>
-      <c r="T36" s="10"/>
-      <c r="U36" s="10"/>
-      <c r="V36" s="10"/>
-      <c r="W36" s="10"/>
-      <c r="X36" s="10"/>
-    </row>
-    <row r="37" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A37">
-        <v>4</v>
-      </c>
-      <c r="B37" t="s">
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="M37" s="10"/>
-      <c r="N37" s="10"/>
-      <c r="O37" s="10"/>
-      <c r="P37" s="10"/>
-      <c r="Q37" s="10"/>
-      <c r="R37" s="10"/>
-      <c r="S37" s="10"/>
-      <c r="T37" s="10"/>
-      <c r="U37" s="10"/>
-      <c r="V37" s="10"/>
-      <c r="W37" s="10"/>
-      <c r="X37" s="10"/>
-    </row>
-    <row r="38" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A38">
-        <v>5</v>
-      </c>
-      <c r="B38" t="s">
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="M38" s="10"/>
-      <c r="N38" s="10"/>
-      <c r="O38" s="10"/>
-      <c r="P38" s="10"/>
-      <c r="Q38" s="10"/>
-      <c r="R38" s="10"/>
-      <c r="S38" s="10"/>
-      <c r="T38" s="10"/>
-      <c r="U38" s="10"/>
-      <c r="V38" s="10"/>
-      <c r="W38" s="10"/>
-      <c r="X38" s="10"/>
-    </row>
-    <row r="39" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A39">
-        <v>6</v>
-      </c>
-      <c r="B39" s="13" t="s">
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
         <v>100</v>
       </c>
-      <c r="C39" s="14"/>
-      <c r="D39" s="14"/>
-      <c r="E39" s="14"/>
-      <c r="M39" s="10"/>
-      <c r="N39" s="10"/>
-      <c r="O39" s="10"/>
-      <c r="P39" s="10"/>
-      <c r="Q39" s="10"/>
-      <c r="R39" s="10"/>
-      <c r="S39" s="10"/>
-      <c r="T39" s="10"/>
-      <c r="U39" s="10"/>
-      <c r="V39" s="10"/>
-      <c r="W39" s="10"/>
-      <c r="X39" s="10"/>
-    </row>
-    <row r="40" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A40">
-        <v>7</v>
-      </c>
-      <c r="B40" s="13" t="s">
-        <v>101</v>
-      </c>
-      <c r="C40" s="14"/>
-      <c r="M40" s="10"/>
-      <c r="N40" s="10"/>
-      <c r="O40" s="10"/>
-      <c r="P40" s="10"/>
-      <c r="Q40" s="10"/>
-      <c r="R40" s="10"/>
-      <c r="S40" s="10"/>
-      <c r="T40" s="10"/>
-      <c r="U40" s="10"/>
-      <c r="V40" s="10"/>
-      <c r="W40" s="10"/>
-      <c r="X40" s="10"/>
-    </row>
-    <row r="41" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A41">
-        <v>8</v>
-      </c>
-      <c r="B41" t="s">
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="M41" s="10"/>
-      <c r="N41" s="10"/>
-      <c r="O41" s="10"/>
-      <c r="P41" s="10"/>
-      <c r="Q41" s="10"/>
-      <c r="R41" s="10"/>
-      <c r="S41" s="10"/>
-      <c r="T41" s="10"/>
-      <c r="U41" s="10"/>
-      <c r="V41" s="10"/>
-      <c r="W41" s="10"/>
-      <c r="X41" s="10"/>
-    </row>
-    <row r="42" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A42">
-        <v>9</v>
-      </c>
-      <c r="B42" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="43" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A43">
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11">
         <v>10</v>
       </c>
-      <c r="B43" t="s">
-        <v>129</v>
+      <c r="B11" t="s">
+        <v>125</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A3:K28"/>
-    <mergeCell ref="M3:X41"/>
-    <mergeCell ref="A33:G33"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add sample readme file
</commit_message>
<xml_diff>
--- a/CareOS-Hospital_ERP_System.xlsx
+++ b/CareOS-Hospital_ERP_System.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hetlimbani/Desktop/Self_Learning/CareOS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E995176-786D-9A47-A128-F69926F4D308}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23D9EA63-E27B-9642-A47A-3A8C81875A9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19420" xr2:uid="{3BCF7A51-5C29-EE4C-8BC3-93CAF12DE1EA}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19420" activeTab="1" xr2:uid="{3BCF7A51-5C29-EE4C-8BC3-93CAF12DE1EA}"/>
   </bookViews>
   <sheets>
     <sheet name="ERP System" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="575" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="679" uniqueCount="227">
   <si>
     <t>Total Roles</t>
   </si>
@@ -635,6 +635,93 @@
   </si>
   <si>
     <t>clinicalNotes</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Billings Collection Schema</t>
+  </si>
+  <si>
+    <t>invoiceNumber</t>
+  </si>
+  <si>
+    <t>doctorId</t>
+  </si>
+  <si>
+    <t>consultationFee</t>
+  </si>
+  <si>
+    <t>treatmentCost</t>
+  </si>
+  <si>
+    <t>medicineCost</t>
+  </si>
+  <si>
+    <t>labCost</t>
+  </si>
+  <si>
+    <t>extraCharges</t>
+  </si>
+  <si>
+    <t>extraChargesNotes</t>
+  </si>
+  <si>
+    <t>grossTotal</t>
+  </si>
+  <si>
+    <t>deductionsPrePaid</t>
+  </si>
+  <si>
+    <t>insuranceCoverageAmount</t>
+  </si>
+  <si>
+    <t>netPayableAmount</t>
+  </si>
+  <si>
+    <t>insurance</t>
+  </si>
+  <si>
+    <t>billingItems</t>
+  </si>
+  <si>
+    <t>paymentMethod</t>
+  </si>
+  <si>
+    <t>receptionistId</t>
+  </si>
+  <si>
+    <t>timestamps</t>
+  </si>
+  <si>
+    <t>userEmail</t>
+  </si>
+  <si>
+    <t>userRole</t>
+  </si>
+  <si>
+    <t>title</t>
+  </si>
+  <si>
+    <t>messages</t>
+  </si>
+  <si>
+    <t>lastMessageAt</t>
+  </si>
+  <si>
+    <t>Chat Sessions Collection Schema</t>
+  </si>
+  <si>
+    <t>Patient_dashboards  Collection Schema</t>
+  </si>
+  <si>
+    <t>allergies</t>
+  </si>
+  <si>
+    <t>chronic_conditions</t>
+  </si>
+  <si>
+    <t>vitals_log</t>
+  </si>
+  <si>
+    <t>vitalsHistory</t>
   </si>
 </sst>
 </file>
@@ -1426,7 +1513,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5186853C-8F41-E14D-BD0A-415B9ACDCBCD}">
-  <dimension ref="A1:F231"/>
+  <dimension ref="A1:F282"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3.5" bestFit="1" customWidth="1"/>
@@ -4024,13 +4111,13 @@
         <v>10</v>
       </c>
       <c r="B211" t="s">
-        <v>182</v>
+        <v>226</v>
       </c>
       <c r="C211" t="s">
-        <v>59</v>
-      </c>
-      <c r="D211" t="s">
-        <v>176</v>
+        <v>107</v>
+      </c>
+      <c r="D211">
+        <v>100</v>
       </c>
     </row>
     <row r="212" spans="1:5" x14ac:dyDescent="0.2">
@@ -4038,7 +4125,7 @@
         <v>11</v>
       </c>
       <c r="B212" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C212" t="s">
         <v>59</v>
@@ -4049,7 +4136,7 @@
         <v>12</v>
       </c>
       <c r="B213" t="s">
-        <v>157</v>
+        <v>183</v>
       </c>
       <c r="C213" t="s">
         <v>59</v>
@@ -4060,60 +4147,54 @@
         <v>13</v>
       </c>
       <c r="B214" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C214" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B217" s="26" t="s">
+    <row r="215" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A215">
+        <v>14</v>
+      </c>
+      <c r="B215" t="s">
+        <v>158</v>
+      </c>
+      <c r="C215" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="218" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B218" s="26" t="s">
         <v>190</v>
       </c>
-      <c r="C217" s="26"/>
-      <c r="D217" s="26"/>
-      <c r="E217" s="26"/>
-    </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A218" s="2" t="s">
+      <c r="C218" s="26"/>
+      <c r="D218" s="26"/>
+      <c r="E218" s="26"/>
+    </row>
+    <row r="219" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A219" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B218" s="7" t="s">
+      <c r="B219" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="C218" s="7" t="s">
+      <c r="C219" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="D218" s="2" t="s">
+      <c r="D219" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="E218" s="2" t="s">
+      <c r="E219" s="2" t="s">
         <v>52</v>
-      </c>
-    </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A219">
-        <v>1</v>
-      </c>
-      <c r="B219" t="s">
-        <v>43</v>
-      </c>
-      <c r="C219" t="s">
-        <v>58</v>
-      </c>
-      <c r="D219">
-        <v>20</v>
-      </c>
-      <c r="E219" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="220" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A220">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B220" t="s">
-        <v>191</v>
+        <v>43</v>
       </c>
       <c r="C220" t="s">
         <v>58</v>
@@ -4122,15 +4203,15 @@
         <v>20</v>
       </c>
       <c r="E220" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="221" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A221">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B221" t="s">
-        <v>154</v>
+        <v>191</v>
       </c>
       <c r="C221" t="s">
         <v>58</v>
@@ -4144,16 +4225,16 @@
     </row>
     <row r="222" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A222">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B222" t="s">
-        <v>127</v>
+        <v>154</v>
       </c>
       <c r="C222" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="D222">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="E222" t="s">
         <v>71</v>
@@ -4161,126 +4242,759 @@
     </row>
     <row r="223" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A223">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B223" t="s">
-        <v>192</v>
+        <v>127</v>
       </c>
       <c r="C223" t="s">
         <v>47</v>
       </c>
       <c r="D223">
-        <v>200</v>
+        <v>100</v>
+      </c>
+      <c r="E223" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="224" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A224">
+        <v>5</v>
+      </c>
+      <c r="B224" t="s">
+        <v>192</v>
+      </c>
+      <c r="C224" t="s">
+        <v>47</v>
+      </c>
+      <c r="D224">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="225" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A225">
         <v>6</v>
       </c>
-      <c r="B224" t="s">
+      <c r="B225" t="s">
         <v>173</v>
       </c>
-      <c r="C224" t="s">
+      <c r="C225" t="s">
         <v>107</v>
       </c>
-      <c r="D224">
+      <c r="D225">
         <v>500</v>
       </c>
     </row>
-    <row r="225" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A225">
+    <row r="226" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A226">
         <v>7</v>
       </c>
-      <c r="B225" t="s">
+      <c r="B226" t="s">
         <v>193</v>
       </c>
-      <c r="C225" t="s">
+      <c r="C226" t="s">
         <v>65</v>
       </c>
-      <c r="D225">
+      <c r="D226">
         <v>10</v>
       </c>
     </row>
-    <row r="226" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A226">
+    <row r="227" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A227">
         <v>8</v>
       </c>
-      <c r="B226" t="s">
+      <c r="B227" t="s">
         <v>194</v>
       </c>
-      <c r="C226" t="s">
-        <v>47</v>
-      </c>
-      <c r="D226">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="227" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A227">
+      <c r="C227" t="s">
+        <v>47</v>
+      </c>
+      <c r="D227">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="228" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A228">
         <v>9</v>
       </c>
-      <c r="B227" t="s">
+      <c r="B228" t="s">
         <v>195</v>
       </c>
-      <c r="C227" t="s">
-        <v>47</v>
-      </c>
-      <c r="D227">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="228" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A228">
+      <c r="C228" t="s">
+        <v>47</v>
+      </c>
+      <c r="D228">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="229" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A229">
         <v>10</v>
       </c>
-      <c r="B228" t="s">
+      <c r="B229" t="s">
         <v>196</v>
       </c>
-      <c r="C228" t="s">
-        <v>47</v>
-      </c>
-      <c r="D228">
+      <c r="C229" t="s">
+        <v>47</v>
+      </c>
+      <c r="D229">
         <v>25</v>
       </c>
     </row>
-    <row r="229" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A229">
+    <row r="230" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A230">
         <v>11</v>
       </c>
-      <c r="B229" t="s">
+      <c r="B230" t="s">
         <v>197</v>
       </c>
-      <c r="C229" t="s">
-        <v>47</v>
-      </c>
-      <c r="D229">
+      <c r="C230" t="s">
+        <v>47</v>
+      </c>
+      <c r="D230">
         <v>1000</v>
       </c>
     </row>
-    <row r="230" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A230">
+    <row r="231" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A231">
         <v>12</v>
       </c>
-      <c r="B230" t="s">
+      <c r="B231" t="s">
         <v>157</v>
-      </c>
-      <c r="C230" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="231" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A231">
-        <v>13</v>
-      </c>
-      <c r="B231" t="s">
-        <v>158</v>
       </c>
       <c r="C231" t="s">
         <v>59</v>
       </c>
     </row>
+    <row r="232" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A232">
+        <v>13</v>
+      </c>
+      <c r="B232" t="s">
+        <v>158</v>
+      </c>
+      <c r="C232" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="235" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B235" s="26" t="s">
+        <v>198</v>
+      </c>
+      <c r="C235" s="26"/>
+      <c r="D235" s="26"/>
+      <c r="E235" s="26"/>
+    </row>
+    <row r="236" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A236" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B236" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C236" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="D236" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E236" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="237" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A237">
+        <v>1</v>
+      </c>
+      <c r="B237" t="s">
+        <v>43</v>
+      </c>
+      <c r="C237" t="s">
+        <v>58</v>
+      </c>
+      <c r="D237">
+        <v>20</v>
+      </c>
+      <c r="E237" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="238" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A238">
+        <v>2</v>
+      </c>
+      <c r="B238" t="s">
+        <v>199</v>
+      </c>
+      <c r="C238" t="s">
+        <v>47</v>
+      </c>
+      <c r="D238">
+        <v>20</v>
+      </c>
+      <c r="E238" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="239" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A239">
+        <v>3</v>
+      </c>
+      <c r="B239" t="s">
+        <v>151</v>
+      </c>
+      <c r="C239" t="s">
+        <v>58</v>
+      </c>
+      <c r="D239">
+        <v>20</v>
+      </c>
+      <c r="E239" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="240" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A240">
+        <v>4</v>
+      </c>
+      <c r="B240" t="s">
+        <v>154</v>
+      </c>
+      <c r="C240" t="s">
+        <v>58</v>
+      </c>
+      <c r="D240">
+        <v>20</v>
+      </c>
+      <c r="E240" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="241" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A241">
+        <v>5</v>
+      </c>
+      <c r="B241" t="s">
+        <v>126</v>
+      </c>
+      <c r="C241" t="s">
+        <v>47</v>
+      </c>
+      <c r="D241">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="242" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A242">
+        <v>6</v>
+      </c>
+      <c r="B242" t="s">
+        <v>200</v>
+      </c>
+      <c r="C242" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="D242">
+        <v>20</v>
+      </c>
+      <c r="E242" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="243" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A243">
+        <v>7</v>
+      </c>
+      <c r="B243" t="s">
+        <v>201</v>
+      </c>
+      <c r="C243" t="s">
+        <v>65</v>
+      </c>
+      <c r="D243">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="244" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A244">
+        <v>8</v>
+      </c>
+      <c r="B244" t="s">
+        <v>202</v>
+      </c>
+      <c r="C244" t="s">
+        <v>65</v>
+      </c>
+      <c r="D244">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="245" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A245">
+        <v>9</v>
+      </c>
+      <c r="B245" t="s">
+        <v>203</v>
+      </c>
+      <c r="C245" t="s">
+        <v>65</v>
+      </c>
+      <c r="D245">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="246" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A246">
+        <v>10</v>
+      </c>
+      <c r="B246" t="s">
+        <v>204</v>
+      </c>
+      <c r="C246" t="s">
+        <v>65</v>
+      </c>
+      <c r="D246">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="247" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A247">
+        <v>11</v>
+      </c>
+      <c r="B247" t="s">
+        <v>205</v>
+      </c>
+      <c r="C247" t="s">
+        <v>65</v>
+      </c>
+      <c r="D247">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="248" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A248">
+        <v>12</v>
+      </c>
+      <c r="B248" t="s">
+        <v>206</v>
+      </c>
+      <c r="C248" t="s">
+        <v>65</v>
+      </c>
+      <c r="D248">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="249" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A249">
+        <v>13</v>
+      </c>
+      <c r="B249" t="s">
+        <v>207</v>
+      </c>
+      <c r="C249" t="s">
+        <v>65</v>
+      </c>
+      <c r="D249">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="250" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A250">
+        <v>14</v>
+      </c>
+      <c r="B250" t="s">
+        <v>208</v>
+      </c>
+      <c r="C250" t="s">
+        <v>65</v>
+      </c>
+      <c r="D250">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="251" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A251">
+        <v>15</v>
+      </c>
+      <c r="B251" t="s">
+        <v>209</v>
+      </c>
+      <c r="C251" t="s">
+        <v>65</v>
+      </c>
+      <c r="D251">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="252" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A252">
+        <v>16</v>
+      </c>
+      <c r="B252" t="s">
+        <v>210</v>
+      </c>
+      <c r="C252" t="s">
+        <v>65</v>
+      </c>
+      <c r="D252">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="253" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A253">
+        <v>17</v>
+      </c>
+      <c r="B253" t="s">
+        <v>211</v>
+      </c>
+      <c r="C253" t="s">
+        <v>107</v>
+      </c>
+      <c r="D253">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="254" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A254">
+        <v>18</v>
+      </c>
+      <c r="B254" t="s">
+        <v>212</v>
+      </c>
+      <c r="C254" t="s">
+        <v>107</v>
+      </c>
+      <c r="D254">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="255" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A255">
+        <v>19</v>
+      </c>
+      <c r="B255" t="s">
+        <v>175</v>
+      </c>
+      <c r="C255" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="D255">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="256" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A256">
+        <v>20</v>
+      </c>
+      <c r="B256" t="s">
+        <v>213</v>
+      </c>
+      <c r="C256" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="D256">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="257" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A257">
+        <v>21</v>
+      </c>
+      <c r="B257" t="s">
+        <v>214</v>
+      </c>
+      <c r="C257" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="D257">
+        <v>20</v>
+      </c>
+      <c r="E257" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="258" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A258">
+        <v>22</v>
+      </c>
+      <c r="B258" t="s">
+        <v>157</v>
+      </c>
+      <c r="C258" s="11" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="259" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A259">
+        <v>23</v>
+      </c>
+      <c r="B259" t="s">
+        <v>158</v>
+      </c>
+      <c r="C259" s="11" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="262" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B262" s="26" t="s">
+        <v>221</v>
+      </c>
+      <c r="C262" s="26"/>
+      <c r="D262" s="26"/>
+      <c r="E262" s="26"/>
+    </row>
+    <row r="263" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A263" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B263" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C263" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="D263" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E263" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="264" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A264">
+        <v>1</v>
+      </c>
+      <c r="B264" t="s">
+        <v>43</v>
+      </c>
+      <c r="C264" t="s">
+        <v>58</v>
+      </c>
+      <c r="D264">
+        <v>20</v>
+      </c>
+      <c r="E264" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="265" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A265">
+        <v>2</v>
+      </c>
+      <c r="B265" t="s">
+        <v>216</v>
+      </c>
+      <c r="C265" t="s">
+        <v>47</v>
+      </c>
+      <c r="D265">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="266" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A266">
+        <v>3</v>
+      </c>
+      <c r="B266" t="s">
+        <v>217</v>
+      </c>
+      <c r="C266" t="s">
+        <v>47</v>
+      </c>
+      <c r="D266">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="267" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A267">
+        <v>4</v>
+      </c>
+      <c r="B267" t="s">
+        <v>218</v>
+      </c>
+      <c r="C267" t="s">
+        <v>47</v>
+      </c>
+      <c r="D267">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="268" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A268">
+        <v>5</v>
+      </c>
+      <c r="B268" t="s">
+        <v>219</v>
+      </c>
+      <c r="C268" t="s">
+        <v>107</v>
+      </c>
+      <c r="D268">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="269" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A269">
+        <v>6</v>
+      </c>
+      <c r="B269" t="s">
+        <v>220</v>
+      </c>
+      <c r="C269" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="270" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A270">
+        <v>7</v>
+      </c>
+      <c r="B270" t="s">
+        <v>157</v>
+      </c>
+      <c r="C270" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="271" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A271">
+        <v>8</v>
+      </c>
+      <c r="B271" t="s">
+        <v>158</v>
+      </c>
+      <c r="C271" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="274" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B274" s="26" t="s">
+        <v>222</v>
+      </c>
+      <c r="C274" s="26"/>
+      <c r="D274" s="26"/>
+      <c r="E274" s="26"/>
+    </row>
+    <row r="275" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A275" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B275" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C275" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="D275" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E275" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="276" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A276">
+        <v>1</v>
+      </c>
+      <c r="B276" t="s">
+        <v>43</v>
+      </c>
+      <c r="C276" t="s">
+        <v>58</v>
+      </c>
+      <c r="D276">
+        <v>20</v>
+      </c>
+      <c r="E276" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="277" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A277">
+        <v>2</v>
+      </c>
+      <c r="B277" t="s">
+        <v>68</v>
+      </c>
+      <c r="C277" t="s">
+        <v>58</v>
+      </c>
+      <c r="D277">
+        <v>20</v>
+      </c>
+      <c r="E277" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="278" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A278">
+        <v>3</v>
+      </c>
+      <c r="B278" t="s">
+        <v>223</v>
+      </c>
+      <c r="C278" t="s">
+        <v>107</v>
+      </c>
+      <c r="D278">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="279" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A279">
+        <v>4</v>
+      </c>
+      <c r="B279" t="s">
+        <v>224</v>
+      </c>
+      <c r="C279" t="s">
+        <v>107</v>
+      </c>
+      <c r="D279">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="280" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A280">
+        <v>5</v>
+      </c>
+      <c r="B280" t="s">
+        <v>225</v>
+      </c>
+      <c r="C280" t="s">
+        <v>107</v>
+      </c>
+      <c r="D280">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="281" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A281">
+        <v>6</v>
+      </c>
+      <c r="B281" t="s">
+        <v>157</v>
+      </c>
+      <c r="C281" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="282" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A282">
+        <v>7</v>
+      </c>
+      <c r="B282" t="s">
+        <v>158</v>
+      </c>
+      <c r="C282" t="s">
+        <v>215</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="19">
+    <mergeCell ref="B235:E235"/>
+    <mergeCell ref="B262:E262"/>
+    <mergeCell ref="B274:E274"/>
     <mergeCell ref="B136:E136"/>
     <mergeCell ref="B77:E77"/>
     <mergeCell ref="B90:E90"/>
@@ -4292,7 +5006,7 @@
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="B17:E17"/>
     <mergeCell ref="B35:E35"/>
-    <mergeCell ref="B217:E217"/>
+    <mergeCell ref="B218:E218"/>
     <mergeCell ref="B152:E152"/>
     <mergeCell ref="B172:E172"/>
     <mergeCell ref="B200:E200"/>

</xml_diff>

<commit_message>
Add infromation in readme
</commit_message>
<xml_diff>
--- a/CareOS-Hospital_ERP_System.xlsx
+++ b/CareOS-Hospital_ERP_System.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hetlimbani/Desktop/Self_Learning/CareOS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23D9EA63-E27B-9642-A47A-3A8C81875A9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6F260D8-41CA-2943-AC7B-40970AE83513}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19420" activeTab="1" xr2:uid="{3BCF7A51-5C29-EE4C-8BC3-93CAF12DE1EA}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19420" activeTab="2" xr2:uid="{3BCF7A51-5C29-EE4C-8BC3-93CAF12DE1EA}"/>
   </bookViews>
   <sheets>
     <sheet name="ERP System" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="679" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="680" uniqueCount="228">
   <si>
     <t>Total Roles</t>
   </si>
@@ -722,6 +722,9 @@
   </si>
   <si>
     <t>vitalsHistory</t>
+  </si>
+  <si>
+    <t>if lab report or medicine bills are pending and paid via insurace than that bill auto paid and come paid via insurace.</t>
   </si>
 </sst>
 </file>
@@ -5018,7 +5021,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD54E32F-1636-154F-88FF-57ECFAEA7F4B}">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3.1640625" bestFit="1" customWidth="1"/>
@@ -5112,6 +5115,14 @@
         <v>123</v>
       </c>
     </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>227</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Solved bugs and complete project
</commit_message>
<xml_diff>
--- a/CareOS-Hospital_ERP_System.xlsx
+++ b/CareOS-Hospital_ERP_System.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hetlimbani/Desktop/Self_Learning/CareOS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8847F041-1E8F-3345-8B02-4D82DD681B47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6909BB8F-23BF-A040-8E8A-D7A1DAA8EDFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19420" xr2:uid="{3BCF7A51-5C29-EE4C-8BC3-93CAF12DE1EA}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19420" activeTab="2" xr2:uid="{3BCF7A51-5C29-EE4C-8BC3-93CAF12DE1EA}"/>
   </bookViews>
   <sheets>
     <sheet name="ERP System" sheetId="1" r:id="rId1"/>
@@ -5011,7 +5011,7 @@
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="10" t="s">
         <v>85</v>
       </c>
     </row>
@@ -5019,7 +5019,7 @@
       <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="10" t="s">
         <v>87</v>
       </c>
     </row>
@@ -5027,7 +5027,7 @@
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="10" t="s">
         <v>88</v>
       </c>
     </row>
@@ -5051,7 +5051,7 @@
       <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="10" t="s">
         <v>91</v>
       </c>
     </row>
@@ -5067,7 +5067,7 @@
       <c r="A11">
         <v>10</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="10" t="s">
         <v>116</v>
       </c>
     </row>
@@ -5075,7 +5075,7 @@
       <c r="A12">
         <v>11</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="10" t="s">
         <v>220</v>
       </c>
     </row>

</xml_diff>